<commit_message>
Update App Content via Excel
</commit_message>
<xml_diff>
--- a/Update_App_Data/upsc_toppers_data.xlsx
+++ b/Update_App_Data/upsc_toppers_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\Storage  Driver\upsc-cse-master-hub\Update_App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09FC4F45-43F0-4AD4-9EEC-B1E21A0FB0E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3574328F-FB8F-4A1C-9CA7-B4DD89D241D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Strategy" sheetId="1" r:id="rId1"/>
@@ -414,7 +414,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -427,6 +427,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -771,7 +777,8 @@
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" style="3"/>
-    <col min="2" max="5" width="11" style="2"/>
+    <col min="2" max="2" width="25.5" style="6" customWidth="1"/>
+    <col min="3" max="5" width="11" style="2"/>
     <col min="6" max="6" width="11" style="3"/>
     <col min="7" max="7" width="44.25" style="3" customWidth="1"/>
     <col min="8" max="8" width="19.5" style="3" customWidth="1"/>
@@ -782,19 +789,19 @@
     <col min="22" max="16384" width="11" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="5" t="s">
         <v>22</v>
       </c>
     </row>
@@ -802,15 +809,15 @@
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2">
-        <v>1</v>
+      <c r="B3" s="6">
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="6">
         <v>2021</v>
       </c>
     </row>
@@ -818,7 +825,7 @@
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="6" t="s">
         <v>23</v>
       </c>
     </row>
@@ -826,103 +833,103 @@
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="6">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="78.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="157.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="63" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="252" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="94.5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="330.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="126" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="173.25" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="5" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="189" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="141.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ht="63" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="157.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="63" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="5" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="173.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="189" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="189" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="63" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="5" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="110.25" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="5" t="s">
         <v>35</v>
       </c>
     </row>
@@ -930,7 +937,7 @@
       <c r="A19" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="3">
+      <c r="B19" s="5">
         <v>173</v>
       </c>
     </row>
@@ -938,23 +945,23 @@
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="3">
+      <c r="B20" s="5">
         <v>932</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" ht="157.5" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="5" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="5" t="s">
         <v>56</v>
       </c>
     </row>
@@ -50066,7 +50073,7 @@
   <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.375" customWidth="1"/>
     <col min="3" max="3" width="15.875" customWidth="1"/>
     <col min="4" max="4" width="19.125" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
feat: add Notes sheet to Excel - all 5 tabs now Excel-editable and Firebase synced
</commit_message>
<xml_diff>
--- a/Update_App_Data/upsc_toppers_data.xlsx
+++ b/Update_App_Data/upsc_toppers_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\Storage  Driver\upsc-cse-master-hub\Update_App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2D64079-03BC-4CB2-BF0C-D7770E961641}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6945E4DF-1237-4C6C-9CB3-E346991AD4F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,12 +18,15 @@
     <sheet name="Routines" sheetId="3" r:id="rId3"/>
     <sheet name="Interviews" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Routines!$A$1:$F$17</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="399">
   <si>
     <t>id</t>
   </si>
@@ -88,54 +91,6 @@
     <t>Aditya Srivastava</t>
   </si>
   <si>
-    <t>shruti-sharma</t>
-  </si>
-  <si>
-    <t>Shruti Sharma</t>
-  </si>
-  <si>
-    <t>History</t>
-  </si>
-  <si>
-    <t>St. Stephen's College &amp; JNU (History)</t>
-  </si>
-  <si>
-    <t>https://images.unsplash.com/photo-1580489944761-15a19d654956?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
-  </si>
-  <si>
-    <t>Own your notes. Making your own consolidated handwritten notes provides an unmatched mental index during the intense 3-hour Mains papers.</t>
-  </si>
-  <si>
-    <t>Prepared self-made digital and handwritten notes directly aligned with UPSC syllabus headings. Extensive answer writing practice at Jamia RCA, focusing on clarity, structure, and subheadings.</t>
-  </si>
-  <si>
-    <t>Deep historiographical perspectives for History; map-based geography; sociological case studies for Society.</t>
-  </si>
-  <si>
-    <t>Structured answers into Constitutional provisions, Statutory backing, Institutional bottlenecks, and Way Forward.</t>
-  </si>
-  <si>
-    <t>Point-wise presentation with data bullets, committee quotes, and clean schematic diagrams.</t>
-  </si>
-  <si>
-    <t>Prepared definitions of all GS4 terms in 1-2 lines with 2 personal and 2 administrative examples.</t>
-  </si>
-  <si>
-    <t>Addressed philosophical topics through varied lenses: individual, societal, administrative, national, and global.</t>
-  </si>
-  <si>
-    <t>History optional requires historiography, archaeological evidence, and high-quality historical site maps.</t>
-  </si>
-  <si>
-    <t>Solved previous 15 years UPSC Prelims papers multiple times to decode UPSC's question drafting mindset.</t>
-  </si>
-  <si>
-    <t>Regular practice of English comprehension and logical syllogisms.</t>
-  </si>
-  <si>
-    <t>Consolidate your own notes for every single line of the syllabus. | PYQs are the best teacher: study the options that UPSC eliminated in previous years. | Write answer copies in the actual UPSC format with margins. | Keep answers balanced, objective, and constructive.</t>
-  </si>
-  <si>
     <t>routineId</t>
   </si>
   <si>
@@ -191,9 +146,6 @@
   </si>
   <si>
     <t>Advaice</t>
-  </si>
-  <si>
-    <t>Kuch Nhi  123123</t>
   </si>
   <si>
     <t>Shruti Modi</t>
@@ -256,13 +208,7 @@
     <t>09:30 PM - 10:30 PM</t>
   </si>
   <si>
-    <t>First-Attempt / Full-Time</t>
-  </si>
-  <si>
     <t>Sadaf Choudhary / Naomi Satam</t>
-  </si>
-  <si>
-    <t>First-Attempt / Full-Time Model - Sadaf Choudhary &amp; Naomi Satam</t>
   </si>
   <si>
     <t>Evening Session</t>
@@ -281,9 +227,6 @@
   </si>
   <si>
     <t>02:00 PM - 05:30 PM</t>
-  </si>
-  <si>
-    <t>Morning Session</t>
   </si>
   <si>
     <t>Standard books, NCERTs, and syllabus mapping (3.5 hrs study + 30 min break)</t>
@@ -373,56 +316,920 @@
     <t>05:30 AM - 08:00 AM</t>
   </si>
   <si>
-    <t>Aariz</t>
+    <t>First-Attempt Full-Time Model - Sadaf Choudhary &amp; Naomi Satam</t>
   </si>
   <si>
-    <t>Aariz Mansuri</t>
+    <t xml:space="preserve">First-Attempt </t>
   </si>
   <si>
-    <t>Pub Add</t>
+    <t>First-Attempt</t>
   </si>
   <si>
-    <t>Ias</t>
+    <t xml:space="preserve">Morning Session D Dga </t>
   </si>
   <si>
-    <t>I am am ias officer</t>
+    <t>Radf</t>
   </si>
   <si>
-    <t xml:space="preserve">De;ta Nrpv </t>
+    <t>DF</t>
   </si>
   <si>
-    <t xml:space="preserve">DD </t>
+    <t>IAS</t>
   </si>
   <si>
-    <t>e</t>
+    <t>Shakti Dubey</t>
   </si>
   <si>
-    <t>Topper talk</t>
+    <t>Shatakshi Sinha</t>
   </si>
   <si>
-    <t>Kuch nhi old book jo bhi ho</t>
+    <t>Rupal Rana</t>
   </si>
   <si>
-    <t>muskan khurana</t>
+    <t>Tanya Singh</t>
   </si>
   <si>
-    <t xml:space="preserve">I tack tes </t>
+    <t>Swati Sharma</t>
   </si>
   <si>
-    <t>Prection</t>
+    <t>Riya Saini</t>
   </si>
   <si>
-    <t xml:space="preserve">only prep for ias </t>
+    <t>Yashvi Jain</t>
   </si>
   <si>
-    <t>ham bnenge ias</t>
+    <t>Garima Jain</t>
+  </si>
+  <si>
+    <t>Komal Mavi</t>
+  </si>
+  <si>
+    <t>Tripti Kalhans</t>
+  </si>
+  <si>
+    <t>Ritu Yadav</t>
+  </si>
+  <si>
+    <t>Preeti Kumari</t>
+  </si>
+  <si>
+    <t>Shobhika Pathak</t>
+  </si>
+  <si>
+    <t>Gamini Singla</t>
+  </si>
+  <si>
+    <t>Shruti Rajalakshmi</t>
+  </si>
+  <si>
+    <t>Anoushka Sharma</t>
+  </si>
+  <si>
+    <t>Pari Bishnoi</t>
+  </si>
+  <si>
+    <t>AIR 1</t>
+  </si>
+  <si>
+    <t>AIR 2</t>
+  </si>
+  <si>
+    <t>AIR 204</t>
+  </si>
+  <si>
+    <t>AIR 26</t>
+  </si>
+  <si>
+    <t>AIR 200</t>
+  </si>
+  <si>
+    <t>AIR 17</t>
+  </si>
+  <si>
+    <t>AIR 22</t>
+  </si>
+  <si>
+    <t>AIR 97</t>
+  </si>
+  <si>
+    <t>AIR 118</t>
+  </si>
+  <si>
+    <t>AIR 199</t>
+  </si>
+  <si>
+    <t>IPS</t>
+  </si>
+  <si>
+    <t>AIR 130</t>
+  </si>
+  <si>
+    <t>AIR 37</t>
+  </si>
+  <si>
+    <t>AIR 3</t>
+  </si>
+  <si>
+    <t>AIR 25</t>
+  </si>
+  <si>
+    <t>AIR 20</t>
+  </si>
+  <si>
+    <t>AIR 30</t>
+  </si>
+  <si>
+    <t>CSE 2024</t>
+  </si>
+  <si>
+    <t>CSE 2023</t>
+  </si>
+  <si>
+    <t>CSE 2025 (IFS)</t>
+  </si>
+  <si>
+    <t>CSE (Year N/A)</t>
+  </si>
+  <si>
+    <t>CSE 2024 (1st Attempt)</t>
+  </si>
+  <si>
+    <t>CSE 2023 (IAS)</t>
+  </si>
+  <si>
+    <t>CSE 2022</t>
+  </si>
+  <si>
+    <t>CSE 2021</t>
+  </si>
+  <si>
+    <t>PSIR (280 अंक)</t>
+  </si>
+  <si>
+    <t>PSIR</t>
+  </si>
+  <si>
+    <t>Sociology (290 अंक: P1-153, P2-137)</t>
+  </si>
+  <si>
+    <t>Economics</t>
+  </si>
+  <si>
+    <t>Political Science / Sociology</t>
+  </si>
+  <si>
+    <t>स्रोत में उल्लेखित नहीं</t>
+  </si>
+  <si>
+    <t>Anthropology (Public Administration से बदलाव)</t>
+  </si>
+  <si>
+    <t>Sociology (284 अंक)</t>
+  </si>
+  <si>
+    <t>Sociology</t>
+  </si>
+  <si>
+    <t>Sociology/Maths</t>
+  </si>
+  <si>
+    <t>Economics (286 अंक)</t>
+  </si>
+  <si>
+    <t>N/A (स्रोत में उल्लेखित नहीं)</t>
+  </si>
+  <si>
+    <t>3rd (CSAT fail in 2nd attempt)</t>
+  </si>
+  <si>
+    <t>4th</t>
+  </si>
+  <si>
+    <t>2nd</t>
+  </si>
+  <si>
+    <t>3rd</t>
+  </si>
+  <si>
+    <t>1st</t>
+  </si>
+  <si>
+    <t>5th (4th Attempt में बिना Mock के सफलता)</t>
+  </si>
+  <si>
+    <t>6th</t>
+  </si>
+  <si>
+    <t>5th</t>
+  </si>
+  <si>
+    <t>5th (2020 से)</t>
+  </si>
+  <si>
+    <t>2nd (1st में Prelims Fail → 6 माह Prelims Focus)</t>
+  </si>
+  <si>
+    <t>PCB (Bio) पृष्ठभूमि</t>
+  </si>
+  <si>
+    <t>CA पृष्ठभूमि</t>
+  </si>
+  <si>
+    <t>B.Tech Electrical Engineering</t>
+  </si>
+  <si>
+    <t>घर पर Self-Study (कोई Coaching Hub नहीं)</t>
+  </si>
+  <si>
+    <t>Goldman Sachs की High-Salary Job छोड़कर Full-Time Preparation</t>
+  </si>
+  <si>
+    <t>BA Economics (CUNY New York), UN Secretariat में 3 माह</t>
+  </si>
+  <si>
+    <t>"किताबें तो पढ़ ली हैं बहुत, बट उनको हटा के नई लगाने में वक्त लगेगा अभी।" | "सपने आपके अपने होते हैं; यदि आप उन्हें पूरा करने के लिए 100% प्रयास दे रहे हैं, तो सफलता निश्चित है।"</t>
+  </si>
+  <si>
+    <t>"Suffer the pain of discipline or suffer the pain of regret." | "Ordinary efforts done in a consistent manner lead to extraordinary results."</t>
+  </si>
+  <si>
+    <t>"I never felt like giving up... even had I not cleared this time, I would have given the exam again."</t>
+  </si>
+  <si>
+    <t>"There is a way out of this exam... learn from your mistakes."</t>
+  </si>
+  <si>
+    <t>"There will be days and weeks when nothing happens, and then there will be weeks when decades happen."</t>
+  </si>
+  <si>
+    <t>एकल स्रोत + बहुस्तरीय Revision (One Source, Multiple Revisions)।</t>
+  </si>
+  <si>
+    <t>PYQs से थीम्स निकालकर Short Notes + High-ROI विषयों पर महारत।</t>
+  </si>
+  <si>
+    <t>"Less is More" — नोट्स को अत्यधिक Condense करना।</t>
+  </si>
+  <si>
+    <t>FOMO से बचने के लिए बुनियादी NCERTs और Laxmikanth तक सीमित।</t>
+  </si>
+  <si>
+    <t>"अंतिम 30 दिनों में कोई नया स्रोत न छुएँ।"</t>
+  </si>
+  <si>
+    <t>"दूसरों की रणनीति अंधाधुंध Copy न करें, अपनी रणनीति बनाएँ।"</t>
+  </si>
+  <si>
+    <t>"Treat Mains as a strategic board exam."</t>
+  </si>
+  <si>
+    <t>"Understand Prelims depth via PYQs."</t>
+  </si>
+  <si>
+    <t>"I don't believe in giving up. If you are honest with your preparation, you will get there." | "कम पढ़ें पर बार-बार Revise करें।"</t>
+  </si>
+  <si>
+    <t>"Please have faith in your preparation and trust yourself."</t>
+  </si>
+  <si>
+    <t>"If you have really put in your efforts as a serious candidate, you will definitely achieve success with UPSC."</t>
+  </si>
+  <si>
+    <t>"UPSC is just an examination, treat it as one... it's not your life, it's just a part of your life."</t>
+  </si>
+  <si>
+    <t>"Motivation is a lie, discipline is real." | "Rank is merely a number until given meaning through dedicated service." | "नदी को किनारे खड़े होकर देखते रहने से नदी पार नहीं होती, प्रयास करना पड़ता है।"</t>
+  </si>
+  <si>
+    <t>Smart Work &gt; Brute Force। एक विषय – एक किताब। दिसंबर तक Mains Ready (Optional, Ethics, Essay, 1-page GS Notes)। थीम-बेस्ड करंट अफेयर्स नोट्स (GS 1-4 कीवर्ड्स अनुसार)। दैनिक 8-10 घंटे को 4 स्लॉट में बाँटना।</t>
+  </si>
+  <si>
+    <t>4-ब्लॉक Target Model (8-9 घंटे गुणवत्ता अध्ययन) | Integrated Approach (Prelims+Mains+Interview एकसाथ) | PYQs को सर्वश्रेष्ठ मित्र बनाना | 5+1+1 नियम (5 पढ़ाई + 1 Buffer + 1 Revision)।</t>
+  </si>
+  <si>
+    <t>सीमित स्रोत + 4 Register में Consolidated Notes + 7-8 बार Revision | Topper Copies (Aditya Srivastava, Maidan Ji) से Answer Structuring + Cross-fertilization | PYQs पर केंद्रित।</t>
+  </si>
+  <si>
+    <t>सीमित किताबें + बहुस्तरीय Revision + गलतियों का सूक्ष्म विश्लेषण | Spectrum को 25 ऑनलाइन पेजों में Condense किया।</t>
+  </si>
+  <si>
+    <t>असीमित सामग्री से बचना | AI Tools (ChatGPT/Gemini) का सारांश व उदाहरण के लिए उपयोग | Monthly/Yearly Magazines के Index Page पर Concise Notes।</t>
+  </si>
+  <si>
+    <t>One Source – Multiple Revisions | फरवरी से Sectional Tests फिर FLTs | PYQs के चारों विकल्पों का गहन विश्लेषण।</t>
+  </si>
+  <si>
+    <t>PYQ Mapping से Themes निकालना | छोटे High-Return विषयों (Internal Security, Disaster Management, Social Justice) पर Special Focus | Prelims ज्ञान → Google Docs → Mains में प्रयोग।</t>
+  </si>
+  <si>
+    <t>'Less is More' — Notes को Maximum Condense | GS1-GS4 को Interlink करके पढ़ना | गणितीय दृष्टिकोण से Essay को 5Ws में तोड़ना।</t>
+  </si>
+  <si>
+    <t>FOMO से बचाव — केवल NCERT + Laxmikanth | PYQs Brainstorming → Topper Copies से Matching | Interview: Personality + Clear Communication।</t>
+  </si>
+  <si>
+    <t>PYQs (2013 से) को Daily Mock की तरह हल करना | Limited Sources + Minimal Newspaper Notes | अंतिम 30 दिन: No New Source।</t>
+  </si>
+  <si>
+    <t>4th Attempt: बिना किसी Coaching Mock के केवल 10 वर्षों (2014 से) के PYQs का गहन विश्लेषण | Optional बदलकर Anthropology + 1 साल का Break लेकर Mains मज़बूत किया।</t>
+  </si>
+  <si>
+    <t>50% Content + 50% Presentation | Bullets, Committee Names, Flowcharts, Maps | कठिन पेपर में घबराने के बजाय 65 मज़बूत प्रश्न चुनना।</t>
+  </si>
+  <si>
+    <t>27 साल के PYQs की Theme-wise Compilation | 99 प्रश्न Attempt | Answer Writing Simulation + Daily Writing।</t>
+  </si>
+  <si>
+    <t>Less is More (सीमित स्रोत, 3-4 बार Revision) | Consolidated Notes (A4 Sheets पर: NCERTs + Static + PYQs + Test Synopsis) | FLTs Only (2-3 Coaching के Full Length Tests) | पेपर पूरा करना अनिवार्य।</t>
+  </si>
+  <si>
+    <t>घर पर तैयारी (बिना Coaching Hub) | सुबह 5 बजे से कड़ा Daily Routine | Self-Discipline + Family Support।</t>
+  </si>
+  <si>
+    <t>Goldman Sachs छोड़कर Full-Time Preparation | अनुशासित रहना + Self-Doubt से उबरना | Daily Current Affairs Notes | 1.5 माह पहले Daily Mock।</t>
+  </si>
+  <si>
+    <t>5-Page Fact Sheets (प्रति Subject) | 3-Round Paper Solving | 35 Mock Tests (गहन Revision) | Limited Sources।</t>
+  </si>
+  <si>
+    <t>Discipline &gt; Motivation | 80/20 नियम: 80% प्रश्न 20% Core Syllabus से | सीमित स्रोत, 3-4 बार Revision | Syllabus + PYQs को Guide बनाना।</t>
+  </si>
+  <si>
+    <t>अंक: 112 | इतिहास: TN Board Cl-11 NCERT + Spectrum/Bipin Chandra | भूगोल: Cl-11,12 NCERTs + Atlas | समाज: उत्कर्ष द्विवेदी टेम्पलेट + NCERT + NFHS/ASER डेटा | विश्व इतिहास: Vision IAS बुकलेट + PYQs।</t>
+  </si>
+  <si>
+    <t>भूगोल: Cl-11,12 NCERTs + Maps अभ्यास | इतिहास: Spectrum/PW Udaan (Modern) + पुरानी NCERTs (Ancient/Medieval) | Art &amp; Culture: NCERTs + Stick Figures (नटराज आदि) | प्रतिदिन 30 मिनट Modern History।</t>
+  </si>
+  <si>
+    <t>विभिन्न GS Papers के ज्ञान को Cross-fertilize करके उत्तर लिखे | 2-3 पेज Concise Notes प्रति विषय।</t>
+  </si>
+  <si>
+    <t>History: Modern → Spectrum (25 pages में condense) + NCERTs (R.S. Sharma, Satish Chandra, Bipan Chandra) | Society: Smriti Ma'am Notes | Comparative Charts: राष्ट्रपति vs राज्यपाल आदि।</t>
+  </si>
+  <si>
+    <t>समाचार पत्र की जगह Monthly/Yearly Magazines के Index Page पर Short Notes + बार-बार Revision।</t>
+  </si>
+  <si>
+    <t>इतिहास/भूगोल के कठिन प्रश्नों में Maps + Diagrams बनाकर अंक खींचे | PYQs (2013 के बाद) के चारों Options का गहन विश्लेषण।</t>
+  </si>
+  <si>
+    <t>PYQs से Themes → Short Notes | Core (Polity, Economy) + Science &amp; Tech + Environment पर महारत।</t>
+  </si>
+  <si>
+    <t>GS विषयों को आपस में Interlink करके पढ़ें | Condensed Notes।</t>
+  </si>
+  <si>
+    <t>NCERT + Basic Sources — FOMO से बचते हुए।</t>
+  </si>
+  <si>
+    <t>History: Spectrum | Art &amp; Culture: NCERTs।</t>
+  </si>
+  <si>
+    <t>PYQ गहन विश्लेषण पर आधारित।</t>
+  </si>
+  <si>
+    <t>50% Content + 50% Presentation | Maps, Diagrams का प्रयोग।</t>
+  </si>
+  <si>
+    <t>27 साल के PYQs से Themes + Answer Writing।</t>
+  </si>
+  <si>
+    <t>अंक: 110+ (लगातार) | इतिहास (Modern): Spectrum → Short Notes + Revision | इतिहास (Ancient/Medieval): TN Board Cl-11, Cl-12 Themes in Indian History | भूगोल: 11-12 NCERTs + PMF IAS Selective + YouTube (Dr. Shivin, Sleepy Classes) | Society: Sociology Optional का ओवरलैप + PYQ Themes + Model Answers।</t>
+  </si>
+  <si>
+    <t>Laxmikanth (Polity) + Basic History NCERTs।</t>
+  </si>
+  <si>
+    <t>Geography: NCERTs (Mandatory) | History: NCERTs (Ancient/Medieval)।</t>
+  </si>
+  <si>
+    <t>History: TN Board 11th + Old NCERTs + CC Leong | Society: Vision Notes।</t>
+  </si>
+  <si>
+    <t>Ancient/Medieval: Old NCERT/R.S. Sharma | Art &amp; Culture: 11th Fine Arts NCERT।</t>
+  </si>
+  <si>
+    <t>अंक: 125 | पॉलिटी: Laxmikanth (Margin Notes) + Abhay Kumar 500 MCQs | शासन: 2nd ARC, सुप्रीम कोर्ट निर्णय | IR: PSIR Optional नोट्स का ओवरलैप + करंट (BRICS, SCO, G20, BIMSTEC) | सामाजिक न्याय: उत्कर्ष टेम्पलेट + SHG/NABARD डेटा।</t>
+  </si>
+  <si>
+    <t>पॉलिटी: Vision IAS Foundation Notes (Amirul Hasan Sir) + Laxmikanth (Margin में नोट्स) | IR: PSIR Optional से भारी ओवरलैप | Governance: Indian Express पैसिव रीडिंग।</t>
+  </si>
+  <si>
+    <t>GS1-GS4 Cross-fertilization | 2-3 पेज नोट्स | Committee Recommendations + Articles का समावेश।</t>
+  </si>
+  <si>
+    <t>Polity: Laxmikanth + 11th NCERT (Constitution at Work) | IR: Shubhra Ranjan + ORF + Indian Express + The Hindu + Jaishankar Speeches | Governance: Committee Recommendations।</t>
+  </si>
+  <si>
+    <t>प्रत्येक GS Paper: केवल 30-35 Pages के Short Notes | Pointer Format: 10-अंक → 8-10 Points, 15-अंक → 12-13 Points।</t>
+  </si>
+  <si>
+    <t>Articles + Committee Recommendations समावेश + Pointwise | Supreme Court Judgements का उल्लेख।</t>
+  </si>
+  <si>
+    <t>Polity + Governance + IR → PYQ Theme Analysis | Prelims के तथ्य → Google Docs → Mains उत्तर।</t>
+  </si>
+  <si>
+    <t>GS1-GS4 Interlinking Strategy।</t>
+  </si>
+  <si>
+    <t>Laxmikanth + NCERT | PYQ Brainstorming + Topper Copy Matching।</t>
+  </si>
+  <si>
+    <t>Polity: 11th NCERTs (Political Theory + Constitution at Work) + Laxmikanth | IR: Current-based।</t>
+  </si>
+  <si>
+    <t>PYQ गहन विश्लेषण + Limited Sources।</t>
+  </si>
+  <si>
+    <t>Bullet Points + Committee Names + Constitutional Articles।</t>
+  </si>
+  <si>
+    <t>PYQ Theme Analysis + Daily Writing।</t>
+  </si>
+  <si>
+    <t>अंक: ~118 | Polity: Laxmikanth (Highlight + बार-बार पढ़ना) + 11th NCERT Political Theory | Governance: 2nd ARC, Mallimath Committee + Constitutional Articles + Health/Education Frameworks (ASER, TSR Subramanian) | IR: Next IAS (Deepin Sir) Notes — 5-6 बार Revision | Social Justice: PYQ Themes।</t>
+  </si>
+  <si>
+    <t>The Hindu / Indian Express + Drishti Daily News Analysis।</t>
+  </si>
+  <si>
+    <t>Polity: Laxmikanth।</t>
+  </si>
+  <si>
+    <t>Polity: Laxmikanth + Mains 365 | MEA Statements + Committee Recommendations | IR: Current।</t>
+  </si>
+  <si>
+    <t>Polity: Laxmikanth (5-6 बार Revision) | Parliament, Judiciary, FRs, DPSPs पर विशेष ध्यान | Supreme Court Cases + Articles।</t>
+  </si>
+  <si>
+    <t>अंक: 86 | अर्थव्यवस्था: Shriram IAS Notes + Budget/Eco Survey (Jayant Sir) + Shivin Sir GS3 Template | आंतरिक सुरक्षा: Shivin Sir Template + अद्यतन डेटा | आपदा: NDMA Template (Utkarsh Dwivedi) | Environment &amp; S&amp;T: Annual Mains Compilations।</t>
+  </si>
+  <si>
+    <t>Economy+Environment+Security: Vision IAS Mains 365 | Budget: 2 पेज क्रिस्प नोट्स | Eco Survey: 3 पेज | Environment Mains 365: 6 पेज | Visual Presentation: Trend Graphs, Flowcharts, Infographics।</t>
+  </si>
+  <si>
+    <t>2-3 पेज नोट्स | Prelims में एकत्र ज्ञान/तथ्य Google Docs में सहेजकर Mains में प्रयोग।</t>
+  </si>
+  <si>
+    <t>GS3: Science &amp; Tech + Environment → Mains 365 | Internal Security → Shivin Sir Notes।</t>
+  </si>
+  <si>
+    <t>30-35 पेज Short Notes | Committee Names, Data, Schemes का समावेश।</t>
+  </si>
+  <si>
+    <t>स्रोत में विशिष्ट GS3 विवरण नहीं, सीमित स्रोत + Revision।</t>
+  </si>
+  <si>
+    <t>Internal Security: Vajiram Yellow Book | Disaster Management: Google का विस्तृत उपयोग | High-ROI Small Subjects पर विशेष ध्यान।</t>
+  </si>
+  <si>
+    <t>GS1-GS4 Interlinking + Condensed Notes।</t>
+  </si>
+  <si>
+    <t>Limited Sources + PYQ Analysis।</t>
+  </si>
+  <si>
+    <t>Economy: Vivek Singh + Budget &amp; Economic Survey Summary।</t>
+  </si>
+  <si>
+    <t>PYQ गहन विश्लेषण।</t>
+  </si>
+  <si>
+    <t>Flowcharts, Maps, Diagrams से Presentation।</t>
+  </si>
+  <si>
+    <t>PYQ-based Preparation + Daily Answer Writing।</t>
+  </si>
+  <si>
+    <t>अर्थव्यवस्था: Budget + Eco Survey से Data/Graphs + Mrunal Sir Free Lectures (YouTube) | कृषि: Ministry Schemes + Dryland Farming + PYQs + Crop Map | S&amp;T: PT365/Mains365 + Blockchain/IoT/Nuclear | Disaster Management: 2013-2024 सभी PYQs Model Format में | Environment: ISFR, UNEP Reports + Current Facts।</t>
+  </si>
+  <si>
+    <t>Newspaper Reading + Basic NCERTs का एकीकरण।</t>
+  </si>
+  <si>
+    <t>Economy: बार-बार पढ़कर महारत (शुरुआत में कठिन था)।</t>
+  </si>
+  <si>
+    <t>Economy: Optional से Covered | S&amp;T: Mains 365 | Security: Notes + Maps/Diagrams।</t>
+  </si>
+  <si>
+    <t>Economy: Shankar Ganesh (150 pages) / Mrunal Notes + Budget &amp; Eco Survey।</t>
+  </si>
+  <si>
+    <t>अंक: 141 (देश में सर्वोच्च में से एक, बिना कोचिंग) | 100 कीवर्ड्स (Syllabus 25-30 + PYQs 50-60) | हर कीवर्ड: परिभाषा + Quote + सिविल सेवक उदाहरण + केस स्टडी | Prahar Magazine बुकलेट + The Better India | दार्शनिक: Aristotle, Plato, Kant, Hannah Arendt | समय: Section A → 1h15m, Case Studies → 1h45m।</t>
+  </si>
+  <si>
+    <t>पसंदीदा विषय | Case Studies: Hub &amp; Spoke Model (Stakeholders) + Pros/Cons Table | समय: Theory → 1h15m, Case Studies → शेष | किसी rigid structure के बिना व्यक्तित्व दिखाएँ।</t>
+  </si>
+  <si>
+    <t>Case Studies: सामान्य सुझावों के बजाय स्पष्ट व्यावहारिक समाधान | Essay: रोजाना एक विषय पर Brainstorming Notes।</t>
+  </si>
+  <si>
+    <t>Ethics: Ansari Sir (Lukman IAS) Notes | 'The Better India' से Real Examples | Ramayana/Mahabharata से नैतिक पाठ | Topper Copies (Shruti Ma'am, Vishakha Ma'am)।</t>
+  </si>
+  <si>
+    <t>Ethics: प्रत्येक उत्तर में कम से कम एक Indian/Western Philosopher का उल्लेख | Case Studies: 3-4 Pre-set Templates (Stakeholder Approach, Values Approach)।</t>
+  </si>
+  <si>
+    <t>Ethics: पहले 10-अंकीय प्रश्न, फिर Case Studies, अंत में Quotation-based प्रश्न हल किए।</t>
+  </si>
+  <si>
+    <t>Essay: स्वामी विवेकानंद के विचार, INA Trial, 'Tryst with Destiny' जैसे ऐतिहासिक संदर्भ।</t>
+  </si>
+  <si>
+    <t>स्रोत में विशिष्ट GS4 विवरण नहीं।</t>
+  </si>
+  <si>
+    <t>PYQ Brainstorming + Model Answer Comparison।</t>
+  </si>
+  <si>
+    <t>Mains के लिए 6-7 माह समर्पित।</t>
+  </si>
+  <si>
+    <t>Practical Solutions + Clear Framework।</t>
+  </si>
+  <si>
+    <t>Daily Writing Practice।</t>
+  </si>
+  <si>
+    <t>अंक: 129 | Section A: Ready-made Frameworks/Templates (Personal/Professional/Social, Concentric Circles) + Diverse Examples (Bhagavad Gita, IPS CAA Protest, Zomato Delivery Boy) + Sakshi Ma'am Mentorship (Vajiram) | Case Studies: Stakeholder के लिए Creative Diagrams (Forest Cutting में Tree Drawing) + Clear Option Selection + Positive Conclusion।</t>
+  </si>
+  <si>
+    <t>Case Studies अभ्यास + Daily Events से Critical Thinking।</t>
+  </si>
+  <si>
+    <t>स्रोत में विशिष्ट GS4 Strategy नहीं।</t>
+  </si>
+  <si>
+    <t>DK Balaji Sir Book | Quotes/Definitions Notes | Section A: 1.5h, Case Studies: 1.5h।</t>
+  </si>
+  <si>
+    <t>Syllabus Keywords की परिभाषाएँ + व्यावहारिक उदाहरण (2-3 Page Sheet)।</t>
+  </si>
+  <si>
+    <t>अंक: 100 | प्रति निबंध 1.5 घंटा (20-30 मिनट माइंड-मैप, 1 घंटा लेखन) | 15-16 बहु-आयामी GS आयाम | दोनों निबंधों का ढाँचा अलग | Haidt की 'The Anxious Generation' जैसे साहित्यिक संदर्भ।</t>
+  </si>
+  <si>
+    <t>अंक: 144 | 5 मिनट Timer → रफ पेज पर सभी आयाम (PESTEL) + Quotes | Anecdote/Quote से आकर्षक शुरुआत | Topper copies से Example Bank तैयार।</t>
+  </si>
+  <si>
+    <t>रोजाना एक दार्शनिक विषय पर Brainstorming Notes | Philosophical Essays में गहरी वैचारिक संरचना।</t>
+  </si>
+  <si>
+    <t>PYQs से मुख्य Themes (Problems, Causes, Solutions, Way Forward) पहचाने।</t>
+  </si>
+  <si>
+    <t>प्रत्येक GS Paper: 30-35 पेज Short Notes | PESTEL दृष्टिकोण।</t>
+  </si>
+  <si>
+    <t>PYQ Analysis + Toppers की Answer Copies से Structuring।</t>
+  </si>
+  <si>
+    <t>Essay: स्वामी विवेकानंद + INA Trial + Tryst with Destiny जैसे ऐतिहासिक संदर्भ | Multi-dimensional दृष्टिकोण।</t>
+  </si>
+  <si>
+    <t>Essay को 5Ws (How, What, Why, When, Who) में तोड़कर Structure | गणितीय दृष्टिकोण से रूपरेखा।</t>
+  </si>
+  <si>
+    <t>PYQs Brainstorming → Topper Copies से Matching।</t>
+  </si>
+  <si>
+    <t>Limited Sources + Revision।</t>
+  </si>
+  <si>
+    <t>Mains के लिए Dedicated 6-7 माह (Prelims से पहले)।</t>
+  </si>
+  <si>
+    <t>Multi-dimensional दृष्टिकोण + Diagrams।</t>
+  </si>
+  <si>
+    <t>Daily Answer Writing + PYQ Simulation।</t>
+  </si>
+  <si>
+    <t>अंक: 138 (2020 में) | Organic &amp; Simple लेखन (रटे-रटाए Formula से बचना) | Structure: Main Theme → पक्ष → 2 Para विपक्ष → Futuristic Conclusion | Framework 1: Individual→Family→Society→Nation→World | Framework 2: Ancient→Medieval→Modern→AI Age | बाहरी Feedback (माता-पिता, Prof.) लेना।</t>
+  </si>
+  <si>
+    <t>Quotes की जगह Real Stories/Case Studies से शुरुआत | 15-16 निबंध लिखे | Multi-dimensional दृष्टिकोण।</t>
+  </si>
+  <si>
+    <t>Prelims के बाद 6-7 Tests (कुल 12-14 निबंध) लिखे।</t>
+  </si>
+  <si>
+    <t>Multi-dimensional दृष्टिकोण | Quotes + Examples।</t>
+  </si>
+  <si>
+    <t>PESTLE Dimensions से Essay Link | 10-15 मिनट Brainstorming + Outline | Anecdote/Quotes से शुरुआत | Way Forward पर Positive Conclusion।</t>
+  </si>
+  <si>
+    <t>PSIR 280 अंक (2023: 230 → 2024: 280) | IGNOU सामग्री + Shriram/Vajiram नोट्स | सितंबर तक Syllabus + PYQs पूरे | 40% दैनिक समय | विचारक + खंडन एकसाथ | IR Paper 2B में करंट इंटीग्रेट।</t>
+  </si>
+  <si>
+    <t>PSIR | PYQs: 2013-2023 Topic-Wise | हर Topic: 2-4 Thinkers (पक्ष+विपक्ष) | तकनीकी शब्दावली | GS2 IR से भारी ओवरलैप।</t>
+  </si>
+  <si>
+    <t>Sociology 290 अंक | 4 मुख्य Register + 4 छोटे Handouts (अंतिम समय हेतु) | Durkheim के सिद्धांत → वर्तमान उदाहरण से जोड़ना | Thinkers को Current Affairs से Link।</t>
+  </si>
+  <si>
+    <t>PSIR: Shubhra Ranjan 80% Base | ORF, Indian Express, The Hindu, Jaishankar Interviews से Value Addition।</t>
+  </si>
+  <si>
+    <t>Economics: Paper 2 को GS3 Indian Economy से Integrate किया | Arjun Gupta Sir के Topper Notes।</t>
+  </si>
+  <si>
+    <t>PSIR: O.P. Gauba, Andrew Heywood (Global Politics) | 20 व 15 अंक वाले प्रश्नों को प्राथमिकता।</t>
+  </si>
+  <si>
+    <t>Political Science/Sociology | PYQ-based तैयारी।</t>
+  </si>
+  <si>
+    <t>स्रोत में विशिष्ट Optional Strategy नहीं।</t>
+  </si>
+  <si>
+    <t>Anthropology (Public Administration से Switch) | 1 साल का Break लेकर Mains को मज़बूत किया।</t>
+  </si>
+  <si>
+    <t>Sociology: 284 अंक | Thinkers → Current Examples से Link।</t>
+  </si>
+  <si>
+    <t>Sociology: 277 अंक (2020) | B.Tech Background पर GS/Essay/Ethics Overlap | Sources: NCERT 11-12 + IGNOU BA | Value Addition: Tusharanshu Sir + Nitin Sangwan (Essential Sociology) + Ritzer (Selective) + LevelUp IAS + Shankar IAS Test Series | Integrated Notes (Paper 1+2 समान Topics) | Humanities Prof. शैली में Paragraph Format + 1-3 Thinkers प्रति उत्तर।</t>
+  </si>
+  <si>
+    <t>Sociology: उपलब्धता + रुचि के आधार पर चयन।</t>
+  </si>
+  <si>
+    <t>Sociology/Maths: Notes बनाना + PYQs पर विशेष जोर।</t>
+  </si>
+  <si>
+    <t>Economics: 144+142 = 286 अंक | H.L. Ahuja, Salvatore, Jhingan | Economic Survey + Budget।</t>
+  </si>
+  <si>
+    <t>Optional चयन के 4 पैमाने: Background/Interest + Syllabus Vastness + Competition Level + Guidance Availability।</t>
+  </si>
+  <si>
+    <t>अंक: 82 (Cutoff: 75) | नया पैटर्न + Shock Absorption माइंडसेट | PYQ थीम एनालिसिस (Art. 19, 21, 32 जैसे हाई-फ्रीक्वेंसी) | Jan-Feb: रिवीजन 1, Mar-15Apr: रिवीजन 2 | 3-इटरेशन पेपर सॉल्विंग | सबसे मज़बूत विषय (Polity) से शुरू।</t>
+  </si>
+  <si>
+    <t>2024 में 98 प्रश्न अटेम्प्ट | Vajiram Power Up Test Series (CA) + Vision IAS Abhyas Tests | Calculated Risk: 30-35 sure-shot + 50-50 elimination | अंतिम 27 दिन: कोई नया रिसोर्स नहीं, केवल नोट्स + PYQs।</t>
+  </si>
+  <si>
+    <t>फरवरी से प्रतिदिन 50 MCQs + सप्ताह में 2-3 Mock Tests | परीक्षा से 1 महीना पहले Mock बंद → केवल PYQs | The Hindu + Monthly Magazines (3-4 बार Revision) | CA के अलग नोट्स नहीं।</t>
+  </si>
+  <si>
+    <t>4th Attempt: 90+ प्रश्न हल किए (पहले 3 में 71-78 से Fail) | Source List: Polity-Laxmikanth+11NCERT, History-Spectrum, Economy-Vivek Singh, Environment-Shankar+PT365, Geography-Rishikesh Notes+11/12 NCERT | Comparative Tables।</t>
+  </si>
+  <si>
+    <t>जनवरी से ऑफलाइन Mock Tests + कमज़ोर विषयों का विश्लेषण | Monthly/Yearly Magazine Index पर Notes | CSAT: केवल PYQs।</t>
+  </si>
+  <si>
+    <t>फरवरी से Sectional Tests → FLTs | 2013 के बाद के PYQs के चारों विकल्पों का विश्लेषण।</t>
+  </si>
+  <si>
+    <t>PYQs से Themes निकालकर Short Notes | Core + Sci&amp;Tech + Environment में बढ़त (Bouncer प्रश्नों में लाभ)।</t>
+  </si>
+  <si>
+    <t>Risk Management: 90-95 प्रश्न हल करने का लक्ष्य | 30 प्रश्न गलत के Margin के बाद भी 100+ Net Positive।</t>
+  </si>
+  <si>
+    <t>FOMO से बचाव — केवल NCERT + Laxmikanth तक सीमित | CSAT: बिना नागा रोजाना अभ्यास + PYQs।</t>
+  </si>
+  <si>
+    <t>2013 के बाद के PYQs को दैनिक 25 प्रश्नों के Mock की तरह हल किया | Polity: 11th NCERTs + Laxmikanth | Economy: Vivek Singh + Budget | History: Spectrum।</t>
+  </si>
+  <si>
+    <t>4th Attempt: बिना Coaching Mock के, केवल पिछले 10 वर्षों (2014 से) के PYQs का गहन विश्लेषण।</t>
+  </si>
+  <si>
+    <t>2023 के कठिन पेपर में घबराए नहीं | 65 मज़बूत प्रश्न पहले चुने → 88 प्रश्न हल किए।</t>
+  </si>
+  <si>
+    <t>27 साल के PYQs की Theme-wise Compilation | 99 प्रश्न Attempt।</t>
+  </si>
+  <si>
+    <t>Less is More — 3 बार Revision | केवल 15+ Full Length Tests (Vision, Forum, Vajiram) | PYQs (2013 से): सभी Options का गहन विश्लेषण + Notes में समाहित | 2021: 100 प्रश्न → &lt;1 अंक से Fail → Calculated Risk (80-95 प्रश्न) | Current Affairs: PT365 + Newspaper 30 मिनट (Ethics/Essay Examples)।</t>
+  </si>
+  <si>
+    <t>1991 से PYQs Solve | अंतिम 2 माह: Daily Mock Tests | घर पर Exam जैसा माहौल।</t>
+  </si>
+  <si>
+    <t>Daily Current Affairs Notes | Prelims से 1.5 माह पहले रोज़ एक Mock Test।</t>
+  </si>
+  <si>
+    <t>35 Mock Tests (गहन Revision) | 5-Page Fact Sheets (प्रति Subject) | 3 Rounds में Paper Solve।</t>
+  </si>
+  <si>
+    <t>1st Attempt Prelims Fail → 6 माह केवल Prelims Focus | एक विषय 10 दिन → Test (Vision/Insights) → 2 दिन Revision → अगला विषय।</t>
+  </si>
+  <si>
+    <t>अंक: 75 | PCB बैकग्राउंड, 10वीं के बाद Maths नहीं | RC: 25-28 प्रश्न (उच्च सटीकता) | Reasoning: 10-15 प्रश्न | Quant: Time-Work, SDT, Percentage, Number System | कुल 45-50 प्रश्न टार्गेट।</t>
+  </si>
+  <si>
+    <t>2nd Attempt में CSAT fail → 3rd में विशेष ध्यान | NDA, CDS, CPSC के पिछले 3 साल के CSAT Papers | RC: प्रश्न पहले पढ़ें → Extreme Options तुरंत खारिज | 27-28 RC में से 22+ सही टार्गेट।</t>
+  </si>
+  <si>
+    <t>स्रोत में विशिष्ट उल्लेख नहीं।</t>
+  </si>
+  <si>
+    <t>Comprehension के लिए केवल UPSC PYQs को मुख्य आधार।</t>
+  </si>
+  <si>
+    <t>CSAT: गणितीय कमज़ोरी पहचानकर Number System, Average, Calendar जैसे High-Yield Topics के लिए Crash Course + अभ्यास।</t>
+  </si>
+  <si>
+    <t>बिना नागा रोजाना प्रश्न अभ्यास | Comprehension के लिए केवल PYQs।</t>
+  </si>
+  <si>
+    <t>R.S. Aggarwal पुस्तक + नियमित अभ्यास।</t>
+  </si>
+  <si>
+    <t>पिछले 5 साल के PYQs → 2 घंटे Time-bound | Formula Sheet (1 Page): Mathematical Formulas, Tricks, Reasoning Rules → GS1-GS2 Break में Revise | 53 Maths/Reasoning में से 27-28 Easy + Comprehension ध्यान से।</t>
+  </si>
+  <si>
+    <t>रोजाना 15-20 मिनट Logical Reasoning + Quant अभ्यास।</t>
+  </si>
+  <si>
+    <t>Mental Ability + Maths पर भरोसा + पुराने Papers Solve।</t>
+  </si>
+  <si>
+    <t>English में Comfortable (30 प्रश्न) | Maths/Reasoning में Selective।</t>
+  </si>
+  <si>
+    <t>Logical Elimination + 50-50 वाले प्रश्नों में Net Positive Strategy।</t>
+  </si>
+  <si>
+    <t>200 / 275</t>
+  </si>
+  <si>
+    <t>187 / 275</t>
+  </si>
+  <si>
+    <t>स्रोत में उल्लेखित नहीं | Mock Interviews से Stage Fear दूर | IR + Newspapers पर विशेष ध्यान।</t>
+  </si>
+  <si>
+    <t>201 / 275</t>
+  </si>
+  <si>
+    <t>स्रोत में उल्लेखित नहीं।</t>
+  </si>
+  <si>
+    <t>206 / 275</t>
+  </si>
+  <si>
+    <t>216 / 275 (Suman Sharma Board)</t>
+  </si>
+  <si>
+    <t>180 / 275 (Sanjay Verma Board)</t>
+  </si>
+  <si>
+    <t>198 / 275</t>
+  </si>
+  <si>
+    <t>195 / 275 (2020: 160 → 2024: 195)</t>
+  </si>
+  <si>
+    <t>204 / 275 (Manoj Soni Board)</t>
+  </si>
+  <si>
+    <t>1st: 176 अंक | 2nd: 200 अंक</t>
+  </si>
+  <si>
+    <t>लिखित: 843/1750 | कुल (Mains+Interview): 1043/2025 | GS1:112, GS2:125, GS3:86, GS4:141, Essay:100, PSIR:280</t>
+  </si>
+  <si>
+    <t>लिखित: 851/1750 | कुल (Mains+Interview): 1038/2025 | Essay: 144, PSIR Optional</t>
+  </si>
+  <si>
+    <t>Sociology: 290 (Paper 1: 153, Paper 2: 137)</t>
+  </si>
+  <si>
+    <t>स्रोत में GS-wise breakup नहीं।</t>
+  </si>
+  <si>
+    <t>स्रोत में विशिष्ट अंक नहीं।</t>
+  </si>
+  <si>
+    <t>Sociology Optional: 284 अंक।</t>
+  </si>
+  <si>
+    <t>GS1: 110+, GS2: ~118, GS4: 129, Essay: 138 (2020), Sociology: 277+ | कुल GS ~435+</t>
+  </si>
+  <si>
+    <t>GS1: 107, GS2: 105, GS3: 85, GS4: 108 | Optional: 144+142 = 286</t>
+  </si>
+  <si>
+    <t>1. दिसंबर तक Mains Ready | 2. एक विषय – एक पुस्तक, 3-4 बार रिवीजन | 3. Active Recall (किताब बंद कर याद करें) | 4. 10-15 पेज की Factbook (डेटा, समितियाँ, निर्णय) | 5. अखबार: 1-1.5 घंटे, केवल Explained Page | 6. Essay+Ethics+Optional पर 50%+ ध्यान।</t>
+  </si>
+  <si>
+    <t>1. घंटे नहीं, Target गिनें (8-9 घंटे गुणवत्ता) | 2. PYQs को रीढ़ बनाएँ | 3. सीमित स्रोत + अधिकतम Revision | 4. 5+1+1 Time-Table Model | 5. सकारात्मक मानसिकता + 7-8 घंटे नींद।</t>
+  </si>
+  <si>
+    <t>नए अभ्यर्थी सबसे पहले PYQs देखें | दैनिक कम से कम 8 घंटे गुणवत्तापूर्ण पढ़ाई | कभी हार न मानें।</t>
+  </si>
+  <si>
+    <t>खुद की रणनीति पर भरोसा रखें | महीने में 1-2 दिन पूर्ण Break (Burnout से बचाव) | Multiple Revisions of Limited Sources।</t>
+  </si>
+  <si>
+    <t>AI Tools का उपयोग करें (उदाहरण + सारांश) | अपने Notes पर भरोसा | Resources सीमित रखें।</t>
+  </si>
+  <si>
+    <t>One Source – Multiple Revisions | गलतियों से सीखें, कमज़ोर क्षेत्रों का विश्लेषण | Maps/Diagrams से Bouncers में अंक।</t>
+  </si>
+  <si>
+    <t>Prelims + Mains की एकीकृत तैयारी | Small High-ROI Topics (Disaster Mgmt, Int. Security) को Priority | Prelims ज्ञान को Mains में Integrate करें।</t>
+  </si>
+  <si>
+    <t>Less is More — Content को Condense करें | GS विषयों को Interlink करके पढ़ें | Calculated Risk लें (90-95 Attempts)।</t>
+  </si>
+  <si>
+    <t>Basic Sources पर टिके रहें (FOMO से बचें) | Personality, Clear Communication, Balanced Thinking | Interview में Subject Knowledge से ज़्यादा Personality।</t>
+  </si>
+  <si>
+    <t>Newspaper के विस्तृत Notes में समय बर्बाद न करें | केवल महत्वपूर्ण Data/Examples नोट करें | परीक्षा के अंतिम 30 दिनों में कोई नया स्रोत नहीं।</t>
+  </si>
+  <si>
+    <t>Toppers की रणनीति अंधाधुंध Copy न करें | अपनी Strength-Weakness समझें और खुद की Strategy बनाएँ।</t>
+  </si>
+  <si>
+    <t>Mains = 50% Content + 50% Presentation | Bullets, Diagrams, Committees, Maps से Presentation | Strategic प्रश्न चयन।</t>
+  </si>
+  <si>
+    <t>27 साल के PYQs Theme-wise हल करें | Daily Answer Writing | Prelims की गहराई PYQs से समझें।</t>
+  </si>
+  <si>
+    <t>1. Consolidation: 10 किताबें नहीं, 1 Booklet 3-4 बार | 2. PYQs ही Source Code हैं | 3. FLTs से Generalist Mindset | 4. समय व स्थान प्रबंधन (Exam Hall जैसा) | 5. सकारात्मकता + मानसिक मजबूती।</t>
+  </si>
+  <si>
+    <t>Discipline &gt; Motivation | Social Media से पूरी दूरी | Family Support पर विश्वास।</t>
+  </si>
+  <si>
+    <t>रोज़ Exercise/Jogging (Stress Buster) | Social Media Apps Delete | Family से संवाद।</t>
+  </si>
+  <si>
+    <t>Hobbies न छोड़ें (Music, Walk, Reading) | Fact Sheets बनाएँ | Multiple Revisions।</t>
+  </si>
+  <si>
+    <t>कम पढ़ें, बार-बार दोहराएँ | Mind Mapping + Active Recall | Test Series से Assess करें | Sustainable Routine (Yoga, Badminton)।</t>
+  </si>
+  <si>
+    <t>पहला प्रयास सबसे गंभीरता से दें | असफलता पर Knowledge/Strategy Gap खोजें | Interview में प्रामाणिकता + तटस्थ प्रशासनिक दृष्टिकोण | 2-3 गंभीर प्रयासों के बाद Plan B खुले रखें।</t>
+  </si>
+  <si>
+    <t>Internal Drive से पढ़ें, बाहरी दबाव नहीं | शुरुआत में Plan B का Comfort Zone से बचें | परिस्थितियों को बहाना न बनने दें (Typhoid के बावजूद Mains दिया) | UPSC केवल परीक्षा नहीं, व्यक्तित्व विकास है।</t>
+  </si>
+  <si>
+    <t>10-अंक प्रश्न: 10-12 Points; 15-अंक: 15-17 Points | 4 Registers में Consolidated Notes, 7-8 बार Revision | PYQs सबसे पहले।</t>
+  </si>
+  <si>
+    <t>Attempt बढ़ाएँ (90+) | Limited Sources को बार-बार Revise करें | Monthly Break लें।</t>
+  </si>
+  <si>
+    <t>अपनी तैयारी और Mentorship पर भरोसा | Resources सीमित | आत्मविश्वास न खोएँ।</t>
+  </si>
+  <si>
+    <t>गलतियों से सीखें | CSAT की गणितीय कमज़ोरी पहले पहचानें | फरवरी से Mock शुरू करें।</t>
+  </si>
+  <si>
+    <t>Prelims ज्ञान को Google Docs में Save करके Mains में उपयोग करें | High-ROI Small Subjects पर विशेष ध्यान।</t>
+  </si>
+  <si>
+    <t>नोट्स को Mental रूप से Condense करते जाएँ | GS1-GS4 को अलग-अलग नहीं, Interlinked पढ़ें।</t>
+  </si>
+  <si>
+    <t>FOMO से बचें | Basic Sources पर विश्वास | Interview के लिए Balanced Personality विकसित करें।</t>
+  </si>
+  <si>
+    <t>अंतिम 30 दिन: No New Source | PYQs को Daily Mock की तरह लें | Newspaper Notes Minimal रखें।</t>
+  </si>
+  <si>
+    <t>Optional बदलने से मत डरें | PYQs ही सबसे बड़ा हथियार | Dedicated Mains Preparation Period रखें।</t>
+  </si>
+  <si>
+    <t>कठिन पेपर में घबराएँ नहीं, Strategic प्रश्न चयन करें | Presentation को Content जितना महत्व दें।</t>
+  </si>
+  <si>
+    <t>PYQs को थीम-वार Compile करें | Daily Answer Writing अनिवार्य।</t>
+  </si>
+  <si>
+    <t>तैयारी को नौकरी की तरह लें (8-10 घंटे) | Social Media/New Material से बचें | अपने Resources पर विश्वास | विफलता से सीखें (Over-Attempt Analysis)।</t>
+  </si>
+  <si>
+    <t>तैयारी की कमान खुद संभालें | अपने निर्णयों पर भरोसा | Social Media Delete करें।</t>
+  </si>
+  <si>
+    <t>रुकें नहीं, निरंतर प्रयास | अपनी क्षमता पर विश्वास | Daily Exercise से Mental Fitness।</t>
+  </si>
+  <si>
+    <t>असफलता से सीखें | Sources सीमित रखें | Revision + Mock Tests पर Focus।</t>
+  </si>
+  <si>
+    <t>College 1st-2nd Year: Personality Development + Newspaper आदत | College Gaps में Library/Hostel में Standard Books पढ़ें।</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -438,21 +1245,54 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1C2833"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFEBF5FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF5FB"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFAED6F1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFAED6F1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFAED6F1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFAED6F1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -473,11 +1313,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -818,283 +1658,1286 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U16384"/>
+  <dimension ref="A1:S16384"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11" style="3"/>
-    <col min="2" max="2" width="25.5" style="6" customWidth="1"/>
-    <col min="3" max="5" width="11" style="2"/>
-    <col min="6" max="6" width="11" style="3"/>
-    <col min="7" max="7" width="44.25" style="3" customWidth="1"/>
-    <col min="8" max="8" width="19.5" style="3" customWidth="1"/>
-    <col min="9" max="9" width="23.625" style="3" customWidth="1"/>
-    <col min="10" max="17" width="19.5" style="3" customWidth="1"/>
-    <col min="18" max="19" width="11" style="3"/>
-    <col min="20" max="20" width="40.625" style="3" customWidth="1"/>
-    <col min="22" max="16384" width="11" style="2"/>
+    <col min="1" max="1" width="19.5" style="3" customWidth="1"/>
+    <col min="2" max="20" width="19.625" style="2" customWidth="1"/>
+    <col min="21" max="16384" width="11" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>21</v>
+        <v>103</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="P1" s="5" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="Q1" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="R1" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="S1" s="5" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>22</v>
+        <v>103</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q2" s="5" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="R2" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="6">
-        <v>2</v>
+      <c r="B3" s="6" t="s">
+        <v>120</v>
       </c>
-      <c r="C3" s="2">
-        <v>45</v>
+      <c r="C3" s="6" t="s">
+        <v>121</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="P3" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="Q3" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="S3" s="6" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="6">
-        <v>2021</v>
+      <c r="B4" s="5" t="s">
+        <v>137</v>
       </c>
-      <c r="C4" s="2">
-        <v>2028</v>
+      <c r="C4" s="5" t="s">
+        <v>137</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D4" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>23</v>
+        <v>145</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>118</v>
+      <c r="C5" s="6" t="s">
+        <v>146</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D5" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="M5" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="O5" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q5" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="R5" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="S5" s="6" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="6">
-        <v>2</v>
+      <c r="B6" s="5" t="s">
+        <v>156</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="C6" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="S6" s="5" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>24</v>
+      <c r="B7" s="6" t="s">
+        <v>167</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="63" x14ac:dyDescent="0.25">
+      <c r="C7" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="M7" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="N7" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="O7" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="P7" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="Q7" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="R7" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="S7" s="6" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>25</v>
+        <v>173</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="C8" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="N8" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="P8" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="Q8" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="R8" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="S8" s="5" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>26</v>
+      <c r="B9" s="6" t="s">
+        <v>191</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>119</v>
+      <c r="C9" s="6" t="s">
+        <v>192</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="126" x14ac:dyDescent="0.25">
+      <c r="D9" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="M9" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="N9" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="O9" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="P9" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q9" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="R9" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="S9" s="6" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" ht="204" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>27</v>
+        <v>209</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>120</v>
+      <c r="C10" s="5" t="s">
+        <v>210</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="D10" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="M10" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="N10" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="O10" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="P10" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="Q10" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="R10" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="S10" s="5" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" ht="178.5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>28</v>
+      <c r="B11" s="6" t="s">
+        <v>227</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>121</v>
+      <c r="C11" s="6" t="s">
+        <v>228</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="D11" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="M11" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="N11" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="O11" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="P11" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="Q11" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="R11" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="S11" s="6" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" ht="204" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>29</v>
+        <v>245</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>122</v>
+      <c r="C12" s="5" t="s">
+        <v>246</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="63" x14ac:dyDescent="0.25">
+      <c r="D12" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="J12" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="L12" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="M12" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="N12" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="O12" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="P12" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="Q12" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="R12" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="S12" s="5" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" ht="229.5" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>30</v>
+      <c r="B13" s="6" t="s">
+        <v>263</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>123</v>
+      <c r="C13" s="6" t="s">
+        <v>264</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" ht="63" x14ac:dyDescent="0.25">
+      <c r="D13" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="L13" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="M13" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="N13" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="O13" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="P13" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="Q13" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="R13" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="S13" s="6" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" ht="191.25" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>31</v>
+        <v>280</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>124</v>
+      <c r="C14" s="5" t="s">
+        <v>281</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="D14" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="L14" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="M14" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="N14" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="O14" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="P14" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="Q14" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="R14" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="S14" s="5" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" ht="229.5" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="5" t="s">
-        <v>32</v>
+      <c r="B15" s="6" t="s">
+        <v>298</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>125</v>
+      <c r="C15" s="6" t="s">
+        <v>299</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="D15" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>302</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>304</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="M15" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="N15" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="O15" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="P15" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="Q15" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="R15" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="S15" s="6" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" ht="165.75" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>33</v>
+        <v>313</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>126</v>
+      <c r="C16" s="5" t="s">
+        <v>314</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" ht="63" x14ac:dyDescent="0.25">
+      <c r="D16" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>320</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>321</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>322</v>
+      </c>
+      <c r="L16" s="5" t="s">
+        <v>323</v>
+      </c>
+      <c r="M16" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="N16" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="O16" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="P16" s="5" t="s">
+        <v>327</v>
+      </c>
+      <c r="Q16" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="R16" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="S16" s="5" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" ht="127.5" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="5" t="s">
-        <v>34</v>
+      <c r="B17" s="6" t="s">
+        <v>331</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>127</v>
+      <c r="C17" s="6" t="s">
+        <v>332</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="D17" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="L17" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="M17" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="N17" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="O17" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="P17" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="Q17" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="R17" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="S17" s="6" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>35</v>
+        <v>343</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>128</v>
+      <c r="C18" s="5" t="s">
+        <v>344</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="D18" s="5" t="s">
+        <v>345</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>348</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="J18" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="K18" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="L18" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="M18" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="N18" s="5" t="s">
+        <v>351</v>
+      </c>
+      <c r="O18" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="P18" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="Q18" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="R18" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="S18" s="5" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="5">
-        <v>173</v>
+      <c r="B19" s="6" t="s">
+        <v>355</v>
       </c>
-      <c r="C19" s="2">
-        <v>175</v>
+      <c r="C19" s="6" t="s">
+        <v>356</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D19" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="L19" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="M19" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="N19" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="O19" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="P19" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="Q19" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="R19" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="S19" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" ht="140.25" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="5">
-        <v>932</v>
+      <c r="B20" s="5" t="s">
+        <v>363</v>
       </c>
-      <c r="C20" s="2">
-        <v>865</v>
+      <c r="C20" s="5" t="s">
+        <v>364</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" ht="157.5" x14ac:dyDescent="0.25">
+      <c r="D20" s="5" t="s">
+        <v>365</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>370</v>
+      </c>
+      <c r="J20" s="5" t="s">
+        <v>371</v>
+      </c>
+      <c r="K20" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="L20" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="M20" s="5" t="s">
+        <v>374</v>
+      </c>
+      <c r="N20" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="O20" s="5" t="s">
+        <v>376</v>
+      </c>
+      <c r="P20" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="Q20" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="R20" s="5" t="s">
+        <v>379</v>
+      </c>
+      <c r="S20" s="5" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" ht="102" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="5" t="s">
-        <v>36</v>
+      <c r="B21" s="6" t="s">
+        <v>381</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>129</v>
+      <c r="C21" s="6" t="s">
+        <v>382</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D21" s="6" t="s">
+        <v>383</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>384</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>389</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="L21" s="6" t="s">
+        <v>391</v>
+      </c>
+      <c r="M21" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="N21" s="6" t="s">
+        <v>393</v>
+      </c>
+      <c r="O21" s="6" t="s">
+        <v>394</v>
+      </c>
+      <c r="P21" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="Q21" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="R21" s="6" t="s">
+        <v>397</v>
+      </c>
+      <c r="S21" s="6" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
-      <c r="B22" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
@@ -50155,6 +51998,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -50172,358 +52016,386 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F17"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.375" customWidth="1"/>
-    <col min="3" max="3" width="15.875" customWidth="1"/>
+    <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.75" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="50.125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="B1" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="C1" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="D1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E1" t="s">
+      <c r="C2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F1" t="s">
+      <c r="D2" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>106</v>
+    <row r="18" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>100</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B18" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>59</v>
-      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F17" xr:uid="{00000000-0001-0000-0200-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Sadaf Choudhary / Naomi Satam"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError sqref="B1:F1" numberStoredAsText="1"/>
@@ -50550,36 +52422,36 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="D2" s="1">
         <v>2023</v>
@@ -50588,13 +52460,13 @@
         <v>200</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: restructure strategy tab, move blueprints to setup, add main details marks, fix localstorage bug
</commit_message>
<xml_diff>
--- a/Update_App_Data/upsc_toppers_data.xlsx
+++ b/Update_App_Data/upsc_toppers_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\Storage  Driver\upsc-cse-master-hub\Update_App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6945E4DF-1237-4C6C-9CB3-E346991AD4F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8079D5F0-F8D7-4064-A1FB-DEB0AA4BCC2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,12 +21,23 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Routines!$A$1:$F$17</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="399">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="222">
   <si>
     <t>id</t>
   </si>
@@ -496,12 +507,6 @@
     <t>Economics (286 अंक)</t>
   </si>
   <si>
-    <t>N/A (स्रोत में उल्लेखित नहीं)</t>
-  </si>
-  <si>
-    <t>3rd (CSAT fail in 2nd attempt)</t>
-  </si>
-  <si>
     <t>4th</t>
   </si>
   <si>
@@ -514,19 +519,10 @@
     <t>1st</t>
   </si>
   <si>
-    <t>5th (4th Attempt में बिना Mock के सफलता)</t>
-  </si>
-  <si>
     <t>6th</t>
   </si>
   <si>
     <t>5th</t>
-  </si>
-  <si>
-    <t>5th (2020 से)</t>
-  </si>
-  <si>
-    <t>2nd (1st में Prelims Fail → 6 माह Prelims Focus)</t>
   </si>
   <si>
     <t>PCB (Bio) पृष्ठभूमि</t>
@@ -599,522 +595,6 @@
   </si>
   <si>
     <t>"Motivation is a lie, discipline is real." | "Rank is merely a number until given meaning through dedicated service." | "नदी को किनारे खड़े होकर देखते रहने से नदी पार नहीं होती, प्रयास करना पड़ता है।"</t>
-  </si>
-  <si>
-    <t>Smart Work &gt; Brute Force। एक विषय – एक किताब। दिसंबर तक Mains Ready (Optional, Ethics, Essay, 1-page GS Notes)। थीम-बेस्ड करंट अफेयर्स नोट्स (GS 1-4 कीवर्ड्स अनुसार)। दैनिक 8-10 घंटे को 4 स्लॉट में बाँटना।</t>
-  </si>
-  <si>
-    <t>4-ब्लॉक Target Model (8-9 घंटे गुणवत्ता अध्ययन) | Integrated Approach (Prelims+Mains+Interview एकसाथ) | PYQs को सर्वश्रेष्ठ मित्र बनाना | 5+1+1 नियम (5 पढ़ाई + 1 Buffer + 1 Revision)।</t>
-  </si>
-  <si>
-    <t>सीमित स्रोत + 4 Register में Consolidated Notes + 7-8 बार Revision | Topper Copies (Aditya Srivastava, Maidan Ji) से Answer Structuring + Cross-fertilization | PYQs पर केंद्रित।</t>
-  </si>
-  <si>
-    <t>सीमित किताबें + बहुस्तरीय Revision + गलतियों का सूक्ष्म विश्लेषण | Spectrum को 25 ऑनलाइन पेजों में Condense किया।</t>
-  </si>
-  <si>
-    <t>असीमित सामग्री से बचना | AI Tools (ChatGPT/Gemini) का सारांश व उदाहरण के लिए उपयोग | Monthly/Yearly Magazines के Index Page पर Concise Notes।</t>
-  </si>
-  <si>
-    <t>One Source – Multiple Revisions | फरवरी से Sectional Tests फिर FLTs | PYQs के चारों विकल्पों का गहन विश्लेषण।</t>
-  </si>
-  <si>
-    <t>PYQ Mapping से Themes निकालना | छोटे High-Return विषयों (Internal Security, Disaster Management, Social Justice) पर Special Focus | Prelims ज्ञान → Google Docs → Mains में प्रयोग।</t>
-  </si>
-  <si>
-    <t>'Less is More' — Notes को Maximum Condense | GS1-GS4 को Interlink करके पढ़ना | गणितीय दृष्टिकोण से Essay को 5Ws में तोड़ना।</t>
-  </si>
-  <si>
-    <t>FOMO से बचाव — केवल NCERT + Laxmikanth | PYQs Brainstorming → Topper Copies से Matching | Interview: Personality + Clear Communication।</t>
-  </si>
-  <si>
-    <t>PYQs (2013 से) को Daily Mock की तरह हल करना | Limited Sources + Minimal Newspaper Notes | अंतिम 30 दिन: No New Source।</t>
-  </si>
-  <si>
-    <t>4th Attempt: बिना किसी Coaching Mock के केवल 10 वर्षों (2014 से) के PYQs का गहन विश्लेषण | Optional बदलकर Anthropology + 1 साल का Break लेकर Mains मज़बूत किया।</t>
-  </si>
-  <si>
-    <t>50% Content + 50% Presentation | Bullets, Committee Names, Flowcharts, Maps | कठिन पेपर में घबराने के बजाय 65 मज़बूत प्रश्न चुनना।</t>
-  </si>
-  <si>
-    <t>27 साल के PYQs की Theme-wise Compilation | 99 प्रश्न Attempt | Answer Writing Simulation + Daily Writing।</t>
-  </si>
-  <si>
-    <t>Less is More (सीमित स्रोत, 3-4 बार Revision) | Consolidated Notes (A4 Sheets पर: NCERTs + Static + PYQs + Test Synopsis) | FLTs Only (2-3 Coaching के Full Length Tests) | पेपर पूरा करना अनिवार्य।</t>
-  </si>
-  <si>
-    <t>घर पर तैयारी (बिना Coaching Hub) | सुबह 5 बजे से कड़ा Daily Routine | Self-Discipline + Family Support।</t>
-  </si>
-  <si>
-    <t>Goldman Sachs छोड़कर Full-Time Preparation | अनुशासित रहना + Self-Doubt से उबरना | Daily Current Affairs Notes | 1.5 माह पहले Daily Mock।</t>
-  </si>
-  <si>
-    <t>5-Page Fact Sheets (प्रति Subject) | 3-Round Paper Solving | 35 Mock Tests (गहन Revision) | Limited Sources।</t>
-  </si>
-  <si>
-    <t>Discipline &gt; Motivation | 80/20 नियम: 80% प्रश्न 20% Core Syllabus से | सीमित स्रोत, 3-4 बार Revision | Syllabus + PYQs को Guide बनाना।</t>
-  </si>
-  <si>
-    <t>अंक: 112 | इतिहास: TN Board Cl-11 NCERT + Spectrum/Bipin Chandra | भूगोल: Cl-11,12 NCERTs + Atlas | समाज: उत्कर्ष द्विवेदी टेम्पलेट + NCERT + NFHS/ASER डेटा | विश्व इतिहास: Vision IAS बुकलेट + PYQs।</t>
-  </si>
-  <si>
-    <t>भूगोल: Cl-11,12 NCERTs + Maps अभ्यास | इतिहास: Spectrum/PW Udaan (Modern) + पुरानी NCERTs (Ancient/Medieval) | Art &amp; Culture: NCERTs + Stick Figures (नटराज आदि) | प्रतिदिन 30 मिनट Modern History।</t>
-  </si>
-  <si>
-    <t>विभिन्न GS Papers के ज्ञान को Cross-fertilize करके उत्तर लिखे | 2-3 पेज Concise Notes प्रति विषय।</t>
-  </si>
-  <si>
-    <t>History: Modern → Spectrum (25 pages में condense) + NCERTs (R.S. Sharma, Satish Chandra, Bipan Chandra) | Society: Smriti Ma'am Notes | Comparative Charts: राष्ट्रपति vs राज्यपाल आदि।</t>
-  </si>
-  <si>
-    <t>समाचार पत्र की जगह Monthly/Yearly Magazines के Index Page पर Short Notes + बार-बार Revision।</t>
-  </si>
-  <si>
-    <t>इतिहास/भूगोल के कठिन प्रश्नों में Maps + Diagrams बनाकर अंक खींचे | PYQs (2013 के बाद) के चारों Options का गहन विश्लेषण।</t>
-  </si>
-  <si>
-    <t>PYQs से Themes → Short Notes | Core (Polity, Economy) + Science &amp; Tech + Environment पर महारत।</t>
-  </si>
-  <si>
-    <t>GS विषयों को आपस में Interlink करके पढ़ें | Condensed Notes।</t>
-  </si>
-  <si>
-    <t>NCERT + Basic Sources — FOMO से बचते हुए।</t>
-  </si>
-  <si>
-    <t>History: Spectrum | Art &amp; Culture: NCERTs।</t>
-  </si>
-  <si>
-    <t>PYQ गहन विश्लेषण पर आधारित।</t>
-  </si>
-  <si>
-    <t>50% Content + 50% Presentation | Maps, Diagrams का प्रयोग।</t>
-  </si>
-  <si>
-    <t>27 साल के PYQs से Themes + Answer Writing।</t>
-  </si>
-  <si>
-    <t>अंक: 110+ (लगातार) | इतिहास (Modern): Spectrum → Short Notes + Revision | इतिहास (Ancient/Medieval): TN Board Cl-11, Cl-12 Themes in Indian History | भूगोल: 11-12 NCERTs + PMF IAS Selective + YouTube (Dr. Shivin, Sleepy Classes) | Society: Sociology Optional का ओवरलैप + PYQ Themes + Model Answers।</t>
-  </si>
-  <si>
-    <t>Laxmikanth (Polity) + Basic History NCERTs।</t>
-  </si>
-  <si>
-    <t>Geography: NCERTs (Mandatory) | History: NCERTs (Ancient/Medieval)।</t>
-  </si>
-  <si>
-    <t>History: TN Board 11th + Old NCERTs + CC Leong | Society: Vision Notes।</t>
-  </si>
-  <si>
-    <t>Ancient/Medieval: Old NCERT/R.S. Sharma | Art &amp; Culture: 11th Fine Arts NCERT।</t>
-  </si>
-  <si>
-    <t>अंक: 125 | पॉलिटी: Laxmikanth (Margin Notes) + Abhay Kumar 500 MCQs | शासन: 2nd ARC, सुप्रीम कोर्ट निर्णय | IR: PSIR Optional नोट्स का ओवरलैप + करंट (BRICS, SCO, G20, BIMSTEC) | सामाजिक न्याय: उत्कर्ष टेम्पलेट + SHG/NABARD डेटा।</t>
-  </si>
-  <si>
-    <t>पॉलिटी: Vision IAS Foundation Notes (Amirul Hasan Sir) + Laxmikanth (Margin में नोट्स) | IR: PSIR Optional से भारी ओवरलैप | Governance: Indian Express पैसिव रीडिंग।</t>
-  </si>
-  <si>
-    <t>GS1-GS4 Cross-fertilization | 2-3 पेज नोट्स | Committee Recommendations + Articles का समावेश।</t>
-  </si>
-  <si>
-    <t>Polity: Laxmikanth + 11th NCERT (Constitution at Work) | IR: Shubhra Ranjan + ORF + Indian Express + The Hindu + Jaishankar Speeches | Governance: Committee Recommendations।</t>
-  </si>
-  <si>
-    <t>प्रत्येक GS Paper: केवल 30-35 Pages के Short Notes | Pointer Format: 10-अंक → 8-10 Points, 15-अंक → 12-13 Points।</t>
-  </si>
-  <si>
-    <t>Articles + Committee Recommendations समावेश + Pointwise | Supreme Court Judgements का उल्लेख।</t>
-  </si>
-  <si>
-    <t>Polity + Governance + IR → PYQ Theme Analysis | Prelims के तथ्य → Google Docs → Mains उत्तर।</t>
-  </si>
-  <si>
-    <t>GS1-GS4 Interlinking Strategy।</t>
-  </si>
-  <si>
-    <t>Laxmikanth + NCERT | PYQ Brainstorming + Topper Copy Matching।</t>
-  </si>
-  <si>
-    <t>Polity: 11th NCERTs (Political Theory + Constitution at Work) + Laxmikanth | IR: Current-based।</t>
-  </si>
-  <si>
-    <t>PYQ गहन विश्लेषण + Limited Sources।</t>
-  </si>
-  <si>
-    <t>Bullet Points + Committee Names + Constitutional Articles।</t>
-  </si>
-  <si>
-    <t>PYQ Theme Analysis + Daily Writing।</t>
-  </si>
-  <si>
-    <t>अंक: ~118 | Polity: Laxmikanth (Highlight + बार-बार पढ़ना) + 11th NCERT Political Theory | Governance: 2nd ARC, Mallimath Committee + Constitutional Articles + Health/Education Frameworks (ASER, TSR Subramanian) | IR: Next IAS (Deepin Sir) Notes — 5-6 बार Revision | Social Justice: PYQ Themes।</t>
-  </si>
-  <si>
-    <t>The Hindu / Indian Express + Drishti Daily News Analysis।</t>
-  </si>
-  <si>
-    <t>Polity: Laxmikanth।</t>
-  </si>
-  <si>
-    <t>Polity: Laxmikanth + Mains 365 | MEA Statements + Committee Recommendations | IR: Current।</t>
-  </si>
-  <si>
-    <t>Polity: Laxmikanth (5-6 बार Revision) | Parliament, Judiciary, FRs, DPSPs पर विशेष ध्यान | Supreme Court Cases + Articles।</t>
-  </si>
-  <si>
-    <t>अंक: 86 | अर्थव्यवस्था: Shriram IAS Notes + Budget/Eco Survey (Jayant Sir) + Shivin Sir GS3 Template | आंतरिक सुरक्षा: Shivin Sir Template + अद्यतन डेटा | आपदा: NDMA Template (Utkarsh Dwivedi) | Environment &amp; S&amp;T: Annual Mains Compilations।</t>
-  </si>
-  <si>
-    <t>Economy+Environment+Security: Vision IAS Mains 365 | Budget: 2 पेज क्रिस्प नोट्स | Eco Survey: 3 पेज | Environment Mains 365: 6 पेज | Visual Presentation: Trend Graphs, Flowcharts, Infographics।</t>
-  </si>
-  <si>
-    <t>2-3 पेज नोट्स | Prelims में एकत्र ज्ञान/तथ्य Google Docs में सहेजकर Mains में प्रयोग।</t>
-  </si>
-  <si>
-    <t>GS3: Science &amp; Tech + Environment → Mains 365 | Internal Security → Shivin Sir Notes।</t>
-  </si>
-  <si>
-    <t>30-35 पेज Short Notes | Committee Names, Data, Schemes का समावेश।</t>
-  </si>
-  <si>
-    <t>स्रोत में विशिष्ट GS3 विवरण नहीं, सीमित स्रोत + Revision।</t>
-  </si>
-  <si>
-    <t>Internal Security: Vajiram Yellow Book | Disaster Management: Google का विस्तृत उपयोग | High-ROI Small Subjects पर विशेष ध्यान।</t>
-  </si>
-  <si>
-    <t>GS1-GS4 Interlinking + Condensed Notes।</t>
-  </si>
-  <si>
-    <t>Limited Sources + PYQ Analysis।</t>
-  </si>
-  <si>
-    <t>Economy: Vivek Singh + Budget &amp; Economic Survey Summary।</t>
-  </si>
-  <si>
-    <t>PYQ गहन विश्लेषण।</t>
-  </si>
-  <si>
-    <t>Flowcharts, Maps, Diagrams से Presentation।</t>
-  </si>
-  <si>
-    <t>PYQ-based Preparation + Daily Answer Writing।</t>
-  </si>
-  <si>
-    <t>अर्थव्यवस्था: Budget + Eco Survey से Data/Graphs + Mrunal Sir Free Lectures (YouTube) | कृषि: Ministry Schemes + Dryland Farming + PYQs + Crop Map | S&amp;T: PT365/Mains365 + Blockchain/IoT/Nuclear | Disaster Management: 2013-2024 सभी PYQs Model Format में | Environment: ISFR, UNEP Reports + Current Facts।</t>
-  </si>
-  <si>
-    <t>Newspaper Reading + Basic NCERTs का एकीकरण।</t>
-  </si>
-  <si>
-    <t>Economy: बार-बार पढ़कर महारत (शुरुआत में कठिन था)।</t>
-  </si>
-  <si>
-    <t>Economy: Optional से Covered | S&amp;T: Mains 365 | Security: Notes + Maps/Diagrams।</t>
-  </si>
-  <si>
-    <t>Economy: Shankar Ganesh (150 pages) / Mrunal Notes + Budget &amp; Eco Survey।</t>
-  </si>
-  <si>
-    <t>अंक: 141 (देश में सर्वोच्च में से एक, बिना कोचिंग) | 100 कीवर्ड्स (Syllabus 25-30 + PYQs 50-60) | हर कीवर्ड: परिभाषा + Quote + सिविल सेवक उदाहरण + केस स्टडी | Prahar Magazine बुकलेट + The Better India | दार्शनिक: Aristotle, Plato, Kant, Hannah Arendt | समय: Section A → 1h15m, Case Studies → 1h45m।</t>
-  </si>
-  <si>
-    <t>पसंदीदा विषय | Case Studies: Hub &amp; Spoke Model (Stakeholders) + Pros/Cons Table | समय: Theory → 1h15m, Case Studies → शेष | किसी rigid structure के बिना व्यक्तित्व दिखाएँ।</t>
-  </si>
-  <si>
-    <t>Case Studies: सामान्य सुझावों के बजाय स्पष्ट व्यावहारिक समाधान | Essay: रोजाना एक विषय पर Brainstorming Notes।</t>
-  </si>
-  <si>
-    <t>Ethics: Ansari Sir (Lukman IAS) Notes | 'The Better India' से Real Examples | Ramayana/Mahabharata से नैतिक पाठ | Topper Copies (Shruti Ma'am, Vishakha Ma'am)।</t>
-  </si>
-  <si>
-    <t>Ethics: प्रत्येक उत्तर में कम से कम एक Indian/Western Philosopher का उल्लेख | Case Studies: 3-4 Pre-set Templates (Stakeholder Approach, Values Approach)।</t>
-  </si>
-  <si>
-    <t>Ethics: पहले 10-अंकीय प्रश्न, फिर Case Studies, अंत में Quotation-based प्रश्न हल किए।</t>
-  </si>
-  <si>
-    <t>Essay: स्वामी विवेकानंद के विचार, INA Trial, 'Tryst with Destiny' जैसे ऐतिहासिक संदर्भ।</t>
-  </si>
-  <si>
-    <t>स्रोत में विशिष्ट GS4 विवरण नहीं।</t>
-  </si>
-  <si>
-    <t>PYQ Brainstorming + Model Answer Comparison।</t>
-  </si>
-  <si>
-    <t>Mains के लिए 6-7 माह समर्पित।</t>
-  </si>
-  <si>
-    <t>Practical Solutions + Clear Framework।</t>
-  </si>
-  <si>
-    <t>Daily Writing Practice।</t>
-  </si>
-  <si>
-    <t>अंक: 129 | Section A: Ready-made Frameworks/Templates (Personal/Professional/Social, Concentric Circles) + Diverse Examples (Bhagavad Gita, IPS CAA Protest, Zomato Delivery Boy) + Sakshi Ma'am Mentorship (Vajiram) | Case Studies: Stakeholder के लिए Creative Diagrams (Forest Cutting में Tree Drawing) + Clear Option Selection + Positive Conclusion।</t>
-  </si>
-  <si>
-    <t>Case Studies अभ्यास + Daily Events से Critical Thinking।</t>
-  </si>
-  <si>
-    <t>स्रोत में विशिष्ट GS4 Strategy नहीं।</t>
-  </si>
-  <si>
-    <t>DK Balaji Sir Book | Quotes/Definitions Notes | Section A: 1.5h, Case Studies: 1.5h।</t>
-  </si>
-  <si>
-    <t>Syllabus Keywords की परिभाषाएँ + व्यावहारिक उदाहरण (2-3 Page Sheet)।</t>
-  </si>
-  <si>
-    <t>अंक: 100 | प्रति निबंध 1.5 घंटा (20-30 मिनट माइंड-मैप, 1 घंटा लेखन) | 15-16 बहु-आयामी GS आयाम | दोनों निबंधों का ढाँचा अलग | Haidt की 'The Anxious Generation' जैसे साहित्यिक संदर्भ।</t>
-  </si>
-  <si>
-    <t>अंक: 144 | 5 मिनट Timer → रफ पेज पर सभी आयाम (PESTEL) + Quotes | Anecdote/Quote से आकर्षक शुरुआत | Topper copies से Example Bank तैयार।</t>
-  </si>
-  <si>
-    <t>रोजाना एक दार्शनिक विषय पर Brainstorming Notes | Philosophical Essays में गहरी वैचारिक संरचना।</t>
-  </si>
-  <si>
-    <t>PYQs से मुख्य Themes (Problems, Causes, Solutions, Way Forward) पहचाने।</t>
-  </si>
-  <si>
-    <t>प्रत्येक GS Paper: 30-35 पेज Short Notes | PESTEL दृष्टिकोण।</t>
-  </si>
-  <si>
-    <t>PYQ Analysis + Toppers की Answer Copies से Structuring।</t>
-  </si>
-  <si>
-    <t>Essay: स्वामी विवेकानंद + INA Trial + Tryst with Destiny जैसे ऐतिहासिक संदर्भ | Multi-dimensional दृष्टिकोण।</t>
-  </si>
-  <si>
-    <t>Essay को 5Ws (How, What, Why, When, Who) में तोड़कर Structure | गणितीय दृष्टिकोण से रूपरेखा।</t>
-  </si>
-  <si>
-    <t>PYQs Brainstorming → Topper Copies से Matching।</t>
-  </si>
-  <si>
-    <t>Limited Sources + Revision।</t>
-  </si>
-  <si>
-    <t>Mains के लिए Dedicated 6-7 माह (Prelims से पहले)।</t>
-  </si>
-  <si>
-    <t>Multi-dimensional दृष्टिकोण + Diagrams।</t>
-  </si>
-  <si>
-    <t>Daily Answer Writing + PYQ Simulation।</t>
-  </si>
-  <si>
-    <t>अंक: 138 (2020 में) | Organic &amp; Simple लेखन (रटे-रटाए Formula से बचना) | Structure: Main Theme → पक्ष → 2 Para विपक्ष → Futuristic Conclusion | Framework 1: Individual→Family→Society→Nation→World | Framework 2: Ancient→Medieval→Modern→AI Age | बाहरी Feedback (माता-पिता, Prof.) लेना।</t>
-  </si>
-  <si>
-    <t>Quotes की जगह Real Stories/Case Studies से शुरुआत | 15-16 निबंध लिखे | Multi-dimensional दृष्टिकोण।</t>
-  </si>
-  <si>
-    <t>Prelims के बाद 6-7 Tests (कुल 12-14 निबंध) लिखे।</t>
-  </si>
-  <si>
-    <t>Multi-dimensional दृष्टिकोण | Quotes + Examples।</t>
-  </si>
-  <si>
-    <t>PESTLE Dimensions से Essay Link | 10-15 मिनट Brainstorming + Outline | Anecdote/Quotes से शुरुआत | Way Forward पर Positive Conclusion।</t>
-  </si>
-  <si>
-    <t>PSIR 280 अंक (2023: 230 → 2024: 280) | IGNOU सामग्री + Shriram/Vajiram नोट्स | सितंबर तक Syllabus + PYQs पूरे | 40% दैनिक समय | विचारक + खंडन एकसाथ | IR Paper 2B में करंट इंटीग्रेट।</t>
-  </si>
-  <si>
-    <t>PSIR | PYQs: 2013-2023 Topic-Wise | हर Topic: 2-4 Thinkers (पक्ष+विपक्ष) | तकनीकी शब्दावली | GS2 IR से भारी ओवरलैप।</t>
-  </si>
-  <si>
-    <t>Sociology 290 अंक | 4 मुख्य Register + 4 छोटे Handouts (अंतिम समय हेतु) | Durkheim के सिद्धांत → वर्तमान उदाहरण से जोड़ना | Thinkers को Current Affairs से Link।</t>
-  </si>
-  <si>
-    <t>PSIR: Shubhra Ranjan 80% Base | ORF, Indian Express, The Hindu, Jaishankar Interviews से Value Addition।</t>
-  </si>
-  <si>
-    <t>Economics: Paper 2 को GS3 Indian Economy से Integrate किया | Arjun Gupta Sir के Topper Notes।</t>
-  </si>
-  <si>
-    <t>PSIR: O.P. Gauba, Andrew Heywood (Global Politics) | 20 व 15 अंक वाले प्रश्नों को प्राथमिकता।</t>
-  </si>
-  <si>
-    <t>Political Science/Sociology | PYQ-based तैयारी।</t>
-  </si>
-  <si>
-    <t>स्रोत में विशिष्ट Optional Strategy नहीं।</t>
-  </si>
-  <si>
-    <t>Anthropology (Public Administration से Switch) | 1 साल का Break लेकर Mains को मज़बूत किया।</t>
-  </si>
-  <si>
-    <t>Sociology: 284 अंक | Thinkers → Current Examples से Link।</t>
-  </si>
-  <si>
-    <t>Sociology: 277 अंक (2020) | B.Tech Background पर GS/Essay/Ethics Overlap | Sources: NCERT 11-12 + IGNOU BA | Value Addition: Tusharanshu Sir + Nitin Sangwan (Essential Sociology) + Ritzer (Selective) + LevelUp IAS + Shankar IAS Test Series | Integrated Notes (Paper 1+2 समान Topics) | Humanities Prof. शैली में Paragraph Format + 1-3 Thinkers प्रति उत्तर।</t>
-  </si>
-  <si>
-    <t>Sociology: उपलब्धता + रुचि के आधार पर चयन।</t>
-  </si>
-  <si>
-    <t>Sociology/Maths: Notes बनाना + PYQs पर विशेष जोर।</t>
-  </si>
-  <si>
-    <t>Economics: 144+142 = 286 अंक | H.L. Ahuja, Salvatore, Jhingan | Economic Survey + Budget।</t>
-  </si>
-  <si>
-    <t>Optional चयन के 4 पैमाने: Background/Interest + Syllabus Vastness + Competition Level + Guidance Availability।</t>
-  </si>
-  <si>
-    <t>अंक: 82 (Cutoff: 75) | नया पैटर्न + Shock Absorption माइंडसेट | PYQ थीम एनालिसिस (Art. 19, 21, 32 जैसे हाई-फ्रीक्वेंसी) | Jan-Feb: रिवीजन 1, Mar-15Apr: रिवीजन 2 | 3-इटरेशन पेपर सॉल्विंग | सबसे मज़बूत विषय (Polity) से शुरू।</t>
-  </si>
-  <si>
-    <t>2024 में 98 प्रश्न अटेम्प्ट | Vajiram Power Up Test Series (CA) + Vision IAS Abhyas Tests | Calculated Risk: 30-35 sure-shot + 50-50 elimination | अंतिम 27 दिन: कोई नया रिसोर्स नहीं, केवल नोट्स + PYQs।</t>
-  </si>
-  <si>
-    <t>फरवरी से प्रतिदिन 50 MCQs + सप्ताह में 2-3 Mock Tests | परीक्षा से 1 महीना पहले Mock बंद → केवल PYQs | The Hindu + Monthly Magazines (3-4 बार Revision) | CA के अलग नोट्स नहीं।</t>
-  </si>
-  <si>
-    <t>4th Attempt: 90+ प्रश्न हल किए (पहले 3 में 71-78 से Fail) | Source List: Polity-Laxmikanth+11NCERT, History-Spectrum, Economy-Vivek Singh, Environment-Shankar+PT365, Geography-Rishikesh Notes+11/12 NCERT | Comparative Tables।</t>
-  </si>
-  <si>
-    <t>जनवरी से ऑफलाइन Mock Tests + कमज़ोर विषयों का विश्लेषण | Monthly/Yearly Magazine Index पर Notes | CSAT: केवल PYQs।</t>
-  </si>
-  <si>
-    <t>फरवरी से Sectional Tests → FLTs | 2013 के बाद के PYQs के चारों विकल्पों का विश्लेषण।</t>
-  </si>
-  <si>
-    <t>PYQs से Themes निकालकर Short Notes | Core + Sci&amp;Tech + Environment में बढ़त (Bouncer प्रश्नों में लाभ)।</t>
-  </si>
-  <si>
-    <t>Risk Management: 90-95 प्रश्न हल करने का लक्ष्य | 30 प्रश्न गलत के Margin के बाद भी 100+ Net Positive।</t>
-  </si>
-  <si>
-    <t>FOMO से बचाव — केवल NCERT + Laxmikanth तक सीमित | CSAT: बिना नागा रोजाना अभ्यास + PYQs।</t>
-  </si>
-  <si>
-    <t>2013 के बाद के PYQs को दैनिक 25 प्रश्नों के Mock की तरह हल किया | Polity: 11th NCERTs + Laxmikanth | Economy: Vivek Singh + Budget | History: Spectrum।</t>
-  </si>
-  <si>
-    <t>4th Attempt: बिना Coaching Mock के, केवल पिछले 10 वर्षों (2014 से) के PYQs का गहन विश्लेषण।</t>
-  </si>
-  <si>
-    <t>2023 के कठिन पेपर में घबराए नहीं | 65 मज़बूत प्रश्न पहले चुने → 88 प्रश्न हल किए।</t>
-  </si>
-  <si>
-    <t>27 साल के PYQs की Theme-wise Compilation | 99 प्रश्न Attempt।</t>
-  </si>
-  <si>
-    <t>Less is More — 3 बार Revision | केवल 15+ Full Length Tests (Vision, Forum, Vajiram) | PYQs (2013 से): सभी Options का गहन विश्लेषण + Notes में समाहित | 2021: 100 प्रश्न → &lt;1 अंक से Fail → Calculated Risk (80-95 प्रश्न) | Current Affairs: PT365 + Newspaper 30 मिनट (Ethics/Essay Examples)।</t>
-  </si>
-  <si>
-    <t>1991 से PYQs Solve | अंतिम 2 माह: Daily Mock Tests | घर पर Exam जैसा माहौल।</t>
-  </si>
-  <si>
-    <t>Daily Current Affairs Notes | Prelims से 1.5 माह पहले रोज़ एक Mock Test।</t>
-  </si>
-  <si>
-    <t>35 Mock Tests (गहन Revision) | 5-Page Fact Sheets (प्रति Subject) | 3 Rounds में Paper Solve।</t>
-  </si>
-  <si>
-    <t>1st Attempt Prelims Fail → 6 माह केवल Prelims Focus | एक विषय 10 दिन → Test (Vision/Insights) → 2 दिन Revision → अगला विषय।</t>
-  </si>
-  <si>
-    <t>अंक: 75 | PCB बैकग्राउंड, 10वीं के बाद Maths नहीं | RC: 25-28 प्रश्न (उच्च सटीकता) | Reasoning: 10-15 प्रश्न | Quant: Time-Work, SDT, Percentage, Number System | कुल 45-50 प्रश्न टार्गेट।</t>
-  </si>
-  <si>
-    <t>2nd Attempt में CSAT fail → 3rd में विशेष ध्यान | NDA, CDS, CPSC के पिछले 3 साल के CSAT Papers | RC: प्रश्न पहले पढ़ें → Extreme Options तुरंत खारिज | 27-28 RC में से 22+ सही टार्गेट।</t>
-  </si>
-  <si>
-    <t>स्रोत में विशिष्ट उल्लेख नहीं।</t>
-  </si>
-  <si>
-    <t>Comprehension के लिए केवल UPSC PYQs को मुख्य आधार।</t>
-  </si>
-  <si>
-    <t>CSAT: गणितीय कमज़ोरी पहचानकर Number System, Average, Calendar जैसे High-Yield Topics के लिए Crash Course + अभ्यास।</t>
-  </si>
-  <si>
-    <t>बिना नागा रोजाना प्रश्न अभ्यास | Comprehension के लिए केवल PYQs।</t>
-  </si>
-  <si>
-    <t>R.S. Aggarwal पुस्तक + नियमित अभ्यास।</t>
-  </si>
-  <si>
-    <t>पिछले 5 साल के PYQs → 2 घंटे Time-bound | Formula Sheet (1 Page): Mathematical Formulas, Tricks, Reasoning Rules → GS1-GS2 Break में Revise | 53 Maths/Reasoning में से 27-28 Easy + Comprehension ध्यान से।</t>
-  </si>
-  <si>
-    <t>रोजाना 15-20 मिनट Logical Reasoning + Quant अभ्यास।</t>
-  </si>
-  <si>
-    <t>Mental Ability + Maths पर भरोसा + पुराने Papers Solve।</t>
-  </si>
-  <si>
-    <t>English में Comfortable (30 प्रश्न) | Maths/Reasoning में Selective।</t>
-  </si>
-  <si>
-    <t>Logical Elimination + 50-50 वाले प्रश्नों में Net Positive Strategy।</t>
-  </si>
-  <si>
-    <t>200 / 275</t>
-  </si>
-  <si>
-    <t>187 / 275</t>
-  </si>
-  <si>
-    <t>स्रोत में उल्लेखित नहीं | Mock Interviews से Stage Fear दूर | IR + Newspapers पर विशेष ध्यान।</t>
-  </si>
-  <si>
-    <t>201 / 275</t>
-  </si>
-  <si>
-    <t>स्रोत में उल्लेखित नहीं।</t>
-  </si>
-  <si>
-    <t>206 / 275</t>
-  </si>
-  <si>
-    <t>216 / 275 (Suman Sharma Board)</t>
-  </si>
-  <si>
-    <t>180 / 275 (Sanjay Verma Board)</t>
-  </si>
-  <si>
-    <t>198 / 275</t>
-  </si>
-  <si>
-    <t>195 / 275 (2020: 160 → 2024: 195)</t>
-  </si>
-  <si>
-    <t>204 / 275 (Manoj Soni Board)</t>
-  </si>
-  <si>
-    <t>1st: 176 अंक | 2nd: 200 अंक</t>
-  </si>
-  <si>
-    <t>लिखित: 843/1750 | कुल (Mains+Interview): 1043/2025 | GS1:112, GS2:125, GS3:86, GS4:141, Essay:100, PSIR:280</t>
-  </si>
-  <si>
-    <t>लिखित: 851/1750 | कुल (Mains+Interview): 1038/2025 | Essay: 144, PSIR Optional</t>
-  </si>
-  <si>
-    <t>Sociology: 290 (Paper 1: 153, Paper 2: 137)</t>
-  </si>
-  <si>
-    <t>स्रोत में GS-wise breakup नहीं।</t>
-  </si>
-  <si>
-    <t>स्रोत में विशिष्ट अंक नहीं।</t>
-  </si>
-  <si>
-    <t>Sociology Optional: 284 अंक।</t>
-  </si>
-  <si>
-    <t>GS1: 110+, GS2: ~118, GS4: 129, Essay: 138 (2020), Sociology: 277+ | कुल GS ~435+</t>
-  </si>
-  <si>
-    <t>GS1: 107, GS2: 105, GS3: 85, GS4: 108 | Optional: 144+142 = 286</t>
   </si>
   <si>
     <t>1. दिसंबर तक Mains Ready | 2. एक विषय – एक पुस्तक, 3-4 बार रिवीजन | 3. Active Recall (किताब बंद कर याद करें) | 4. 10-15 पेज की Factbook (डेटा, समितियाँ, निर्णय) | 5. अखबार: 1-1.5 घंटे, केवल Explained Page | 6. Essay+Ethics+Optional पर 50%+ ध्यान।</t>
@@ -1662,7 +1142,8 @@
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5" style="3" customWidth="1"/>
-    <col min="2" max="20" width="19.625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="22.75" style="2" customWidth="1"/>
+    <col min="3" max="20" width="19.625" style="2" customWidth="1"/>
     <col min="21" max="16384" width="11" style="2"/>
   </cols>
   <sheetData>
@@ -1961,63 +1442,63 @@
         <v>150</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="5">
+        <v>5</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="E6" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="G6" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="H6" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="I6" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="J6" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="K6" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="M6" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="H6" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="J6" s="5" t="s">
+      <c r="N6" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="K6" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="L6" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="M6" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>164</v>
-      </c>
       <c r="O6" s="5" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="38.25" x14ac:dyDescent="0.25">
@@ -2025,10 +1506,10 @@
         <v>5</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>150</v>
@@ -2064,850 +1545,526 @@
         <v>150</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="P7" s="6" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="Q7" s="6" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="R7" s="6" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="S7" s="6" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="K8" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="L8" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="M8" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="N8" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="O8" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="P8" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="Q8" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="R8" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="S8" s="5" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>191</v>
+      <c r="B9" s="5" t="s">
+        <v>168</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>192</v>
+      <c r="C9" s="5" t="s">
+        <v>169</v>
       </c>
-      <c r="D9" s="6" t="s">
-        <v>193</v>
+      <c r="D9" s="5" t="s">
+        <v>170</v>
       </c>
-      <c r="E9" s="6" t="s">
-        <v>194</v>
+      <c r="E9" s="5" t="s">
+        <v>171</v>
       </c>
-      <c r="F9" s="6" t="s">
-        <v>195</v>
+      <c r="F9" s="5" t="s">
+        <v>172</v>
       </c>
-      <c r="G9" s="6" t="s">
-        <v>196</v>
+      <c r="G9" s="5" t="s">
+        <v>173</v>
       </c>
-      <c r="H9" s="6" t="s">
-        <v>197</v>
+      <c r="H9" s="5" t="s">
+        <v>174</v>
       </c>
-      <c r="I9" s="6" t="s">
-        <v>198</v>
+      <c r="I9" s="5" t="s">
+        <v>175</v>
       </c>
-      <c r="J9" s="6" t="s">
-        <v>199</v>
+      <c r="J9" s="5" t="s">
+        <v>176</v>
       </c>
-      <c r="K9" s="6" t="s">
-        <v>200</v>
+      <c r="K9" s="5" t="s">
+        <v>177</v>
       </c>
-      <c r="L9" s="6" t="s">
-        <v>201</v>
+      <c r="L9" s="5" t="s">
+        <v>178</v>
       </c>
-      <c r="M9" s="6" t="s">
-        <v>202</v>
+      <c r="M9" s="5" t="s">
+        <v>179</v>
       </c>
-      <c r="N9" s="6" t="s">
-        <v>203</v>
+      <c r="N9" s="5" t="s">
+        <v>180</v>
       </c>
-      <c r="O9" s="6" t="s">
-        <v>204</v>
+      <c r="O9" s="5" t="s">
+        <v>181</v>
       </c>
-      <c r="P9" s="6" t="s">
-        <v>205</v>
+      <c r="P9" s="5" t="s">
+        <v>182</v>
       </c>
-      <c r="Q9" s="6" t="s">
-        <v>206</v>
+      <c r="Q9" s="5" t="s">
+        <v>183</v>
       </c>
-      <c r="R9" s="6" t="s">
-        <v>207</v>
+      <c r="R9" s="5" t="s">
+        <v>184</v>
       </c>
-      <c r="S9" s="6" t="s">
-        <v>208</v>
+      <c r="S9" s="5" t="s">
+        <v>185</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="204" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="J10" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="K10" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="L10" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="M10" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="N10" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="O10" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="P10" s="5" t="s">
-        <v>223</v>
-      </c>
-      <c r="Q10" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="R10" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="S10" s="5" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" ht="178.5" x14ac:dyDescent="0.25">
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
+      <c r="P10" s="5"/>
+      <c r="Q10" s="5"/>
+      <c r="R10" s="5"/>
+      <c r="S10" s="5"/>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>229</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>230</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>231</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>232</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>234</v>
-      </c>
-      <c r="J11" s="6" t="s">
-        <v>235</v>
-      </c>
-      <c r="K11" s="6" t="s">
-        <v>236</v>
-      </c>
-      <c r="L11" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="M11" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="N11" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="O11" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="P11" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="Q11" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="R11" s="6" t="s">
-        <v>243</v>
-      </c>
-      <c r="S11" s="6" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="12" spans="1:19" ht="204" x14ac:dyDescent="0.25">
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
+      <c r="L11" s="6"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
+      <c r="O11" s="6"/>
+      <c r="P11" s="6"/>
+      <c r="Q11" s="6"/>
+      <c r="R11" s="6"/>
+      <c r="S11" s="6"/>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="5" t="s">
-        <v>245</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>246</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>247</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>249</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>250</v>
-      </c>
-      <c r="H12" s="5" t="s">
-        <v>251</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>252</v>
-      </c>
-      <c r="J12" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="K12" s="5" t="s">
-        <v>254</v>
-      </c>
-      <c r="L12" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="M12" s="5" t="s">
-        <v>256</v>
-      </c>
-      <c r="N12" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="O12" s="5" t="s">
-        <v>258</v>
-      </c>
-      <c r="P12" s="5" t="s">
-        <v>259</v>
-      </c>
-      <c r="Q12" s="5" t="s">
-        <v>260</v>
-      </c>
-      <c r="R12" s="5" t="s">
-        <v>261</v>
-      </c>
-      <c r="S12" s="5" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19" ht="229.5" x14ac:dyDescent="0.25">
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="5"/>
+      <c r="L12" s="5"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="5"/>
+      <c r="O12" s="5"/>
+      <c r="P12" s="5"/>
+      <c r="Q12" s="5"/>
+      <c r="R12" s="5"/>
+      <c r="S12" s="5"/>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>264</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>265</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>266</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>267</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>269</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>270</v>
-      </c>
-      <c r="J13" s="6" t="s">
-        <v>271</v>
-      </c>
-      <c r="K13" s="6" t="s">
-        <v>270</v>
-      </c>
-      <c r="L13" s="6" t="s">
-        <v>272</v>
-      </c>
-      <c r="M13" s="6" t="s">
-        <v>273</v>
-      </c>
-      <c r="N13" s="6" t="s">
-        <v>274</v>
-      </c>
-      <c r="O13" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="P13" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="Q13" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="R13" s="6" t="s">
-        <v>278</v>
-      </c>
-      <c r="S13" s="6" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19" ht="191.25" x14ac:dyDescent="0.25">
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="6"/>
+      <c r="S13" s="6"/>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>280</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>281</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>282</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>283</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>284</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>285</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>286</v>
-      </c>
-      <c r="I14" s="5" t="s">
-        <v>287</v>
-      </c>
-      <c r="J14" s="5" t="s">
-        <v>288</v>
-      </c>
-      <c r="K14" s="5" t="s">
-        <v>289</v>
-      </c>
-      <c r="L14" s="5" t="s">
-        <v>290</v>
-      </c>
-      <c r="M14" s="5" t="s">
-        <v>291</v>
-      </c>
-      <c r="N14" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="O14" s="5" t="s">
-        <v>293</v>
-      </c>
-      <c r="P14" s="5" t="s">
-        <v>294</v>
-      </c>
-      <c r="Q14" s="5" t="s">
-        <v>295</v>
-      </c>
-      <c r="R14" s="5" t="s">
-        <v>296</v>
-      </c>
-      <c r="S14" s="5" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19" ht="229.5" x14ac:dyDescent="0.25">
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
+      <c r="P14" s="5"/>
+      <c r="Q14" s="5"/>
+      <c r="R14" s="5"/>
+      <c r="S14" s="5"/>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>298</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>299</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>300</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>301</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>302</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>303</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>304</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>305</v>
-      </c>
-      <c r="J15" s="6" t="s">
-        <v>305</v>
-      </c>
-      <c r="K15" s="6" t="s">
-        <v>305</v>
-      </c>
-      <c r="L15" s="6" t="s">
-        <v>306</v>
-      </c>
-      <c r="M15" s="6" t="s">
-        <v>307</v>
-      </c>
-      <c r="N15" s="6" t="s">
-        <v>305</v>
-      </c>
-      <c r="O15" s="6" t="s">
-        <v>308</v>
-      </c>
-      <c r="P15" s="6" t="s">
-        <v>309</v>
-      </c>
-      <c r="Q15" s="6" t="s">
-        <v>310</v>
-      </c>
-      <c r="R15" s="6" t="s">
-        <v>311</v>
-      </c>
-      <c r="S15" s="6" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19" ht="165.75" x14ac:dyDescent="0.25">
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="6"/>
+      <c r="K15" s="6"/>
+      <c r="L15" s="6"/>
+      <c r="M15" s="6"/>
+      <c r="N15" s="6"/>
+      <c r="O15" s="6"/>
+      <c r="P15" s="6"/>
+      <c r="Q15" s="6"/>
+      <c r="R15" s="6"/>
+      <c r="S15" s="6"/>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>313</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>314</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>315</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>316</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>317</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>318</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>319</v>
-      </c>
-      <c r="I16" s="5" t="s">
-        <v>320</v>
-      </c>
-      <c r="J16" s="5" t="s">
-        <v>321</v>
-      </c>
-      <c r="K16" s="5" t="s">
-        <v>322</v>
-      </c>
-      <c r="L16" s="5" t="s">
-        <v>323</v>
-      </c>
-      <c r="M16" s="5" t="s">
-        <v>324</v>
-      </c>
-      <c r="N16" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="O16" s="5" t="s">
-        <v>326</v>
-      </c>
-      <c r="P16" s="5" t="s">
-        <v>327</v>
-      </c>
-      <c r="Q16" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="R16" s="5" t="s">
-        <v>329</v>
-      </c>
-      <c r="S16" s="5" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="17" spans="1:19" ht="127.5" x14ac:dyDescent="0.25">
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="5"/>
+      <c r="N16" s="5"/>
+      <c r="O16" s="5"/>
+      <c r="P16" s="5"/>
+      <c r="Q16" s="5"/>
+      <c r="R16" s="5"/>
+      <c r="S16" s="5"/>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>331</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>332</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>333</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>333</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>334</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>335</v>
-      </c>
-      <c r="H17" s="6" t="s">
-        <v>333</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>333</v>
-      </c>
-      <c r="J17" s="6" t="s">
-        <v>336</v>
-      </c>
-      <c r="K17" s="6" t="s">
-        <v>333</v>
-      </c>
-      <c r="L17" s="6" t="s">
-        <v>337</v>
-      </c>
-      <c r="M17" s="6" t="s">
-        <v>333</v>
-      </c>
-      <c r="N17" s="6" t="s">
-        <v>333</v>
-      </c>
-      <c r="O17" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="P17" s="6" t="s">
-        <v>339</v>
-      </c>
-      <c r="Q17" s="6" t="s">
-        <v>340</v>
-      </c>
-      <c r="R17" s="6" t="s">
-        <v>341</v>
-      </c>
-      <c r="S17" s="6" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="18" spans="1:19" ht="63.75" x14ac:dyDescent="0.25">
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="6"/>
+      <c r="K17" s="6"/>
+      <c r="L17" s="6"/>
+      <c r="M17" s="6"/>
+      <c r="N17" s="6"/>
+      <c r="O17" s="6"/>
+      <c r="P17" s="6"/>
+      <c r="Q17" s="6"/>
+      <c r="R17" s="6"/>
+      <c r="S17" s="6"/>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="5" t="s">
-        <v>343</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>344</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>345</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>347</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>347</v>
-      </c>
-      <c r="H18" s="5" t="s">
-        <v>348</v>
-      </c>
-      <c r="I18" s="5" t="s">
-        <v>347</v>
-      </c>
-      <c r="J18" s="5" t="s">
-        <v>347</v>
-      </c>
-      <c r="K18" s="5" t="s">
-        <v>349</v>
-      </c>
-      <c r="L18" s="5" t="s">
-        <v>350</v>
-      </c>
-      <c r="M18" s="5" t="s">
-        <v>344</v>
-      </c>
-      <c r="N18" s="5" t="s">
-        <v>351</v>
-      </c>
-      <c r="O18" s="5" t="s">
-        <v>352</v>
-      </c>
-      <c r="P18" s="5" t="s">
-        <v>347</v>
-      </c>
-      <c r="Q18" s="5" t="s">
-        <v>347</v>
-      </c>
-      <c r="R18" s="5" t="s">
-        <v>353</v>
-      </c>
-      <c r="S18" s="5" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="19" spans="1:19" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
+      <c r="N18" s="5"/>
+      <c r="O18" s="5"/>
+      <c r="P18" s="5"/>
+      <c r="Q18" s="5"/>
+      <c r="R18" s="5"/>
+      <c r="S18" s="5"/>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="6" t="s">
-        <v>355</v>
+      <c r="B19" s="6">
+        <v>175</v>
       </c>
-      <c r="C19" s="6" t="s">
-        <v>356</v>
+      <c r="C19" s="6">
+        <v>205</v>
       </c>
-      <c r="D19" s="6" t="s">
-        <v>357</v>
+      <c r="D19" s="6">
+        <v>156</v>
       </c>
-      <c r="E19" s="6" t="s">
-        <v>358</v>
+      <c r="E19" s="6">
+        <v>180</v>
       </c>
-      <c r="F19" s="6" t="s">
-        <v>359</v>
+      <c r="F19" s="6">
+        <v>198</v>
       </c>
-      <c r="G19" s="6" t="s">
-        <v>358</v>
+      <c r="G19" s="6">
+        <v>150</v>
       </c>
-      <c r="H19" s="6" t="s">
-        <v>358</v>
+      <c r="H19" s="6">
+        <v>175</v>
       </c>
-      <c r="I19" s="6" t="s">
-        <v>359</v>
+      <c r="I19" s="6">
+        <v>180</v>
       </c>
-      <c r="J19" s="6" t="s">
-        <v>359</v>
+      <c r="J19" s="6">
+        <v>165</v>
       </c>
-      <c r="K19" s="6" t="s">
-        <v>358</v>
+      <c r="K19" s="6">
+        <v>185</v>
       </c>
-      <c r="L19" s="6" t="s">
-        <v>358</v>
+      <c r="L19" s="6">
+        <v>195</v>
       </c>
-      <c r="M19" s="6" t="s">
-        <v>360</v>
+      <c r="M19" s="6">
+        <v>220</v>
       </c>
-      <c r="N19" s="6" t="s">
-        <v>358</v>
+      <c r="N19" s="6">
+        <v>200</v>
       </c>
-      <c r="O19" s="6" t="s">
-        <v>361</v>
+      <c r="O19" s="6">
+        <v>195</v>
       </c>
-      <c r="P19" s="6" t="s">
-        <v>359</v>
+      <c r="P19" s="6">
+        <v>189</v>
       </c>
-      <c r="Q19" s="6" t="s">
-        <v>359</v>
+      <c r="Q19" s="6">
+        <v>185</v>
       </c>
-      <c r="R19" s="6" t="s">
-        <v>362</v>
+      <c r="R19" s="6">
+        <v>199</v>
       </c>
-      <c r="S19" s="6" t="s">
-        <v>358</v>
+      <c r="S19" s="6">
+        <v>200</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>363</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>364</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>365</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>366</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>367</v>
-      </c>
-      <c r="G20" s="5" t="s">
-        <v>368</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>369</v>
-      </c>
-      <c r="I20" s="5" t="s">
-        <v>370</v>
-      </c>
-      <c r="J20" s="5" t="s">
-        <v>371</v>
-      </c>
-      <c r="K20" s="5" t="s">
-        <v>372</v>
-      </c>
-      <c r="L20" s="5" t="s">
-        <v>373</v>
-      </c>
-      <c r="M20" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="N20" s="5" t="s">
-        <v>375</v>
-      </c>
-      <c r="O20" s="5" t="s">
-        <v>376</v>
-      </c>
-      <c r="P20" s="5" t="s">
-        <v>377</v>
-      </c>
-      <c r="Q20" s="5" t="s">
-        <v>378</v>
-      </c>
-      <c r="R20" s="5" t="s">
-        <v>379</v>
-      </c>
-      <c r="S20" s="5" t="s">
+      <c r="B20" s="2">
         <v>380</v>
       </c>
-    </row>
-    <row r="21" spans="1:19" ht="102" x14ac:dyDescent="0.25">
+      <c r="C20" s="2">
+        <v>450</v>
+      </c>
+      <c r="D20" s="2">
+        <v>350</v>
+      </c>
+      <c r="E20" s="2">
+        <v>450</v>
+      </c>
+      <c r="F20" s="2">
+        <v>558</v>
+      </c>
+      <c r="G20" s="2">
+        <v>482</v>
+      </c>
+      <c r="H20" s="2">
+        <v>395</v>
+      </c>
+      <c r="I20" s="2">
+        <v>546</v>
+      </c>
+      <c r="J20" s="2">
+        <v>516</v>
+      </c>
+      <c r="K20" s="2">
+        <v>458</v>
+      </c>
+      <c r="L20" s="2">
+        <v>545</v>
+      </c>
+      <c r="M20" s="2">
+        <v>656</v>
+      </c>
+      <c r="N20" s="2">
+        <v>846</v>
+      </c>
+      <c r="O20" s="2">
+        <v>541</v>
+      </c>
+      <c r="P20" s="2">
+        <v>350</v>
+      </c>
+      <c r="Q20" s="2">
+        <v>356</v>
+      </c>
+      <c r="R20" s="2">
+        <v>486</v>
+      </c>
+      <c r="S20" s="2">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" ht="127.5" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>381</v>
+      <c r="B21" s="5" t="s">
+        <v>186</v>
       </c>
-      <c r="C21" s="6" t="s">
-        <v>382</v>
+      <c r="C21" s="5" t="s">
+        <v>187</v>
       </c>
-      <c r="D21" s="6" t="s">
-        <v>383</v>
+      <c r="D21" s="5" t="s">
+        <v>188</v>
       </c>
-      <c r="E21" s="6" t="s">
-        <v>384</v>
+      <c r="E21" s="5" t="s">
+        <v>189</v>
       </c>
-      <c r="F21" s="6" t="s">
-        <v>385</v>
+      <c r="F21" s="5" t="s">
+        <v>190</v>
       </c>
-      <c r="G21" s="6" t="s">
-        <v>386</v>
+      <c r="G21" s="5" t="s">
+        <v>191</v>
       </c>
-      <c r="H21" s="6" t="s">
-        <v>387</v>
+      <c r="H21" s="5" t="s">
+        <v>192</v>
       </c>
-      <c r="I21" s="6" t="s">
-        <v>388</v>
+      <c r="I21" s="5" t="s">
+        <v>193</v>
       </c>
-      <c r="J21" s="6" t="s">
-        <v>389</v>
+      <c r="J21" s="5" t="s">
+        <v>194</v>
       </c>
-      <c r="K21" s="6" t="s">
-        <v>390</v>
+      <c r="K21" s="5" t="s">
+        <v>195</v>
       </c>
-      <c r="L21" s="6" t="s">
-        <v>391</v>
+      <c r="L21" s="5" t="s">
+        <v>196</v>
       </c>
-      <c r="M21" s="6" t="s">
-        <v>392</v>
+      <c r="M21" s="5" t="s">
+        <v>197</v>
       </c>
-      <c r="N21" s="6" t="s">
-        <v>393</v>
+      <c r="N21" s="5" t="s">
+        <v>198</v>
       </c>
-      <c r="O21" s="6" t="s">
-        <v>394</v>
+      <c r="O21" s="5" t="s">
+        <v>199</v>
       </c>
-      <c r="P21" s="6" t="s">
-        <v>395</v>
+      <c r="P21" s="5" t="s">
+        <v>200</v>
       </c>
-      <c r="Q21" s="6" t="s">
-        <v>396</v>
+      <c r="Q21" s="5" t="s">
+        <v>201</v>
       </c>
-      <c r="R21" s="6" t="s">
-        <v>397</v>
+      <c r="R21" s="5" t="s">
+        <v>202</v>
       </c>
-      <c r="S21" s="6" t="s">
-        <v>398</v>
+      <c r="S21" s="5" t="s">
+        <v>203</v>
       </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19" ht="102" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>39</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="J22" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="L22" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="M22" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="N22" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="O22" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="P22" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="Q22" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="R22" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="S22" s="6" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
fix: resolve timetable overflow, remove master strategies cards
</commit_message>
<xml_diff>
--- a/Update_App_Data/upsc_toppers_data.xlsx
+++ b/Update_App_Data/upsc_toppers_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\Storage  Driver\upsc-cse-master-hub\Update_App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8079D5F0-F8D7-4064-A1FB-DEB0AA4BCC2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B34727C-679A-4E0C-972A-3D6C6A4F2B32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="229">
   <si>
     <t>id</t>
   </si>
@@ -704,6 +704,27 @@
   <si>
     <t>College 1st-2nd Year: Personality Development + Newspaper आदत | College Gaps में Library/Hostel में Standard Books पढ़ें।</t>
   </si>
+  <si>
+    <t>prelimsGsMarks</t>
+  </si>
+  <si>
+    <t>prelimsCsatMarks</t>
+  </si>
+  <si>
+    <t>gs4Marks</t>
+  </si>
+  <si>
+    <t>gs1Marks</t>
+  </si>
+  <si>
+    <t>gs3Marks</t>
+  </si>
+  <si>
+    <t>gs2Marks</t>
+  </si>
+  <si>
+    <t> essayMarks</t>
+  </si>
 </sst>
 </file>
 
@@ -1141,7 +1162,7 @@
   <dimension ref="A1:S16384"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.5" style="3" customWidth="1"/>
+    <col min="1" max="1" width="15.625" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.75" style="2" customWidth="1"/>
     <col min="3" max="20" width="19.625" style="2" customWidth="1"/>
     <col min="21" max="16384" width="11" style="2"/>
@@ -2068,25 +2089,60 @@
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A23" s="2"/>
+      <c r="A23" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B23" s="2">
+        <v>89</v>
+      </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A24" s="2"/>
+      <c r="A24" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B24" s="2">
+        <v>65</v>
+      </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A25" s="2"/>
+      <c r="A25" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B25" s="2">
+        <v>135</v>
+      </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A26" s="2"/>
+      <c r="A26" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B26" s="2">
+        <v>110</v>
+      </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A27" s="2"/>
+      <c r="A27" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B27" s="2">
+        <v>95</v>
+      </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A28" s="2"/>
+      <c r="A28" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B28" s="2">
+        <v>128</v>
+      </c>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A29" s="2"/>
+      <c r="A29" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B29" s="2">
+        <v>135</v>
+      </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>

</xml_diff>

<commit_message>
Add revised 3x, 4x, 5x status tracking for micro topics
</commit_message>
<xml_diff>
--- a/Update_App_Data/upsc_toppers_data.xlsx
+++ b/Update_App_Data/upsc_toppers_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\Storage  Driver\upsc-cse-master-hub\Update_App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B34727C-679A-4E0C-972A-3D6C6A4F2B32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C06EC70D-DD54-41C4-A2B5-D19E792CB6F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="363">
   <si>
     <t>id</t>
   </si>
@@ -725,6 +725,408 @@
   <si>
     <t> essayMarks</t>
   </si>
+  <si>
+    <t>अंक: 112 | इतिहास: TN Board Cl-11 NCERT + Spectrum/Bipin Chandra | भूगोल: Cl-11,12 NCERTs + Atlas | समाज: उत्कर्ष द्विवेदी टेम्पलेट + NCERT + NFHS/ASER डेटा | विश्व इतिहास: Vision IAS बुकलेट + PYQs।</t>
+  </si>
+  <si>
+    <t>भूगोल: Cl-11,12 NCERTs + Maps अभ्यास | इतिहास: Spectrum/PW Udaan (Modern) + पुरानी NCERTs (Ancient/Medieval) | Art &amp; Culture: NCERTs + Stick Figures (नटराज आदि) | प्रतिदिन 30 मिनट Modern History।</t>
+  </si>
+  <si>
+    <t>विभिन्न GS Papers के ज्ञान को Cross-fertilize करके उत्तर लिखे | 2-3 पेज Concise Notes प्रति विषय।</t>
+  </si>
+  <si>
+    <t>History: Modern → Spectrum (25 pages में condense) + NCERTs (R.S. Sharma, Satish Chandra, Bipan Chandra) | Society: Smriti Ma'am Notes | Comparative Charts: राष्ट्रपति vs राज्यपाल आदि।</t>
+  </si>
+  <si>
+    <t>समाचार पत्र की जगह Monthly/Yearly Magazines के Index Page पर Short Notes + बार-बार Revision।</t>
+  </si>
+  <si>
+    <t>इतिहास/भूगोल के कठिन प्रश्नों में Maps + Diagrams बनाकर अंक खींचे | PYQs (2013 के बाद) के चारों Options का गहन विश्लेषण।</t>
+  </si>
+  <si>
+    <t>PYQs से Themes → Short Notes | Core (Polity, Economy) + Science &amp; Tech + Environment पर महारत।</t>
+  </si>
+  <si>
+    <t>GS विषयों को आपस में Interlink करके पढ़ें | Condensed Notes।</t>
+  </si>
+  <si>
+    <t>NCERT + Basic Sources — FOMO से बचते हुए।</t>
+  </si>
+  <si>
+    <t>History: Spectrum | Art &amp; Culture: NCERTs।</t>
+  </si>
+  <si>
+    <t>PYQ गहन विश्लेषण पर आधारित।</t>
+  </si>
+  <si>
+    <t>50% Content + 50% Presentation | Maps, Diagrams का प्रयोग।</t>
+  </si>
+  <si>
+    <t>27 साल के PYQs से Themes + Answer Writing।</t>
+  </si>
+  <si>
+    <t>अंक: 110+ (लगातार) | इतिहास (Modern): Spectrum → Short Notes + Revision | इतिहास (Ancient/Medieval): TN Board Cl-11, Cl-12 Themes in Indian History | भूगोल: 11-12 NCERTs + PMF IAS Selective + YouTube (Dr. Shivin, Sleepy Classes) | Society: Sociology Optional का ओवरलैप + PYQ Themes + Model Answers।</t>
+  </si>
+  <si>
+    <t>Laxmikanth (Polity) + Basic History NCERTs।</t>
+  </si>
+  <si>
+    <t>Geography: NCERTs (Mandatory) | History: NCERTs (Ancient/Medieval)।</t>
+  </si>
+  <si>
+    <t>History: TN Board 11th + Old NCERTs + CC Leong | Society: Vision Notes।</t>
+  </si>
+  <si>
+    <t>Ancient/Medieval: Old NCERT/R.S. Sharma | Art &amp; Culture: 11th Fine Arts NCERT।</t>
+  </si>
+  <si>
+    <t>अंक: 125 | पॉलिटी: Laxmikanth (Margin Notes) + Abhay Kumar 500 MCQs | शासन: 2nd ARC, सुप्रीम कोर्ट निर्णय | IR: PSIR Optional नोट्स का ओवरलैप + करंट (BRICS, SCO, G20, BIMSTEC) | सामाजिक न्याय: उत्कर्ष टेम्पलेट + SHG/NABARD डेटा।</t>
+  </si>
+  <si>
+    <t>पॉलिटी: Vision IAS Foundation Notes (Amirul Hasan Sir) + Laxmikanth (Margin में नोट्स) | IR: PSIR Optional से भारी ओवरलैप | Governance: Indian Express पैसिव रीडिंग।</t>
+  </si>
+  <si>
+    <t>GS1-GS4 Cross-fertilization | 2-3 पेज नोट्स | Committee Recommendations + Articles का समावेश।</t>
+  </si>
+  <si>
+    <t>Polity: Laxmikanth + 11th NCERT (Constitution at Work) | IR: Shubhra Ranjan + ORF + Indian Express + The Hindu + Jaishankar Speeches | Governance: Committee Recommendations।</t>
+  </si>
+  <si>
+    <t>प्रत्येक GS Paper: केवल 30-35 Pages के Short Notes | Pointer Format: 10-अंक → 8-10 Points, 15-अंक → 12-13 Points।</t>
+  </si>
+  <si>
+    <t>Articles + Committee Recommendations समावेश + Pointwise | Supreme Court Judgements का उल्लेख।</t>
+  </si>
+  <si>
+    <t>Polity + Governance + IR → PYQ Theme Analysis | Prelims के तथ्य → Google Docs → Mains उत्तर।</t>
+  </si>
+  <si>
+    <t>GS1-GS4 Interlinking Strategy।</t>
+  </si>
+  <si>
+    <t>Laxmikanth + NCERT | PYQ Brainstorming + Topper Copy Matching।</t>
+  </si>
+  <si>
+    <t>Polity: 11th NCERTs (Political Theory + Constitution at Work) + Laxmikanth | IR: Current-based।</t>
+  </si>
+  <si>
+    <t>PYQ गहन विश्लेषण + Limited Sources।</t>
+  </si>
+  <si>
+    <t>Bullet Points + Committee Names + Constitutional Articles।</t>
+  </si>
+  <si>
+    <t>PYQ Theme Analysis + Daily Writing।</t>
+  </si>
+  <si>
+    <t>अंक: ~118 | Polity: Laxmikanth (Highlight + बार-बार पढ़ना) + 11th NCERT Political Theory | Governance: 2nd ARC, Mallimath Committee + Constitutional Articles + Health/Education Frameworks (ASER, TSR Subramanian) | IR: Next IAS (Deepin Sir) Notes — 5-6 बार Revision | Social Justice: PYQ Themes।</t>
+  </si>
+  <si>
+    <t>The Hindu / Indian Express + Drishti Daily News Analysis।</t>
+  </si>
+  <si>
+    <t>Polity: Laxmikanth।</t>
+  </si>
+  <si>
+    <t>Polity: Laxmikanth + Mains 365 | MEA Statements + Committee Recommendations | IR: Current।</t>
+  </si>
+  <si>
+    <t>Polity: Laxmikanth (5-6 बार Revision) | Parliament, Judiciary, FRs, DPSPs पर विशेष ध्यान | Supreme Court Cases + Articles।</t>
+  </si>
+  <si>
+    <t>अंक: 86 | अर्थव्यवस्था: Shriram IAS Notes + Budget/Eco Survey (Jayant Sir) + Shivin Sir GS3 Template | आंतरिक सुरक्षा: Shivin Sir Template + अद्यतन डेटा | आपदा: NDMA Template (Utkarsh Dwivedi) | Environment &amp; S&amp;T: Annual Mains Compilations।</t>
+  </si>
+  <si>
+    <t>Economy+Environment+Security: Vision IAS Mains 365 | Budget: 2 पेज क्रिस्प नोट्स | Eco Survey: 3 पेज | Environment Mains 365: 6 पेज | Visual Presentation: Trend Graphs, Flowcharts, Infographics।</t>
+  </si>
+  <si>
+    <t>2-3 पेज नोट्स | Prelims में एकत्र ज्ञान/तथ्य Google Docs में सहेजकर Mains में प्रयोग।</t>
+  </si>
+  <si>
+    <t>GS3: Science &amp; Tech + Environment → Mains 365 | Internal Security → Shivin Sir Notes।</t>
+  </si>
+  <si>
+    <t>30-35 पेज Short Notes | Committee Names, Data, Schemes का समावेश।</t>
+  </si>
+  <si>
+    <t>स्रोत में विशिष्ट GS3 विवरण नहीं, सीमित स्रोत + Revision।</t>
+  </si>
+  <si>
+    <t>Internal Security: Vajiram Yellow Book | Disaster Management: Google का विस्तृत उपयोग | High-ROI Small Subjects पर विशेष ध्यान।</t>
+  </si>
+  <si>
+    <t>GS1-GS4 Interlinking + Condensed Notes।</t>
+  </si>
+  <si>
+    <t>Limited Sources + PYQ Analysis।</t>
+  </si>
+  <si>
+    <t>Economy: Vivek Singh + Budget &amp; Economic Survey Summary।</t>
+  </si>
+  <si>
+    <t>PYQ गहन विश्लेषण।</t>
+  </si>
+  <si>
+    <t>Flowcharts, Maps, Diagrams से Presentation।</t>
+  </si>
+  <si>
+    <t>PYQ-based Preparation + Daily Answer Writing।</t>
+  </si>
+  <si>
+    <t>अर्थव्यवस्था: Budget + Eco Survey से Data/Graphs + Mrunal Sir Free Lectures (YouTube) | कृषि: Ministry Schemes + Dryland Farming + PYQs + Crop Map | S&amp;T: PT365/Mains365 + Blockchain/IoT/Nuclear | Disaster Management: 2013-2024 सभी PYQs Model Format में | Environment: ISFR, UNEP Reports + Current Facts।</t>
+  </si>
+  <si>
+    <t>Newspaper Reading + Basic NCERTs का एकीकरण।</t>
+  </si>
+  <si>
+    <t>Economy: बार-बार पढ़कर महारत (शुरुआत में कठिन था)।</t>
+  </si>
+  <si>
+    <t>Economy: Optional से Covered | S&amp;T: Mains 365 | Security: Notes + Maps/Diagrams।</t>
+  </si>
+  <si>
+    <t>Economy: Shankar Ganesh (150 pages) / Mrunal Notes + Budget &amp; Eco Survey।</t>
+  </si>
+  <si>
+    <t>अंक: 141 (देश में सर्वोच्च में से एक, बिना कोचिंग) | 100 कीवर्ड्स (Syllabus 25-30 + PYQs 50-60) | हर कीवर्ड: परिभाषा + Quote + सिविल सेवक उदाहरण + केस स्टडी | Prahar Magazine बुकलेट + The Better India | दार्शनिक: Aristotle, Plato, Kant, Hannah Arendt | समय: Section A → 1h15m, Case Studies → 1h45m।</t>
+  </si>
+  <si>
+    <t>पसंदीदा विषय | Case Studies: Hub &amp; Spoke Model (Stakeholders) + Pros/Cons Table | समय: Theory → 1h15m, Case Studies → शेष | किसी rigid structure के बिना व्यक्तित्व दिखाएँ।</t>
+  </si>
+  <si>
+    <t>Case Studies: सामान्य सुझावों के बजाय स्पष्ट व्यावहारिक समाधान | Essay: रोजाना एक विषय पर Brainstorming Notes।</t>
+  </si>
+  <si>
+    <t>Ethics: Ansari Sir (Lukman IAS) Notes | 'The Better India' से Real Examples | Ramayana/Mahabharata से नैतिक पाठ | Topper Copies (Shruti Ma'am, Vishakha Ma'am)।</t>
+  </si>
+  <si>
+    <t>Ethics: प्रत्येक उत्तर में कम से कम एक Indian/Western Philosopher का उल्लेख | Case Studies: 3-4 Pre-set Templates (Stakeholder Approach, Values Approach)।</t>
+  </si>
+  <si>
+    <t>Ethics: पहले 10-अंकीय प्रश्न, फिर Case Studies, अंत में Quotation-based प्रश्न हल किए।</t>
+  </si>
+  <si>
+    <t>Essay: स्वामी विवेकानंद के विचार, INA Trial, 'Tryst with Destiny' जैसे ऐतिहासिक संदर्भ।</t>
+  </si>
+  <si>
+    <t>स्रोत में विशिष्ट GS4 विवरण नहीं।</t>
+  </si>
+  <si>
+    <t>PYQ Brainstorming + Model Answer Comparison।</t>
+  </si>
+  <si>
+    <t>Mains के लिए 6-7 माह समर्पित।</t>
+  </si>
+  <si>
+    <t>Practical Solutions + Clear Framework।</t>
+  </si>
+  <si>
+    <t>Daily Writing Practice।</t>
+  </si>
+  <si>
+    <t>अंक: 129 | Section A: Ready-made Frameworks/Templates (Personal/Professional/Social, Concentric Circles) + Diverse Examples (Bhagavad Gita, IPS CAA Protest, Zomato Delivery Boy) + Sakshi Ma'am Mentorship (Vajiram) | Case Studies: Stakeholder के लिए Creative Diagrams (Forest Cutting में Tree Drawing) + Clear Option Selection + Positive Conclusion।</t>
+  </si>
+  <si>
+    <t>Case Studies अभ्यास + Daily Events से Critical Thinking।</t>
+  </si>
+  <si>
+    <t>स्रोत में विशिष्ट GS4 Strategy नहीं।</t>
+  </si>
+  <si>
+    <t>DK Balaji Sir Book | Quotes/Definitions Notes | Section A: 1.5h, Case Studies: 1.5h।</t>
+  </si>
+  <si>
+    <t>Syllabus Keywords की परिभाषाएँ + व्यावहारिक उदाहरण (2-3 Page Sheet)।</t>
+  </si>
+  <si>
+    <t>अंक: 100 | प्रति निबंध 1.5 घंटा (20-30 मिनट माइंड-मैप, 1 घंटा लेखन) | 15-16 बहु-आयामी GS आयाम | दोनों निबंधों का ढाँचा अलग | Haidt की 'The Anxious Generation' जैसे साहित्यिक संदर्भ।</t>
+  </si>
+  <si>
+    <t>अंक: 144 | 5 मिनट Timer → रफ पेज पर सभी आयाम (PESTEL) + Quotes | Anecdote/Quote से आकर्षक शुरुआत | Topper copies से Example Bank तैयार।</t>
+  </si>
+  <si>
+    <t>रोजाना एक दार्शनिक विषय पर Brainstorming Notes | Philosophical Essays में गहरी वैचारिक संरचना।</t>
+  </si>
+  <si>
+    <t>PYQs से मुख्य Themes (Problems, Causes, Solutions, Way Forward) पहचाने।</t>
+  </si>
+  <si>
+    <t>प्रत्येक GS Paper: 30-35 पेज Short Notes | PESTEL दृष्टिकोण।</t>
+  </si>
+  <si>
+    <t>PYQ Analysis + Toppers की Answer Copies से Structuring।</t>
+  </si>
+  <si>
+    <t>Essay: स्वामी विवेकानंद + INA Trial + Tryst with Destiny जैसे ऐतिहासिक संदर्भ | Multi-dimensional दृष्टिकोण।</t>
+  </si>
+  <si>
+    <t>Essay को 5Ws (How, What, Why, When, Who) में तोड़कर Structure | गणितीय दृष्टिकोण से रूपरेखा।</t>
+  </si>
+  <si>
+    <t>PYQs Brainstorming → Topper Copies से Matching।</t>
+  </si>
+  <si>
+    <t>Limited Sources + Revision।</t>
+  </si>
+  <si>
+    <t>Mains के लिए Dedicated 6-7 माह (Prelims से पहले)।</t>
+  </si>
+  <si>
+    <t>Multi-dimensional दृष्टिकोण + Diagrams।</t>
+  </si>
+  <si>
+    <t>Daily Answer Writing + PYQ Simulation।</t>
+  </si>
+  <si>
+    <t>अंक: 138 (2020 में) | Organic &amp; Simple लेखन (रटे-रटाए Formula से बचना) | Structure: Main Theme → पक्ष → 2 Para विपक्ष → Futuristic Conclusion | Framework 1: Individual→Family→Society→Nation→World | Framework 2: Ancient→Medieval→Modern→AI Age | बाहरी Feedback (माता-पिता, Prof.) लेना।</t>
+  </si>
+  <si>
+    <t>Quotes की जगह Real Stories/Case Studies से शुरुआत | 15-16 निबंध लिखे | Multi-dimensional दृष्टिकोण।</t>
+  </si>
+  <si>
+    <t>Prelims के बाद 6-7 Tests (कुल 12-14 निबंध) लिखे।</t>
+  </si>
+  <si>
+    <t>Multi-dimensional दृष्टिकोण | Quotes + Examples।</t>
+  </si>
+  <si>
+    <t>PESTLE Dimensions से Essay Link | 10-15 मिनट Brainstorming + Outline | Anecdote/Quotes से शुरुआत | Way Forward पर Positive Conclusion।</t>
+  </si>
+  <si>
+    <t>PSIR 280 अंक (2023: 230 → 2024: 280) | IGNOU सामग्री + Shriram/Vajiram नोट्स | सितंबर तक Syllabus + PYQs पूरे | 40% दैनिक समय | विचारक + खंडन एकसाथ | IR Paper 2B में करंट इंटीग्रेट।</t>
+  </si>
+  <si>
+    <t>PSIR | PYQs: 2013-2023 Topic-Wise | हर Topic: 2-4 Thinkers (पक्ष+विपक्ष) | तकनीकी शब्दावली | GS2 IR से भारी ओवरलैप।</t>
+  </si>
+  <si>
+    <t>Sociology 290 अंक | 4 मुख्य Register + 4 छोटे Handouts (अंतिम समय हेतु) | Durkheim के सिद्धांत → वर्तमान उदाहरण से जोड़ना | Thinkers को Current Affairs से Link।</t>
+  </si>
+  <si>
+    <t>PSIR: Shubhra Ranjan 80% Base | ORF, Indian Express, The Hindu, Jaishankar Interviews से Value Addition।</t>
+  </si>
+  <si>
+    <t>Economics: Paper 2 को GS3 Indian Economy से Integrate किया | Arjun Gupta Sir के Topper Notes।</t>
+  </si>
+  <si>
+    <t>PSIR: O.P. Gauba, Andrew Heywood (Global Politics) | 20 व 15 अंक वाले प्रश्नों को प्राथमिकता।</t>
+  </si>
+  <si>
+    <t>Political Science/Sociology | PYQ-based तैयारी।</t>
+  </si>
+  <si>
+    <t>स्रोत में विशिष्ट Optional Strategy नहीं।</t>
+  </si>
+  <si>
+    <t>Anthropology (Public Administration से Switch) | 1 साल का Break लेकर Mains को मज़बूत किया।</t>
+  </si>
+  <si>
+    <t>Sociology: 284 अंक | Thinkers → Current Examples से Link।</t>
+  </si>
+  <si>
+    <t>Sociology: 277 अंक (2020) | B.Tech Background पर GS/Essay/Ethics Overlap | Sources: NCERT 11-12 + IGNOU BA | Value Addition: Tusharanshu Sir + Nitin Sangwan (Essential Sociology) + Ritzer (Selective) + LevelUp IAS + Shankar IAS Test Series | Integrated Notes (Paper 1+2 समान Topics) | Humanities Prof. शैली में Paragraph Format + 1-3 Thinkers प्रति उत्तर।</t>
+  </si>
+  <si>
+    <t>Sociology: उपलब्धता + रुचि के आधार पर चयन।</t>
+  </si>
+  <si>
+    <t>Sociology/Maths: Notes बनाना + PYQs पर विशेष जोर।</t>
+  </si>
+  <si>
+    <t>Economics: 144+142 = 286 अंक | H.L. Ahuja, Salvatore, Jhingan | Economic Survey + Budget।</t>
+  </si>
+  <si>
+    <t>Optional चयन के 4 पैमाने: Background/Interest + Syllabus Vastness + Competition Level + Guidance Availability।</t>
+  </si>
+  <si>
+    <t>अंक: 82 (Cutoff: 75) | नया पैटर्न + Shock Absorption माइंडसेट | PYQ थीम एनालिसिस (Art. 19, 21, 32 जैसे हाई-फ्रीक्वेंसी) | Jan-Feb: रिवीजन 1, Mar-15Apr: रिवीजन 2 | 3-इटरेशन पेपर सॉल्विंग | सबसे मज़बूत विषय (Polity) से शुरू।</t>
+  </si>
+  <si>
+    <t>2024 में 98 प्रश्न अटेम्प्ट | Vajiram Power Up Test Series (CA) + Vision IAS Abhyas Tests | Calculated Risk: 30-35 sure-shot + 50-50 elimination | अंतिम 27 दिन: कोई नया रिसोर्स नहीं, केवल नोट्स + PYQs।</t>
+  </si>
+  <si>
+    <t>फरवरी से प्रतिदिन 50 MCQs + सप्ताह में 2-3 Mock Tests | परीक्षा से 1 महीना पहले Mock बंद → केवल PYQs | The Hindu + Monthly Magazines (3-4 बार Revision) | CA के अलग नोट्स नहीं।</t>
+  </si>
+  <si>
+    <t>4th Attempt: 90+ प्रश्न हल किए (पहले 3 में 71-78 से Fail) | Source List: Polity-Laxmikanth+11NCERT, History-Spectrum, Economy-Vivek Singh, Environment-Shankar+PT365, Geography-Rishikesh Notes+11/12 NCERT | Comparative Tables।</t>
+  </si>
+  <si>
+    <t>जनवरी से ऑफलाइन Mock Tests + कमज़ोर विषयों का विश्लेषण | Monthly/Yearly Magazine Index पर Notes | CSAT: केवल PYQs।</t>
+  </si>
+  <si>
+    <t>फरवरी से Sectional Tests → FLTs | 2013 के बाद के PYQs के चारों विकल्पों का विश्लेषण।</t>
+  </si>
+  <si>
+    <t>PYQs से Themes निकालकर Short Notes | Core + Sci&amp;Tech + Environment में बढ़त (Bouncer प्रश्नों में लाभ)।</t>
+  </si>
+  <si>
+    <t>Risk Management: 90-95 प्रश्न हल करने का लक्ष्य | 30 प्रश्न गलत के Margin के बाद भी 100+ Net Positive।</t>
+  </si>
+  <si>
+    <t>FOMO से बचाव — केवल NCERT + Laxmikanth तक सीमित | CSAT: बिना नागा रोजाना अभ्यास + PYQs।</t>
+  </si>
+  <si>
+    <t>2013 के बाद के PYQs को दैनिक 25 प्रश्नों के Mock की तरह हल किया | Polity: 11th NCERTs + Laxmikanth | Economy: Vivek Singh + Budget | History: Spectrum।</t>
+  </si>
+  <si>
+    <t>4th Attempt: बिना Coaching Mock के, केवल पिछले 10 वर्षों (2014 से) के PYQs का गहन विश्लेषण।</t>
+  </si>
+  <si>
+    <t>2023 के कठिन पेपर में घबराए नहीं | 65 मज़बूत प्रश्न पहले चुने → 88 प्रश्न हल किए।</t>
+  </si>
+  <si>
+    <t>27 साल के PYQs की Theme-wise Compilation | 99 प्रश्न Attempt।</t>
+  </si>
+  <si>
+    <t>Less is More — 3 बार Revision | केवल 15+ Full Length Tests (Vision, Forum, Vajiram) | PYQs (2013 से): सभी Options का गहन विश्लेषण + Notes में समाहित | 2021: 100 प्रश्न → &lt;1 अंक से Fail → Calculated Risk (80-95 प्रश्न) | Current Affairs: PT365 + Newspaper 30 मिनट (Ethics/Essay Examples)।</t>
+  </si>
+  <si>
+    <t>1991 से PYQs Solve | अंतिम 2 माह: Daily Mock Tests | घर पर Exam जैसा माहौल।</t>
+  </si>
+  <si>
+    <t>Daily Current Affairs Notes | Prelims से 1.5 माह पहले रोज़ एक Mock Test।</t>
+  </si>
+  <si>
+    <t>35 Mock Tests (गहन Revision) | 5-Page Fact Sheets (प्रति Subject) | 3 Rounds में Paper Solve।</t>
+  </si>
+  <si>
+    <t>1st Attempt Prelims Fail → 6 माह केवल Prelims Focus | एक विषय 10 दिन → Test (Vision/Insights) → 2 दिन Revision → अगला विषय।</t>
+  </si>
+  <si>
+    <t>अंक: 75 | PCB बैकग्राउंड, 10वीं के बाद Maths नहीं | RC: 25-28 प्रश्न (उच्च सटीकता) | Reasoning: 10-15 प्रश्न | Quant: Time-Work, SDT, Percentage, Number System | कुल 45-50 प्रश्न टार्गेट।</t>
+  </si>
+  <si>
+    <t>2nd Attempt में CSAT fail → 3rd में विशेष ध्यान | NDA, CDS, CPSC के पिछले 3 साल के CSAT Papers | RC: प्रश्न पहले पढ़ें → Extreme Options तुरंत खारिज | 27-28 RC में से 22+ सही टार्गेट।</t>
+  </si>
+  <si>
+    <t>स्रोत में विशिष्ट उल्लेख नहीं।</t>
+  </si>
+  <si>
+    <t>Comprehension के लिए केवल UPSC PYQs को मुख्य आधार।</t>
+  </si>
+  <si>
+    <t>CSAT: गणितीय कमज़ोरी पहचानकर Number System, Average, Calendar जैसे High-Yield Topics के लिए Crash Course + अभ्यास।</t>
+  </si>
+  <si>
+    <t>बिना नागा रोजाना प्रश्न अभ्यास | Comprehension के लिए केवल PYQs।</t>
+  </si>
+  <si>
+    <t>R.S. Aggarwal पुस्तक + नियमित अभ्यास।</t>
+  </si>
+  <si>
+    <t>पिछले 5 साल के PYQs → 2 घंटे Time-bound | Formula Sheet (1 Page): Mathematical Formulas, Tricks, Reasoning Rules → GS1-GS2 Break में Revise | 53 Maths/Reasoning में से 27-28 Easy + Comprehension ध्यान से।</t>
+  </si>
+  <si>
+    <t>रोजाना 15-20 मिनट Logical Reasoning + Quant अभ्यास।</t>
+  </si>
+  <si>
+    <t>Mental Ability + Maths पर भरोसा + पुराने Papers Solve।</t>
+  </si>
+  <si>
+    <t>English में Comfortable (30 प्रश्न) | Maths/Reasoning में Selective।</t>
+  </si>
+  <si>
+    <t>Logical Elimination + 50-50 वाले प्रश्नों में Net Positive Strategy।</t>
+  </si>
 </sst>
 </file>
 
@@ -750,7 +1152,7 @@
       <sz val="10"/>
       <color rgb="FF1C2833"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1668,189 +2070,477 @@
       <c r="R10" s="5"/>
       <c r="S10" s="5"/>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" ht="204" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="6"/>
-      <c r="P11" s="6"/>
-      <c r="Q11" s="6"/>
-      <c r="R11" s="6"/>
-      <c r="S11" s="6"/>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B11" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="L11" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="M11" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="N11" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="O11" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="P11" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="Q11" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="R11" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="S11" s="5" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" ht="178.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-      <c r="O12" s="5"/>
-      <c r="P12" s="5"/>
-      <c r="Q12" s="5"/>
-      <c r="R12" s="5"/>
-      <c r="S12" s="5"/>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B12" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="L12" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="M12" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="N12" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="O12" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="P12" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="Q12" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="R12" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="S12" s="6" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" ht="204" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
-      <c r="N13" s="6"/>
-      <c r="O13" s="6"/>
-      <c r="P13" s="6"/>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="6"/>
-      <c r="S13" s="6"/>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B13" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="L13" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="M13" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="N13" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="O13" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="P13" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="Q13" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="R13" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="S13" s="5" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" ht="229.5" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-      <c r="O14" s="5"/>
-      <c r="P14" s="5"/>
-      <c r="Q14" s="5"/>
-      <c r="R14" s="5"/>
-      <c r="S14" s="5"/>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B14" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="L14" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="M14" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="N14" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="O14" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="P14" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="Q14" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="R14" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="S14" s="6" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" ht="191.25" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="6"/>
-      <c r="M15" s="6"/>
-      <c r="N15" s="6"/>
-      <c r="O15" s="6"/>
-      <c r="P15" s="6"/>
-      <c r="Q15" s="6"/>
-      <c r="R15" s="6"/>
-      <c r="S15" s="6"/>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B15" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="L15" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="M15" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="N15" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="O15" s="5" t="s">
+        <v>313</v>
+      </c>
+      <c r="P15" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="Q15" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="R15" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="S15" s="5" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" ht="229.5" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
-      <c r="N16" s="5"/>
-      <c r="O16" s="5"/>
-      <c r="P16" s="5"/>
-      <c r="Q16" s="5"/>
-      <c r="R16" s="5"/>
-      <c r="S16" s="5"/>
-    </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B16" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="M16" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="N16" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="O16" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="P16" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="Q16" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="R16" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="S16" s="6" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" ht="165.75" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="6"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="6"/>
-      <c r="M17" s="6"/>
-      <c r="N17" s="6"/>
-      <c r="O17" s="6"/>
-      <c r="P17" s="6"/>
-      <c r="Q17" s="6"/>
-      <c r="R17" s="6"/>
-      <c r="S17" s="6"/>
-    </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B17" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>335</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>337</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="L17" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="M17" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="N17" s="5" t="s">
+        <v>345</v>
+      </c>
+      <c r="O17" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="P17" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="Q17" s="5" t="s">
+        <v>348</v>
+      </c>
+      <c r="R17" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="S17" s="5" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" ht="127.5" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
-      <c r="N18" s="5"/>
-      <c r="O18" s="5"/>
-      <c r="P18" s="5"/>
-      <c r="Q18" s="5"/>
-      <c r="R18" s="5"/>
-      <c r="S18" s="5"/>
+      <c r="B18" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="M18" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="N18" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="O18" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="P18" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="Q18" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="R18" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="S18" s="6" t="s">
+        <v>362</v>
+      </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">

</xml_diff>

<commit_message>
Enhance Mock Test forms, UI, and clear Quick Revision dummy data
</commit_message>
<xml_diff>
--- a/Update_App_Data/upsc_toppers_data.xlsx
+++ b/Update_App_Data/upsc_toppers_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\Storage  Driver\upsc-cse-master-hub\Update_App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C06EC70D-DD54-41C4-A2B5-D19E792CB6F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6283E969-5410-4693-922E-2B4D9840F6C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Strategy" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="383">
   <si>
     <t>id</t>
   </si>
@@ -145,9 +145,6 @@
   </si>
   <si>
     <t>Why did you leave Goldman Sachs for Civil Services?</t>
-  </si>
-  <si>
-    <t>While corporate life offered financial growth, I wanted to work on larger societal impact...</t>
   </si>
   <si>
     <t>DAF / Work Experience</t>
@@ -1127,6 +1124,69 @@
   <si>
     <t>Logical Elimination + 50-50 वाले प्रश्नों में Net Positive Strategy।</t>
   </si>
+  <si>
+    <t>SELF SEI</t>
+  </si>
+  <si>
+    <t>interview-2</t>
+  </si>
+  <si>
+    <t>RAJ</t>
+  </si>
+  <si>
+    <t>KM</t>
+  </si>
+  <si>
+    <t>KUCH BHI</t>
+  </si>
+  <si>
+    <t>APNE AP</t>
+  </si>
+  <si>
+    <t>KYA AAP BHI KU C LDF</t>
+  </si>
+  <si>
+    <t>Sudfj</t>
+  </si>
+  <si>
+    <t>Kumar B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shi hai </t>
+  </si>
+  <si>
+    <t xml:space="preserve">kya </t>
+  </si>
+  <si>
+    <t>sbhi shi hai</t>
+  </si>
+  <si>
+    <t>raj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kumar </t>
+  </si>
+  <si>
+    <t>pub add 1</t>
+  </si>
+  <si>
+    <t>history</t>
+  </si>
+  <si>
+    <t>cast</t>
+  </si>
+  <si>
+    <t>polity</t>
+  </si>
+  <si>
+    <t>mlkx</t>
+  </si>
+  <si>
+    <t>gutu</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
 </sst>
 </file>
 
@@ -1575,117 +1635,117 @@
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C1" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="Q1" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="R1" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="S1" s="5" t="s">
         <v>118</v>
-      </c>
-      <c r="S1" s="5" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="G2" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="H2" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="I2" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="J2" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="K2" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="L2" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="M2" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="N2" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="O2" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="P2" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="Q2" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="Q2" s="5" t="s">
+      <c r="R2" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="R2" s="5" t="s">
+      <c r="S2" s="5" t="s">
         <v>118</v>
-      </c>
-      <c r="S2" s="5" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
@@ -1693,58 +1753,58 @@
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="H3" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="I3" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="J3" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="K3" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="L3" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="K3" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="L3" s="6" t="s">
+      <c r="M3" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="M3" s="6" t="s">
+      <c r="N3" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="N3" s="6" t="s">
+      <c r="O3" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="O3" s="6" t="s">
+      <c r="P3" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="P3" s="6" t="s">
+      <c r="Q3" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="Q3" s="6" t="s">
+      <c r="R3" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="R3" s="6" t="s">
+      <c r="S3" s="6" t="s">
         <v>135</v>
-      </c>
-      <c r="S3" s="6" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
@@ -1752,58 +1812,58 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="F4" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="G4" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="F4" s="5" t="s">
+      <c r="H4" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="I4" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="G4" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="I4" s="5" t="s">
+      <c r="J4" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="K4" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="L4" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="K4" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="L4" s="5" t="s">
+      <c r="M4" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="N4" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="M4" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="N4" s="5" t="s">
+      <c r="O4" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="P4" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="O4" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="P4" s="5" t="s">
-        <v>144</v>
-      </c>
       <c r="Q4" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:19" ht="25.5" x14ac:dyDescent="0.25">
@@ -1811,58 +1871,58 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="E5" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="H5" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="G5" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="H5" s="6" t="s">
+      <c r="I5" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="J5" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="L5" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="J5" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="L5" s="6" t="s">
+      <c r="M5" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="M5" s="6" t="s">
+      <c r="N5" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="O5" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="N5" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="O5" s="6" t="s">
+      <c r="P5" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="Q5" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="P5" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="Q5" s="6" t="s">
+      <c r="R5" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="R5" s="6" t="s">
-        <v>155</v>
-      </c>
       <c r="S5" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
@@ -1873,55 +1933,55 @@
         <v>5</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="J6" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="K6" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="L6" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="S6" s="5" t="s">
         <v>156</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="L6" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="M6" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="O6" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="P6" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="Q6" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="R6" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="S6" s="5" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="38.25" x14ac:dyDescent="0.25">
@@ -1929,58 +1989,58 @@
         <v>5</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="D7" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="M7" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="N7" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="O7" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="D7" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="K7" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="L7" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="M7" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="N7" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="O7" s="6" t="s">
+      <c r="P7" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="P7" s="6" t="s">
+      <c r="Q7" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="Q7" s="6" t="s">
+      <c r="R7" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="R7" s="6" t="s">
-        <v>167</v>
-      </c>
       <c r="S7" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
@@ -1993,58 +2053,58 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="D9" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="E9" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="F9" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="G9" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="H9" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="I9" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="J9" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="K9" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="K9" s="5" t="s">
+      <c r="L9" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="L9" s="5" t="s">
+      <c r="M9" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="M9" s="5" t="s">
+      <c r="N9" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="N9" s="5" t="s">
+      <c r="O9" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="O9" s="5" t="s">
+      <c r="P9" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="P9" s="5" t="s">
+      <c r="Q9" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="Q9" s="5" t="s">
+      <c r="R9" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="R9" s="5" t="s">
+      <c r="S9" s="5" t="s">
         <v>184</v>
-      </c>
-      <c r="S9" s="5" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
@@ -2075,58 +2135,58 @@
         <v>9</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="F11" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="G11" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="H11" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="I11" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="J11" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="J11" s="5" t="s">
+      <c r="K11" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="K11" s="5" t="s">
+      <c r="L11" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="L11" s="5" t="s">
+      <c r="M11" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="M11" s="5" t="s">
+      <c r="N11" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="N11" s="5" t="s">
+      <c r="O11" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="O11" s="5" t="s">
+      <c r="P11" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="P11" s="5" t="s">
+      <c r="Q11" s="5" t="s">
         <v>243</v>
       </c>
-      <c r="Q11" s="5" t="s">
+      <c r="R11" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="R11" s="5" t="s">
+      <c r="S11" s="5" t="s">
         <v>245</v>
-      </c>
-      <c r="S11" s="5" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="12" spans="1:19" ht="178.5" x14ac:dyDescent="0.25">
@@ -2134,58 +2194,58 @@
         <v>10</v>
       </c>
       <c r="B12" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="D12" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="E12" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="F12" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="G12" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="H12" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="I12" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="I12" s="6" t="s">
+      <c r="J12" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="J12" s="6" t="s">
+      <c r="K12" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="K12" s="6" t="s">
+      <c r="L12" s="6" t="s">
         <v>256</v>
       </c>
-      <c r="L12" s="6" t="s">
+      <c r="M12" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="M12" s="6" t="s">
+      <c r="N12" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="N12" s="6" t="s">
+      <c r="O12" s="6" t="s">
         <v>259</v>
       </c>
-      <c r="O12" s="6" t="s">
+      <c r="P12" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="P12" s="6" t="s">
+      <c r="Q12" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="Q12" s="6" t="s">
+      <c r="R12" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="R12" s="6" t="s">
+      <c r="S12" s="6" t="s">
         <v>263</v>
-      </c>
-      <c r="S12" s="6" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="13" spans="1:19" ht="204" x14ac:dyDescent="0.25">
@@ -2193,58 +2253,58 @@
         <v>11</v>
       </c>
       <c r="B13" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>267</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="F13" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="G13" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="H13" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="I13" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="J13" s="5" t="s">
         <v>272</v>
       </c>
-      <c r="J13" s="5" t="s">
+      <c r="K13" s="5" t="s">
         <v>273</v>
       </c>
-      <c r="K13" s="5" t="s">
+      <c r="L13" s="5" t="s">
         <v>274</v>
       </c>
-      <c r="L13" s="5" t="s">
+      <c r="M13" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="M13" s="5" t="s">
+      <c r="N13" s="5" t="s">
         <v>276</v>
       </c>
-      <c r="N13" s="5" t="s">
+      <c r="O13" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="O13" s="5" t="s">
+      <c r="P13" s="5" t="s">
         <v>278</v>
       </c>
-      <c r="P13" s="5" t="s">
+      <c r="Q13" s="5" t="s">
         <v>279</v>
       </c>
-      <c r="Q13" s="5" t="s">
+      <c r="R13" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="R13" s="5" t="s">
+      <c r="S13" s="5" t="s">
         <v>281</v>
-      </c>
-      <c r="S13" s="5" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="229.5" x14ac:dyDescent="0.25">
@@ -2252,58 +2312,58 @@
         <v>12</v>
       </c>
       <c r="B14" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="C14" s="6" t="s">
         <v>283</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="D14" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="E14" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="F14" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="G14" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="H14" s="6" t="s">
         <v>288</v>
       </c>
-      <c r="H14" s="6" t="s">
+      <c r="I14" s="6" t="s">
         <v>289</v>
       </c>
-      <c r="I14" s="6" t="s">
+      <c r="J14" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="J14" s="6" t="s">
+      <c r="K14" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="L14" s="6" t="s">
         <v>291</v>
       </c>
-      <c r="K14" s="6" t="s">
-        <v>290</v>
-      </c>
-      <c r="L14" s="6" t="s">
+      <c r="M14" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="M14" s="6" t="s">
+      <c r="N14" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="N14" s="6" t="s">
+      <c r="O14" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="O14" s="6" t="s">
+      <c r="P14" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="P14" s="6" t="s">
+      <c r="Q14" s="6" t="s">
         <v>296</v>
       </c>
-      <c r="Q14" s="6" t="s">
+      <c r="R14" s="6" t="s">
         <v>297</v>
       </c>
-      <c r="R14" s="6" t="s">
+      <c r="S14" s="6" t="s">
         <v>298</v>
-      </c>
-      <c r="S14" s="6" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="15" spans="1:19" ht="191.25" x14ac:dyDescent="0.25">
@@ -2311,58 +2371,58 @@
         <v>13</v>
       </c>
       <c r="B15" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>301</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="E15" s="5" t="s">
         <v>302</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="F15" s="5" t="s">
         <v>303</v>
       </c>
-      <c r="F15" s="5" t="s">
+      <c r="G15" s="5" t="s">
         <v>304</v>
       </c>
-      <c r="G15" s="5" t="s">
+      <c r="H15" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="H15" s="5" t="s">
+      <c r="I15" s="5" t="s">
         <v>306</v>
       </c>
-      <c r="I15" s="5" t="s">
+      <c r="J15" s="5" t="s">
         <v>307</v>
       </c>
-      <c r="J15" s="5" t="s">
+      <c r="K15" s="5" t="s">
         <v>308</v>
       </c>
-      <c r="K15" s="5" t="s">
+      <c r="L15" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="L15" s="5" t="s">
+      <c r="M15" s="5" t="s">
         <v>310</v>
       </c>
-      <c r="M15" s="5" t="s">
+      <c r="N15" s="5" t="s">
         <v>311</v>
       </c>
-      <c r="N15" s="5" t="s">
+      <c r="O15" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="O15" s="5" t="s">
+      <c r="P15" s="5" t="s">
         <v>313</v>
       </c>
-      <c r="P15" s="5" t="s">
+      <c r="Q15" s="5" t="s">
         <v>314</v>
       </c>
-      <c r="Q15" s="5" t="s">
+      <c r="R15" s="5" t="s">
         <v>315</v>
       </c>
-      <c r="R15" s="5" t="s">
+      <c r="S15" s="5" t="s">
         <v>316</v>
-      </c>
-      <c r="S15" s="5" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="16" spans="1:19" ht="229.5" x14ac:dyDescent="0.25">
@@ -2370,58 +2430,58 @@
         <v>14</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>318</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="D16" s="6" t="s">
         <v>319</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="E16" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>321</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="G16" s="6" t="s">
         <v>322</v>
       </c>
-      <c r="G16" s="6" t="s">
+      <c r="H16" s="6" t="s">
         <v>323</v>
       </c>
-      <c r="H16" s="6" t="s">
+      <c r="I16" s="6" t="s">
         <v>324</v>
       </c>
-      <c r="I16" s="6" t="s">
+      <c r="J16" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="L16" s="6" t="s">
         <v>325</v>
       </c>
-      <c r="J16" s="6" t="s">
-        <v>325</v>
-      </c>
-      <c r="K16" s="6" t="s">
-        <v>325</v>
-      </c>
-      <c r="L16" s="6" t="s">
+      <c r="M16" s="6" t="s">
         <v>326</v>
       </c>
-      <c r="M16" s="6" t="s">
+      <c r="N16" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="O16" s="6" t="s">
         <v>327</v>
       </c>
-      <c r="N16" s="6" t="s">
-        <v>325</v>
-      </c>
-      <c r="O16" s="6" t="s">
+      <c r="P16" s="6" t="s">
         <v>328</v>
       </c>
-      <c r="P16" s="6" t="s">
+      <c r="Q16" s="6" t="s">
         <v>329</v>
       </c>
-      <c r="Q16" s="6" t="s">
+      <c r="R16" s="6" t="s">
         <v>330</v>
       </c>
-      <c r="R16" s="6" t="s">
+      <c r="S16" s="6" t="s">
         <v>331</v>
-      </c>
-      <c r="S16" s="6" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="17" spans="1:19" ht="165.75" x14ac:dyDescent="0.25">
@@ -2429,58 +2489,58 @@
         <v>15</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>333</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="D17" s="5" t="s">
         <v>334</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="E17" s="5" t="s">
         <v>335</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="F17" s="5" t="s">
         <v>336</v>
       </c>
-      <c r="F17" s="5" t="s">
+      <c r="G17" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="G17" s="5" t="s">
+      <c r="H17" s="5" t="s">
         <v>338</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="I17" s="5" t="s">
         <v>339</v>
       </c>
-      <c r="I17" s="5" t="s">
+      <c r="J17" s="5" t="s">
         <v>340</v>
       </c>
-      <c r="J17" s="5" t="s">
+      <c r="K17" s="5" t="s">
         <v>341</v>
       </c>
-      <c r="K17" s="5" t="s">
+      <c r="L17" s="5" t="s">
         <v>342</v>
       </c>
-      <c r="L17" s="5" t="s">
+      <c r="M17" s="5" t="s">
         <v>343</v>
       </c>
-      <c r="M17" s="5" t="s">
+      <c r="N17" s="5" t="s">
         <v>344</v>
       </c>
-      <c r="N17" s="5" t="s">
+      <c r="O17" s="5" t="s">
         <v>345</v>
       </c>
-      <c r="O17" s="5" t="s">
+      <c r="P17" s="5" t="s">
         <v>346</v>
       </c>
-      <c r="P17" s="5" t="s">
+      <c r="Q17" s="5" t="s">
         <v>347</v>
       </c>
-      <c r="Q17" s="5" t="s">
+      <c r="R17" s="5" t="s">
         <v>348</v>
       </c>
-      <c r="R17" s="5" t="s">
+      <c r="S17" s="5" t="s">
         <v>349</v>
-      </c>
-      <c r="S17" s="5" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="127.5" x14ac:dyDescent="0.25">
@@ -2488,58 +2548,58 @@
         <v>16</v>
       </c>
       <c r="B18" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>351</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="D18" s="6" t="s">
         <v>352</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="E18" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="F18" s="6" t="s">
         <v>353</v>
       </c>
-      <c r="E18" s="6" t="s">
-        <v>353</v>
-      </c>
-      <c r="F18" s="6" t="s">
+      <c r="G18" s="6" t="s">
         <v>354</v>
       </c>
-      <c r="G18" s="6" t="s">
+      <c r="H18" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="J18" s="6" t="s">
         <v>355</v>
       </c>
-      <c r="H18" s="6" t="s">
-        <v>353</v>
-      </c>
-      <c r="I18" s="6" t="s">
-        <v>353</v>
-      </c>
-      <c r="J18" s="6" t="s">
+      <c r="K18" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="L18" s="6" t="s">
         <v>356</v>
       </c>
-      <c r="K18" s="6" t="s">
-        <v>353</v>
-      </c>
-      <c r="L18" s="6" t="s">
+      <c r="M18" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="N18" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="O18" s="6" t="s">
         <v>357</v>
       </c>
-      <c r="M18" s="6" t="s">
-        <v>353</v>
-      </c>
-      <c r="N18" s="6" t="s">
-        <v>353</v>
-      </c>
-      <c r="O18" s="6" t="s">
+      <c r="P18" s="6" t="s">
         <v>358</v>
       </c>
-      <c r="P18" s="6" t="s">
+      <c r="Q18" s="6" t="s">
         <v>359</v>
       </c>
-      <c r="Q18" s="6" t="s">
+      <c r="R18" s="6" t="s">
         <v>360</v>
       </c>
-      <c r="R18" s="6" t="s">
+      <c r="S18" s="6" t="s">
         <v>361</v>
-      </c>
-      <c r="S18" s="6" t="s">
-        <v>362</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
@@ -2665,122 +2725,122 @@
         <v>19</v>
       </c>
       <c r="B21" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="E21" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="F21" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="F21" s="5" t="s">
+      <c r="G21" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="G21" s="5" t="s">
+      <c r="H21" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="H21" s="5" t="s">
+      <c r="I21" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="I21" s="5" t="s">
+      <c r="J21" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="J21" s="5" t="s">
+      <c r="K21" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="K21" s="5" t="s">
+      <c r="L21" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="L21" s="5" t="s">
+      <c r="M21" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="M21" s="5" t="s">
+      <c r="N21" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="N21" s="5" t="s">
+      <c r="O21" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="O21" s="5" t="s">
+      <c r="P21" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="P21" s="5" t="s">
+      <c r="Q21" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="Q21" s="5" t="s">
+      <c r="R21" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="R21" s="5" t="s">
+      <c r="S21" s="5" t="s">
         <v>202</v>
-      </c>
-      <c r="S21" s="5" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="22" spans="1:19" ht="102" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B22" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="C22" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="D22" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="E22" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="F22" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="G22" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="G22" s="6" t="s">
+      <c r="H22" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="H22" s="6" t="s">
+      <c r="I22" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="I22" s="6" t="s">
+      <c r="J22" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="J22" s="6" t="s">
+      <c r="K22" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="K22" s="6" t="s">
+      <c r="L22" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="L22" s="6" t="s">
+      <c r="M22" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="M22" s="6" t="s">
+      <c r="N22" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="N22" s="6" t="s">
+      <c r="O22" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="O22" s="6" t="s">
+      <c r="P22" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="P22" s="6" t="s">
+      <c r="Q22" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="Q22" s="6" t="s">
+      <c r="R22" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="R22" s="6" t="s">
+      <c r="S22" s="6" t="s">
         <v>220</v>
-      </c>
-      <c r="S22" s="6" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B23" s="2">
         <v>89</v>
@@ -2788,7 +2848,7 @@
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B24" s="2">
         <v>65</v>
@@ -2796,7 +2856,7 @@
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B25" s="2">
         <v>135</v>
@@ -2804,7 +2864,7 @@
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B26" s="2">
         <v>110</v>
@@ -2812,7 +2872,7 @@
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B27" s="2">
         <v>95</v>
@@ -2820,7 +2880,7 @@
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B28" s="2">
         <v>128</v>
@@ -2828,7 +2888,7 @@
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B29" s="2">
         <v>135</v>
@@ -51907,13 +51967,45 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>376</v>
+      </c>
+      <c r="B1" t="s">
+        <v>376</v>
+      </c>
+      <c r="C1" t="s">
+        <v>377</v>
+      </c>
+      <c r="D1" t="s">
+        <v>378</v>
+      </c>
+      <c r="E1" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>374</v>
+      </c>
+      <c r="B2" t="s">
+        <v>375</v>
+      </c>
+      <c r="C2" t="s">
+        <v>382</v>
+      </c>
+      <c r="D2" t="s">
+        <v>381</v>
+      </c>
+      <c r="E2" t="s">
+        <v>380</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -51953,342 +52045,342 @@
     </row>
     <row r="2" spans="1:6" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>41</v>
-      </c>
       <c r="D2" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>41</v>
-      </c>
       <c r="D3" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>41</v>
-      </c>
       <c r="D5" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>77</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="D10" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="D12" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>101</v>
-      </c>
       <c r="C18" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -52308,7 +52400,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" style="1" bestFit="1" customWidth="1"/>
@@ -52366,16 +52458,68 @@
         <v>35</v>
       </c>
       <c r="G2" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>37</v>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="D3" s="1">
+        <v>2025</v>
+      </c>
+      <c r="E3" s="1">
+        <v>320</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="D4" s="1">
+        <v>1546</v>
+      </c>
+      <c r="E4" s="1">
+        <v>352</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>373</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:H2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:H1 A2:F2 H2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix TypeScript spread errors and missing modal usages
</commit_message>
<xml_diff>
--- a/Update_App_Data/upsc_toppers_data.xlsx
+++ b/Update_App_Data/upsc_toppers_data.xlsx
@@ -8,18 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\Storage  Driver\upsc-cse-master-hub\Update_App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6283E969-5410-4693-922E-2B4D9840F6C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{332ABBC6-E225-41FF-BFD9-627456E5F1C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Strategy" sheetId="1" r:id="rId1"/>
-    <sheet name="Books" sheetId="2" r:id="rId2"/>
-    <sheet name="Routines" sheetId="3" r:id="rId3"/>
-    <sheet name="Interviews" sheetId="4" r:id="rId4"/>
+    <sheet name="Routines" sheetId="3" r:id="rId2"/>
+    <sheet name="Interviews" sheetId="4" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Routines!$A$1:$F$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Routines!$A$1:$F$17</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="374">
   <si>
     <t>id</t>
   </si>
@@ -1160,33 +1159,6 @@
   <si>
     <t>sbhi shi hai</t>
   </si>
-  <si>
-    <t>raj</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kumar </t>
-  </si>
-  <si>
-    <t>pub add 1</t>
-  </si>
-  <si>
-    <t>history</t>
-  </si>
-  <si>
-    <t>cast</t>
-  </si>
-  <si>
-    <t>polity</t>
-  </si>
-  <si>
-    <t>mlkx</t>
-  </si>
-  <si>
-    <t>gutu</t>
-  </si>
-  <si>
-    <t>notes</t>
-  </si>
 </sst>
 </file>
 
@@ -51966,50 +51938,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>376</v>
-      </c>
-      <c r="B1" t="s">
-        <v>376</v>
-      </c>
-      <c r="C1" t="s">
-        <v>377</v>
-      </c>
-      <c r="D1" t="s">
-        <v>378</v>
-      </c>
-      <c r="E1" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>374</v>
-      </c>
-      <c r="B2" t="s">
-        <v>375</v>
-      </c>
-      <c r="C2" t="s">
-        <v>382</v>
-      </c>
-      <c r="D2" t="s">
-        <v>381</v>
-      </c>
-      <c r="E2" t="s">
-        <v>380</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:F18"/>
@@ -52398,7 +52326,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
feat: implement hierarchical dropdowns, dynamic weak areas, timer linking, and rename papers to subjects
</commit_message>
<xml_diff>
--- a/Update_App_Data/upsc_toppers_data.xlsx
+++ b/Update_App_Data/upsc_toppers_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\Storage  Driver\upsc-cse-master-hub\Update_App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{332ABBC6-E225-41FF-BFD9-627456E5F1C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F375E39-F60E-4036-8D1A-BFBDC6B41B52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Strategy" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Interviews" sheetId="4" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Routines!$A$1:$F$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Routines!$A$1:$F$19</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="375">
   <si>
     <t>id</t>
   </si>
@@ -1159,6 +1159,9 @@
   <si>
     <t>sbhi shi hai</t>
   </si>
+  <si>
+    <t>01:30 AM - 02:00 AM</t>
+  </si>
 </sst>
 </file>
 
@@ -51940,13 +51943,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.875" customWidth="1"/>
     <col min="5" max="5" width="50.125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.5" customWidth="1"/>
   </cols>
@@ -51971,7 +51974,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>85</v>
       </c>
@@ -51991,7 +51994,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>85</v>
       </c>
@@ -52011,7 +52014,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>85</v>
       </c>
@@ -52031,7 +52034,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>85</v>
       </c>
@@ -52291,7 +52294,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>99</v>
       </c>
@@ -52311,11 +52314,52 @@
         <v>56</v>
       </c>
     </row>
+    <row r="19" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F17" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <autoFilter ref="A1:F19" xr:uid="{00000000-0001-0000-0200-000000000000}">
     <filterColumn colId="1">
       <filters>
         <filter val="Sadaf Choudhary / Naomi Satam"/>
+        <filter val="Shruti Modi"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
feat: move MindmapsGallery to Toppers > Mindmaps & Notes section
</commit_message>
<xml_diff>
--- a/Update_App_Data/upsc_toppers_data.xlsx
+++ b/Update_App_Data/upsc_toppers_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\Storage  Driver\upsc-cse-master-hub\Update_App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F375E39-F60E-4036-8D1A-BFBDC6B41B52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F79A657-46E9-4AB9-88F4-1F839B911BAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="461">
   <si>
     <t>id</t>
   </si>
@@ -1162,12 +1162,350 @@
   <si>
     <t>01:30 AM - 02:00 AM</t>
   </si>
+  <si>
+    <t>Warda Khan</t>
+  </si>
+  <si>
+    <t>Full-Time Model -  Warda Khan</t>
+  </si>
+  <si>
+    <t>09:30 AM - 11:30 AM</t>
+  </si>
+  <si>
+    <t>मैं एक समय पर दो विषय पढ़ा करती थी। जैसे कि, मान लीजिए अगर किसी महीने मैंने पढ़ने के लिए चुना—मान लीजिए पॉलिटी (राजव्यवस्था) और इकॉनमी (अर्थव्यवस्था)</t>
+  </si>
+  <si>
+    <t>Morning Slot 1</t>
+  </si>
+  <si>
+    <t>02:00 PM - 04:10 PM</t>
+  </si>
+  <si>
+    <t>2 घंटे CSAT की भी प्रैक्टिस करती, हालाँकि वह दिसंबर के बाद से शुरू हुआ था।</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Afternoon Session </t>
+  </si>
+  <si>
+    <t>05:30 PM - 08:00 PM</t>
+  </si>
+  <si>
+    <t>दोपहर/शाम की शिफ्ट में मैं दूसरा विषय पढ़ती थी, और रात में डिनर के बाद मैं अपना ऑप्शनल (वैकल्पिक विषय) पढ़ा करती थी।"</t>
+  </si>
+  <si>
+    <t>Natasha Goyal</t>
+  </si>
+  <si>
+    <t>Full-Time Model -  Natasha Goyal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2nd -Attempt </t>
+  </si>
+  <si>
+    <t>6:30 से 7:00 बजे के आसपास मैं उठती हूँ</t>
+  </si>
+  <si>
+    <t>06:30 AM - 07:00 AM</t>
+  </si>
+  <si>
+    <t>----</t>
+  </si>
+  <si>
+    <t>मैं देखती हूँ कि आज क्या-क्या करना है। अगर SFG टेस्ट है, तो उसका क्या टारगेट है; अगर मेन्स की तैयारी करनी है, तो उसका क्या टारगेट है।</t>
+  </si>
+  <si>
+    <t>लगभग 8:00 बजे से लेकर 3:30 बजे तक</t>
+  </si>
+  <si>
+    <t>मैं लगातार एक ही बार में पढ़ाई करती थी।</t>
+  </si>
+  <si>
+    <t xml:space="preserve">फिर 3:30 बजे </t>
+  </si>
+  <si>
+    <t>मैं खाना खाती थी, उसके बाद लगभग 1 घंटे का ब्रेक होता था।</t>
+  </si>
+  <si>
+    <t>उसके बाद लगभग 7:30 बजे</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> मैं छत या बालकनी में टहलने चली जाती थी।</t>
+  </si>
+  <si>
+    <t>फिर करीब 4:30 बजे</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> दोबारा पढ़ाई के लिए बैठती थी।</t>
+  </si>
+  <si>
+    <t xml:space="preserve">फिर 8:30 से लगभग 10:30 बजे तक का </t>
+  </si>
+  <si>
+    <t>आखिरी स्लॉट होता था। बस यही मेरा रूटीन था।"</t>
+  </si>
+  <si>
+    <t>Ziniya Arora</t>
+  </si>
+  <si>
+    <t>"4 बजे मैंने उठना शुरू किया था।</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 बजे तक आपने स्लॉट लगा लिया।उसके बाद आप 7 से 8 एक टेस्ट होता था मेरा  </t>
+  </si>
+  <si>
+    <t>फिर वापस 9 बजे बैठे। फिर आप 9 से 12 लगातार पढ़ाई करें...</t>
+  </si>
+  <si>
+    <t>09:00 PM - 12:00 AM</t>
+  </si>
+  <si>
+    <t>07:00 PM - 08:00 PM</t>
+  </si>
+  <si>
+    <t>सुबह 6:00 बजे उठने में, और 6:00 बजे उठने के बाद रिवाइज़ भी करना होता था</t>
+  </si>
+  <si>
+    <t>गीतिका अरोड़ा</t>
+  </si>
+  <si>
+    <t>फिर यहाँ पे आती थी क्योंकि सीट्स भी भर जाती हैं स्टार्टिंग फ़ेज़ में, तो around 6:30 I used to leave from my PG.</t>
+  </si>
+  <si>
+    <t>I used to revise one more time. उसके बाद मैं टेस्ट देती थी 8:00 बजे तक।</t>
+  </si>
+  <si>
+    <t>leave my bank at 5:00 and by 5:30 I used to sit in my library chair.</t>
+  </si>
+  <si>
+    <t>SHTURI MODI</t>
+  </si>
+  <si>
+    <t>MODI SHRUTI</t>
+  </si>
+  <si>
+    <t>05:00 PM - 05:40 PM</t>
+  </si>
+  <si>
+    <t>8 hours, 9 hours, 10 hours, बट कंटेंट इधर-उधर का पढ़ते रहते हैं। stick to the basic notes. I used ChatGPT too much कि कहाँ से एग्ज़ांपल्स मिलें, फ़ैक्ट्स मिलें, डेटा मिले। I think right... आंसर राइटिंग बहुत इंपॉर्टेंट है।"</t>
+  </si>
+  <si>
+    <t>08:00 PM - 12:30 AM</t>
+  </si>
+  <si>
+    <t>अपना स्टडी पैटर्न</t>
+  </si>
+  <si>
+    <t>"हेलो एवरीवन।</t>
+  </si>
+  <si>
+    <t>आप हर रोज़ पढ़ाई करो और जो एवरेज है वो 7 टू 8 आवर्स रहे।</t>
+  </si>
+  <si>
+    <t>देन थर्सडे, फ्राइडे को थोड़ा कम हो जाता था, 7 टू 8 हो जाता था। सैटरडे, संडे जनरली 5 टू 6 आवर्स रहता था।</t>
+  </si>
+  <si>
+    <t>सो फॉर एग्जांपल, जैसे मैं अपना स्टडी पैटर्न—जो मैंने अपने डायरी में लिख के खुद से समझा भी है—दैट इज़ कि मैं जैसे शुरू करती थी वीक को, तो मंडे को, क्योंकि फुल्ली रिचार्ज रहते थे, वीक शुरू होता था, तो मंडे, ट्यूसडे, वेडनसडे जनरली 9 टू 10 आवर्स, ईवन 11 तक भी चला जाता था पढ़ाई।</t>
+  </si>
+  <si>
+    <t>तो इसके बाद जब मैं वीक का एवरेज देखती थी, तो वो 7 टू 8 आवर्स या फिर 8 टू 9 आवर्स जो है, इसके अप्रोक्स रहता था।</t>
+  </si>
+  <si>
+    <t>06:30 AM – 07:30 AM</t>
+  </si>
+  <si>
+    <t>मॉर्निंग रूटीन</t>
+  </si>
+  <si>
+    <t>फ्रेश होना, हल्का व्यायाम या ध्यान</t>
+  </si>
+  <si>
+    <t>07:30 AM – 09:30 AM</t>
+  </si>
+  <si>
+    <r>
+      <t>स्लॉट 1: करंट अफेयर्स</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (2 घंटे)</t>
+    </r>
+  </si>
+  <si>
+    <t>दैनिक समाचार पत्र (द हिंदू/इंडियन एक्सप्रेस) और समसामयिकी नोट्स</t>
+  </si>
+  <si>
+    <t>09:30 AM – 10:30 AM</t>
+  </si>
+  <si>
+    <t>ब्रेकफास्ट ब्रेक</t>
+  </si>
+  <si>
+    <t>नाश्ता और आराम</t>
+  </si>
+  <si>
+    <t>10:30 AM – 01:30 PM</t>
+  </si>
+  <si>
+    <r>
+      <t>स्लॉट 2: सामान्य अध्ययन (GS)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (3 घंटे)</t>
+    </r>
+  </si>
+  <si>
+    <t>कोर जीएस विषय (पॉलिटी, हिस्ट्री, इकॉनमी, या ज्योग्राफी)</t>
+  </si>
+  <si>
+    <t>01:30 PM – 03:00 PM</t>
+  </si>
+  <si>
+    <t>लंच &amp; पावर नैप</t>
+  </si>
+  <si>
+    <t>दोपहर का भोजन और विश्राम</t>
+  </si>
+  <si>
+    <t>03:00 PM – 06:00 PM</t>
+  </si>
+  <si>
+    <r>
+      <t>स्लॉट 3: ऑप्शनल सब्जेक्ट</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (3 घंटे)</t>
+    </r>
+  </si>
+  <si>
+    <t>वैकल्पिक विषय का गहन अध्ययन और नोट्स रिवीज़न</t>
+  </si>
+  <si>
+    <t>06:00 PM – 07:00 PM</t>
+  </si>
+  <si>
+    <t>इवनिंग ब्रेक</t>
+  </si>
+  <si>
+    <t>चाय, वॉक या हल्का समय</t>
+  </si>
+  <si>
+    <t>07:00 PM – 08:00 PM</t>
+  </si>
+  <si>
+    <t>जीएस / ऑप्शनल रिवीज़न (1 घंटा)</t>
+  </si>
+  <si>
+    <t>दिनभर पढ़े गए टॉपिक्स का क्विक रीकॉल</t>
+  </si>
+  <si>
+    <t>08:00 PM – 09:00 PM</t>
+  </si>
+  <si>
+    <t>डिनर ब्रेक</t>
+  </si>
+  <si>
+    <t>रात का खाना</t>
+  </si>
+  <si>
+    <t>09:00 PM – 11:00 PM</t>
+  </si>
+  <si>
+    <r>
+      <t>स्लॉट 4: टेस्ट प्रैक्टिस &amp; एक्टिव रीकॉल</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (2 घंटे)</t>
+    </r>
+  </si>
+  <si>
+    <t>10 CA MCQs, 25 स्टैटिक MCQs, 1-2 मेन्स प्रश्नों की ब्रेनस्टॉर्मिंग</t>
+  </si>
+  <si>
+    <t>11:00 PM – 06:30 AM</t>
+  </si>
+  <si>
+    <t>नींद</t>
+  </si>
+  <si>
+    <t>7.5 घंटे की पूरी नींद</t>
+  </si>
+  <si>
+    <r>
+      <t>नाईट स्लॉट (9–11 PM) नॉन-नेगोशिएबल:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> दिन में चाहे किसी विषय का मन न लगे, लेकिन रात के 2 घंटे MCQs और ब्रेनस्टॉर्मिंग को बिना नागा पूरा करें ताकि दिमाग में एक्टिव रिट्रीवल की आदत बनी रहे।</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>एक्टिव रीकॉल पर ज़ोर:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> केवल किताबें खुली रखकर पढ़ने के बजाय पन्ने पलटकर आँखें बंद करके पॉइंट्स को खुद से दोहराएँ।</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>फ्लेक्सिबिलिटी:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> जिस विषय में स्कोर कम हो (जैसे ऑप्शनल), स्लॉट 2 और स्लॉट 3 के समय को अपनी आवश्यकतानुसार आपस में अदल-बदल सकते हैं।</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">3rd  </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1186,6 +1524,19 @@
     <font>
       <sz val="10"/>
       <color rgb="FF1C2833"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -1210,7 +1561,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1233,11 +1584,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC4C7C5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFC4C7C5"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1256,6 +1622,18 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -51943,15 +52321,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.875" customWidth="1"/>
-    <col min="5" max="5" width="50.125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.5" customWidth="1"/>
+    <col min="4" max="4" width="34.625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="50.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.875" style="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -51964,13 +52342,13 @@
       <c r="C1" t="s">
         <v>23</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="9" t="s">
         <v>26</v>
       </c>
     </row>
@@ -52352,6 +52730,606 @@
       </c>
       <c r="F20" s="1" t="s">
         <v>92</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="B21" t="s">
+        <v>375</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="B22" t="s">
+        <v>375</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="B23" t="s">
+        <v>375</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="B24" t="s">
+        <v>385</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="B25" t="s">
+        <v>385</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>390</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="B26" t="s">
+        <v>385</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="B27" t="s">
+        <v>385</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="B28" t="s">
+        <v>385</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="B29" t="s">
+        <v>385</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="B30" t="s">
+        <v>385</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A34" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A36" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="B37" t="s">
+        <v>413</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="63" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="B38" t="s">
+        <v>413</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>419</v>
+      </c>
+      <c r="B39" t="s">
+        <v>418</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>422</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>419</v>
+      </c>
+      <c r="B40" t="s">
+        <v>418</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>419</v>
+      </c>
+      <c r="B41" t="s">
+        <v>418</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>423</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B42" t="s">
+        <v>102</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D42" s="11" t="s">
+        <v>424</v>
+      </c>
+      <c r="E42" s="12" t="s">
+        <v>425</v>
+      </c>
+      <c r="F42" s="12" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B43" t="s">
+        <v>102</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D43" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="E43" s="11" t="s">
+        <v>428</v>
+      </c>
+      <c r="F43" s="12" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B44" t="s">
+        <v>102</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D44" s="11" t="s">
+        <v>430</v>
+      </c>
+      <c r="E44" s="12" t="s">
+        <v>431</v>
+      </c>
+      <c r="F44" s="12" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B45" t="s">
+        <v>102</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D45" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="E45" s="11" t="s">
+        <v>434</v>
+      </c>
+      <c r="F45" s="12" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B46" t="s">
+        <v>102</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D46" s="11" t="s">
+        <v>436</v>
+      </c>
+      <c r="E46" s="12" t="s">
+        <v>437</v>
+      </c>
+      <c r="F46" s="12" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B47" t="s">
+        <v>102</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D47" s="11" t="s">
+        <v>439</v>
+      </c>
+      <c r="E47" s="11" t="s">
+        <v>440</v>
+      </c>
+      <c r="F47" s="12" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B48" t="s">
+        <v>102</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D48" s="11" t="s">
+        <v>442</v>
+      </c>
+      <c r="E48" s="12" t="s">
+        <v>443</v>
+      </c>
+      <c r="F48" s="12" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B49" t="s">
+        <v>102</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D49" s="11" t="s">
+        <v>445</v>
+      </c>
+      <c r="E49" s="12" t="s">
+        <v>446</v>
+      </c>
+      <c r="F49" s="12" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B50" t="s">
+        <v>102</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D50" s="11" t="s">
+        <v>448</v>
+      </c>
+      <c r="E50" s="12" t="s">
+        <v>449</v>
+      </c>
+      <c r="F50" s="12" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B51" t="s">
+        <v>102</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D51" s="11" t="s">
+        <v>451</v>
+      </c>
+      <c r="E51" s="11" t="s">
+        <v>452</v>
+      </c>
+      <c r="F51" s="12" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B52" t="s">
+        <v>102</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D52" s="11" t="s">
+        <v>454</v>
+      </c>
+      <c r="E52" s="12" t="s">
+        <v>455</v>
+      </c>
+      <c r="F52" s="12" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="63" x14ac:dyDescent="0.25">
+      <c r="A53" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B53" t="s">
+        <v>102</v>
+      </c>
+      <c r="C53" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D53" s="10" t="s">
+        <v>457</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>458</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>459</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-calculate routine stats on save and remove manual inputs
</commit_message>
<xml_diff>
--- a/Update_App_Data/upsc_toppers_data.xlsx
+++ b/Update_App_Data/upsc_toppers_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\Storage  Driver\upsc-cse-master-hub\Update_App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F79A657-46E9-4AB9-88F4-1F839B911BAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3146911-EFC1-47FD-8AB4-F3ABA6D61DFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="459">
   <si>
     <t>id</t>
   </si>
@@ -1187,9 +1187,6 @@
     <t xml:space="preserve">Afternoon Session </t>
   </si>
   <si>
-    <t>05:30 PM - 08:00 PM</t>
-  </si>
-  <si>
     <t>दोपहर/शाम की शिफ्ट में मैं दूसरा विषय पढ़ती थी, और रात में डिनर के बाद मैं अपना ऑप्शनल (वैकल्पिक विषय) पढ़ा करती थी।"</t>
   </si>
   <si>
@@ -1214,31 +1211,13 @@
     <t>मैं देखती हूँ कि आज क्या-क्या करना है। अगर SFG टेस्ट है, तो उसका क्या टारगेट है; अगर मेन्स की तैयारी करनी है, तो उसका क्या टारगेट है।</t>
   </si>
   <si>
-    <t>लगभग 8:00 बजे से लेकर 3:30 बजे तक</t>
-  </si>
-  <si>
-    <t>मैं लगातार एक ही बार में पढ़ाई करती थी।</t>
-  </si>
-  <si>
-    <t xml:space="preserve">फिर 3:30 बजे </t>
-  </si>
-  <si>
     <t>मैं खाना खाती थी, उसके बाद लगभग 1 घंटे का ब्रेक होता था।</t>
-  </si>
-  <si>
-    <t>उसके बाद लगभग 7:30 बजे</t>
   </si>
   <si>
     <t xml:space="preserve"> मैं छत या बालकनी में टहलने चली जाती थी।</t>
   </si>
   <si>
-    <t>फिर करीब 4:30 बजे</t>
-  </si>
-  <si>
     <t xml:space="preserve"> दोबारा पढ़ाई के लिए बैठती थी।</t>
-  </si>
-  <si>
-    <t xml:space="preserve">फिर 8:30 से लगभग 10:30 बजे तक का </t>
   </si>
   <si>
     <t>आखिरी स्लॉट होता था। बस यही मेरा रूटीन था।"</t>
@@ -1254,12 +1233,6 @@
   </si>
   <si>
     <t>फिर वापस 9 बजे बैठे। फिर आप 9 से 12 लगातार पढ़ाई करें...</t>
-  </si>
-  <si>
-    <t>09:00 PM - 12:00 AM</t>
-  </si>
-  <si>
-    <t>07:00 PM - 08:00 PM</t>
   </si>
   <si>
     <t>सुबह 6:00 बजे उठने में, और 6:00 बजे उठने के बाद रिवाइज़ भी करना होता था</t>
@@ -1299,15 +1272,6 @@
   </si>
   <si>
     <t>आप हर रोज़ पढ़ाई करो और जो एवरेज है वो 7 टू 8 आवर्स रहे।</t>
-  </si>
-  <si>
-    <t>देन थर्सडे, फ्राइडे को थोड़ा कम हो जाता था, 7 टू 8 हो जाता था। सैटरडे, संडे जनरली 5 टू 6 आवर्स रहता था।</t>
-  </si>
-  <si>
-    <t>सो फॉर एग्जांपल, जैसे मैं अपना स्टडी पैटर्न—जो मैंने अपने डायरी में लिख के खुद से समझा भी है—दैट इज़ कि मैं जैसे शुरू करती थी वीक को, तो मंडे को, क्योंकि फुल्ली रिचार्ज रहते थे, वीक शुरू होता था, तो मंडे, ट्यूसडे, वेडनसडे जनरली 9 टू 10 आवर्स, ईवन 11 तक भी चला जाता था पढ़ाई।</t>
-  </si>
-  <si>
-    <t>तो इसके बाद जब मैं वीक का एवरेज देखती थी, तो वो 7 टू 8 आवर्स या फिर 8 टू 9 आवर्स जो है, इसके अप्रोक्स रहता था।</t>
   </si>
   <si>
     <t>06:30 AM – 07:30 AM</t>
@@ -1454,21 +1418,6 @@
   </si>
   <si>
     <r>
-      <t>नाईट स्लॉट (9–11 PM) नॉन-नेगोशिएबल:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> दिन में चाहे किसी विषय का मन न लगे, लेकिन रात के 2 घंटे MCQs और ब्रेनस्टॉर्मिंग को बिना नागा पूरा करें ताकि दिमाग में एक्टिव रिट्रीवल की आदत बनी रहे।</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>एक्टिव रीकॉल पर ज़ोर:</t>
     </r>
     <r>
@@ -1499,6 +1448,39 @@
   </si>
   <si>
     <t xml:space="preserve">3rd  </t>
+  </si>
+  <si>
+    <t>01:30 PM - 03:00 PM</t>
+  </si>
+  <si>
+    <t>04:30 PM - 07:00 PM</t>
+  </si>
+  <si>
+    <t>07:30 PM - 08:00 PM</t>
+  </si>
+  <si>
+    <t>09:00 PM - 11:00 PM</t>
+  </si>
+  <si>
+    <t>04:00 AM - 4:30 AM</t>
+  </si>
+  <si>
+    <t>07:00 AM - 08:00 AM</t>
+  </si>
+  <si>
+    <t>09:00 AM - 12:00 PM</t>
+  </si>
+  <si>
+    <t>12:20 PM - 01:30 PM</t>
+  </si>
+  <si>
+    <t>06:00 AM - 06:30 AM</t>
+  </si>
+  <si>
+    <t>08:00 AM - 09:0 AM</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
 </sst>
 </file>
@@ -1603,7 +1585,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1627,8 +1609,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -52329,7 +52309,7 @@
     <col min="3" max="3" width="12.75" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="34.625" style="1" customWidth="1"/>
     <col min="5" max="5" width="50.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="40.875" style="9" customWidth="1"/>
+    <col min="6" max="6" width="40.875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -52348,7 +52328,7 @@
       <c r="E1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -52783,10 +52763,10 @@
         <v>96</v>
       </c>
       <c r="D23" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>383</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>384</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>60</v>
@@ -52794,36 +52774,36 @@
     </row>
     <row r="24" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="B24" t="s">
+        <v>384</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="B24" t="s">
-        <v>385</v>
-      </c>
-      <c r="C24" s="1" t="s">
+      <c r="D24" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="E24" s="1" t="s">
         <v>387</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>389</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="B25" t="s">
+        <v>384</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="B25" t="s">
-        <v>385</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>387</v>
-      </c>
       <c r="D25" s="7" t="s">
+        <v>389</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>390</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>391</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>379</v>
@@ -52831,265 +52811,274 @@
     </row>
     <row r="26" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="B26" t="s">
+        <v>384</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="B26" t="s">
-        <v>385</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>387</v>
-      </c>
       <c r="D26" s="1" t="s">
-        <v>392</v>
+        <v>448</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="B27" t="s">
+        <v>384</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="B27" t="s">
-        <v>385</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>387</v>
-      </c>
       <c r="D27" s="1" t="s">
-        <v>394</v>
+        <v>449</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="B28" t="s">
+        <v>384</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="B28" t="s">
-        <v>385</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>387</v>
-      </c>
       <c r="D28" s="1" t="s">
-        <v>398</v>
+        <v>450</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>399</v>
+        <v>392</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="B29" t="s">
+        <v>384</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="B29" t="s">
-        <v>385</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>387</v>
-      </c>
       <c r="D29" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="E30" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="E29" s="1" t="s">
+    </row>
+    <row r="31" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="E31" s="1" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="s">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="B30" t="s">
-        <v>385</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>387</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>400</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
-        <v>402</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>402</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>387</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>394</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A32" s="4" t="s">
-        <v>402</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>402</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>387</v>
-      </c>
       <c r="D32" s="1" t="s">
-        <v>407</v>
+        <v>454</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
-        <v>402</v>
+        <v>395</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>402</v>
+        <v>395</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>406</v>
+        <v>455</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>387</v>
+        <v>386</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>456</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>408</v>
+        <v>399</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>387</v>
+        <v>386</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>388</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>410</v>
+        <v>401</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>387</v>
+        <v>386</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>457</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>411</v>
+        <v>402</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>414</v>
+        <v>405</v>
       </c>
       <c r="B37" t="s">
-        <v>413</v>
+        <v>404</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>415</v>
+        <v>406</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>412</v>
+        <v>403</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="63" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>414</v>
+        <v>405</v>
       </c>
       <c r="B38" t="s">
-        <v>413</v>
+        <v>404</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>417</v>
+        <v>408</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>416</v>
+        <v>407</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>419</v>
+        <v>410</v>
       </c>
       <c r="B39" t="s">
-        <v>418</v>
+        <v>409</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>460</v>
-      </c>
-      <c r="D39" s="9" t="s">
-        <v>422</v>
+        <v>447</v>
+      </c>
+      <c r="D39" t="s">
+        <v>458</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>420</v>
+        <v>411</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>419</v>
+        <v>410</v>
       </c>
       <c r="B40" t="s">
-        <v>418</v>
+        <v>409</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>460</v>
-      </c>
-      <c r="D40" s="9" t="s">
-        <v>421</v>
+        <v>447</v>
+      </c>
+      <c r="D40" t="s">
+        <v>458</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>420</v>
+        <v>411</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>419</v>
+        <v>410</v>
       </c>
       <c r="B41" t="s">
-        <v>418</v>
+        <v>409</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>460</v>
-      </c>
-      <c r="D41" s="9" t="s">
-        <v>423</v>
+        <v>447</v>
+      </c>
+      <c r="D41" t="s">
+        <v>458</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>420</v>
+        <v>411</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -53102,14 +53091,14 @@
       <c r="C42" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="D42" s="11" t="s">
-        <v>424</v>
-      </c>
-      <c r="E42" s="12" t="s">
-        <v>425</v>
-      </c>
-      <c r="F42" s="12" t="s">
-        <v>426</v>
+      <c r="D42" s="9" t="s">
+        <v>412</v>
+      </c>
+      <c r="E42" s="10" t="s">
+        <v>413</v>
+      </c>
+      <c r="F42" s="10" t="s">
+        <v>414</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -53122,14 +53111,14 @@
       <c r="C43" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="D43" s="11" t="s">
-        <v>427</v>
-      </c>
-      <c r="E43" s="11" t="s">
-        <v>428</v>
-      </c>
-      <c r="F43" s="12" t="s">
-        <v>429</v>
+      <c r="D43" s="9" t="s">
+        <v>415</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>416</v>
+      </c>
+      <c r="F43" s="10" t="s">
+        <v>417</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -53142,14 +53131,14 @@
       <c r="C44" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="D44" s="11" t="s">
-        <v>430</v>
-      </c>
-      <c r="E44" s="12" t="s">
-        <v>431</v>
-      </c>
-      <c r="F44" s="12" t="s">
-        <v>432</v>
+      <c r="D44" s="9" t="s">
+        <v>418</v>
+      </c>
+      <c r="E44" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="F44" s="10" t="s">
+        <v>420</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -53162,14 +53151,14 @@
       <c r="C45" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="D45" s="11" t="s">
-        <v>433</v>
-      </c>
-      <c r="E45" s="11" t="s">
-        <v>434</v>
-      </c>
-      <c r="F45" s="12" t="s">
-        <v>435</v>
+      <c r="D45" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>422</v>
+      </c>
+      <c r="F45" s="10" t="s">
+        <v>423</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -53182,14 +53171,14 @@
       <c r="C46" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="D46" s="11" t="s">
-        <v>436</v>
-      </c>
-      <c r="E46" s="12" t="s">
-        <v>437</v>
-      </c>
-      <c r="F46" s="12" t="s">
-        <v>438</v>
+      <c r="D46" s="9" t="s">
+        <v>424</v>
+      </c>
+      <c r="E46" s="10" t="s">
+        <v>425</v>
+      </c>
+      <c r="F46" s="10" t="s">
+        <v>426</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -53202,14 +53191,14 @@
       <c r="C47" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="D47" s="11" t="s">
-        <v>439</v>
-      </c>
-      <c r="E47" s="11" t="s">
-        <v>440</v>
-      </c>
-      <c r="F47" s="12" t="s">
-        <v>441</v>
+      <c r="D47" s="9" t="s">
+        <v>427</v>
+      </c>
+      <c r="E47" s="9" t="s">
+        <v>428</v>
+      </c>
+      <c r="F47" s="10" t="s">
+        <v>429</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -53222,14 +53211,14 @@
       <c r="C48" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="D48" s="11" t="s">
-        <v>442</v>
-      </c>
-      <c r="E48" s="12" t="s">
-        <v>443</v>
-      </c>
-      <c r="F48" s="12" t="s">
-        <v>444</v>
+      <c r="D48" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="E48" s="10" t="s">
+        <v>431</v>
+      </c>
+      <c r="F48" s="10" t="s">
+        <v>432</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -53242,14 +53231,14 @@
       <c r="C49" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="D49" s="11" t="s">
-        <v>445</v>
-      </c>
-      <c r="E49" s="12" t="s">
-        <v>446</v>
-      </c>
-      <c r="F49" s="12" t="s">
-        <v>447</v>
+      <c r="D49" s="9" t="s">
+        <v>433</v>
+      </c>
+      <c r="E49" s="10" t="s">
+        <v>434</v>
+      </c>
+      <c r="F49" s="10" t="s">
+        <v>435</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -53262,14 +53251,14 @@
       <c r="C50" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="D50" s="11" t="s">
-        <v>448</v>
-      </c>
-      <c r="E50" s="12" t="s">
-        <v>449</v>
-      </c>
-      <c r="F50" s="12" t="s">
-        <v>450</v>
+      <c r="D50" s="9" t="s">
+        <v>436</v>
+      </c>
+      <c r="E50" s="10" t="s">
+        <v>437</v>
+      </c>
+      <c r="F50" s="10" t="s">
+        <v>438</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -53282,14 +53271,14 @@
       <c r="C51" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="D51" s="11" t="s">
-        <v>451</v>
-      </c>
-      <c r="E51" s="11" t="s">
-        <v>452</v>
-      </c>
-      <c r="F51" s="12" t="s">
-        <v>453</v>
+      <c r="D51" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="E51" s="9" t="s">
+        <v>440</v>
+      </c>
+      <c r="F51" s="10" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -53302,17 +53291,17 @@
       <c r="C52" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="D52" s="11" t="s">
-        <v>454</v>
-      </c>
-      <c r="E52" s="12" t="s">
-        <v>455</v>
-      </c>
-      <c r="F52" s="12" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" ht="63" x14ac:dyDescent="0.25">
+      <c r="D52" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="E52" s="10" t="s">
+        <v>443</v>
+      </c>
+      <c r="F52" s="10" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>37</v>
       </c>
@@ -53322,14 +53311,14 @@
       <c r="C53" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="D53" s="10" t="s">
-        <v>457</v>
+      <c r="D53" s="9" t="s">
+        <v>439</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>458</v>
+        <v>445</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>459</v>
+        <v>446</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: Forced topper avatar to use ranker logo, bypassing dirty localStorage state
</commit_message>
<xml_diff>
--- a/Update_App_Data/upsc_toppers_data.xlsx
+++ b/Update_App_Data/upsc_toppers_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\Storage  Driver\upsc-cse-master-hub\Update_App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3146911-EFC1-47FD-8AB4-F3ABA6D61DFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59B5FD0C-A5AF-4A43-9511-C79D9FEF0D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Strategy" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="459">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="461">
   <si>
     <t>id</t>
   </si>
@@ -119,22 +119,7 @@
     <t>category</t>
   </si>
   <si>
-    <t>candidate</t>
-  </si>
-  <si>
-    <t>board</t>
-  </si>
-  <si>
-    <t>score</t>
-  </si>
-  <si>
     <t>question</t>
-  </si>
-  <si>
-    <t>answer</t>
-  </si>
-  <si>
-    <t>topic</t>
   </si>
   <si>
     <t>interview-1</t>
@@ -1482,6 +1467,27 @@
   <si>
     <t>-</t>
   </si>
+  <si>
+    <t>Your rank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kya chaye to </t>
+  </si>
+  <si>
+    <t xml:space="preserve">advice </t>
+  </si>
+  <si>
+    <t>subject</t>
+  </si>
+  <si>
+    <t>Topper Name</t>
+  </si>
+  <si>
+    <t>Paper</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
 </sst>
 </file>
 
@@ -1968,117 +1974,117 @@
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="C1" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="D1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="Q1" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="R1" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="S1" s="5" t="s">
         <v>113</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="P1" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="R1" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="S1" s="5" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="H2" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="D2" s="5" t="s">
+      <c r="I2" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="J2" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="K2" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="L2" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="M2" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="N2" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="O2" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="P2" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="Q2" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="R2" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="S2" s="5" t="s">
         <v>113</v>
-      </c>
-      <c r="O2" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="P2" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="Q2" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="R2" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="S2" s="5" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
@@ -2086,58 +2092,58 @@
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="G3" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="H3" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="I3" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="J3" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="K3" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="L3" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="M3" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="N3" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="O3" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="P3" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="K3" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="L3" s="6" t="s">
+      <c r="Q3" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="M3" s="6" t="s">
+      <c r="R3" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="N3" s="6" t="s">
+      <c r="S3" s="6" t="s">
         <v>130</v>
-      </c>
-      <c r="O3" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="P3" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="Q3" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="R3" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="S3" s="6" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
@@ -2145,58 +2151,58 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="L4" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="E4" s="5" t="s">
+      <c r="M4" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="N4" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="O4" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="P4" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="Q4" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="R4" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="H4" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="L4" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="M4" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="N4" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="O4" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="P4" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="Q4" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="R4" s="5" t="s">
-        <v>142</v>
-      </c>
       <c r="S4" s="5" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" spans="1:19" ht="25.5" x14ac:dyDescent="0.25">
@@ -2204,58 +2210,58 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="I5" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="J5" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="L5" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="M5" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="E5" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="F5" s="6" t="s">
+      <c r="N5" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="O5" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="G5" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="H5" s="6" t="s">
+      <c r="P5" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q5" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="R5" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="J5" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="L5" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="M5" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="N5" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="O5" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="P5" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="Q5" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="R5" s="6" t="s">
-        <v>154</v>
-      </c>
       <c r="S5" s="6" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
@@ -2266,55 +2272,55 @@
         <v>5</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="D6" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="L6" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="M6" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="N6" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="L6" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="M6" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>160</v>
-      </c>
       <c r="O6" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="38.25" x14ac:dyDescent="0.25">
@@ -2322,58 +2328,58 @@
         <v>5</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="M7" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="N7" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="O7" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="P7" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="Q7" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="R7" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="K7" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="L7" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="M7" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="N7" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="O7" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="P7" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="Q7" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="R7" s="6" t="s">
-        <v>166</v>
-      </c>
       <c r="S7" s="6" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
@@ -2386,58 +2392,58 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="H9" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="I9" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="J9" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="K9" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="L9" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="M9" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="N9" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="O9" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="K9" s="5" t="s">
+      <c r="P9" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="L9" s="5" t="s">
+      <c r="Q9" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="M9" s="5" t="s">
+      <c r="R9" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="N9" s="5" t="s">
+      <c r="S9" s="5" t="s">
         <v>179</v>
-      </c>
-      <c r="O9" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="P9" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="Q9" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="R9" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="S9" s="5" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
@@ -2468,58 +2474,58 @@
         <v>9</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="G11" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="H11" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="I11" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="J11" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="K11" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="L11" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="M11" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="N11" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="J11" s="5" t="s">
+      <c r="O11" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="K11" s="5" t="s">
+      <c r="P11" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="L11" s="5" t="s">
+      <c r="Q11" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="M11" s="5" t="s">
+      <c r="R11" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="N11" s="5" t="s">
+      <c r="S11" s="5" t="s">
         <v>240</v>
-      </c>
-      <c r="O11" s="5" t="s">
-        <v>241</v>
-      </c>
-      <c r="P11" s="5" t="s">
-        <v>242</v>
-      </c>
-      <c r="Q11" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="R11" s="5" t="s">
-        <v>244</v>
-      </c>
-      <c r="S11" s="5" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="12" spans="1:19" ht="178.5" x14ac:dyDescent="0.25">
@@ -2527,58 +2533,58 @@
         <v>10</v>
       </c>
       <c r="B12" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="G12" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="H12" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="I12" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="J12" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="K12" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="L12" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="M12" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="I12" s="6" t="s">
+      <c r="N12" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="J12" s="6" t="s">
+      <c r="O12" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="K12" s="6" t="s">
+      <c r="P12" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="L12" s="6" t="s">
+      <c r="Q12" s="6" t="s">
         <v>256</v>
       </c>
-      <c r="M12" s="6" t="s">
+      <c r="R12" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="N12" s="6" t="s">
+      <c r="S12" s="6" t="s">
         <v>258</v>
-      </c>
-      <c r="O12" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="P12" s="6" t="s">
-        <v>260</v>
-      </c>
-      <c r="Q12" s="6" t="s">
-        <v>261</v>
-      </c>
-      <c r="R12" s="6" t="s">
-        <v>262</v>
-      </c>
-      <c r="S12" s="6" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="13" spans="1:19" ht="204" x14ac:dyDescent="0.25">
@@ -2586,58 +2592,58 @@
         <v>11</v>
       </c>
       <c r="B13" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="G13" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="H13" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="I13" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="J13" s="5" t="s">
         <v>267</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="K13" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="L13" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="M13" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="N13" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="J13" s="5" t="s">
+      <c r="O13" s="5" t="s">
         <v>272</v>
       </c>
-      <c r="K13" s="5" t="s">
+      <c r="P13" s="5" t="s">
         <v>273</v>
       </c>
-      <c r="L13" s="5" t="s">
+      <c r="Q13" s="5" t="s">
         <v>274</v>
       </c>
-      <c r="M13" s="5" t="s">
+      <c r="R13" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="N13" s="5" t="s">
+      <c r="S13" s="5" t="s">
         <v>276</v>
-      </c>
-      <c r="O13" s="5" t="s">
-        <v>277</v>
-      </c>
-      <c r="P13" s="5" t="s">
-        <v>278</v>
-      </c>
-      <c r="Q13" s="5" t="s">
-        <v>279</v>
-      </c>
-      <c r="R13" s="5" t="s">
-        <v>280</v>
-      </c>
-      <c r="S13" s="5" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="229.5" x14ac:dyDescent="0.25">
@@ -2645,58 +2651,58 @@
         <v>12</v>
       </c>
       <c r="B14" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="G14" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="H14" s="6" t="s">
         <v>283</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="I14" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="J14" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="K14" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L14" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="M14" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="H14" s="6" t="s">
+      <c r="N14" s="6" t="s">
         <v>288</v>
       </c>
-      <c r="I14" s="6" t="s">
+      <c r="O14" s="6" t="s">
         <v>289</v>
       </c>
-      <c r="J14" s="6" t="s">
+      <c r="P14" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="K14" s="6" t="s">
-        <v>289</v>
-      </c>
-      <c r="L14" s="6" t="s">
+      <c r="Q14" s="6" t="s">
         <v>291</v>
       </c>
-      <c r="M14" s="6" t="s">
+      <c r="R14" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="N14" s="6" t="s">
+      <c r="S14" s="6" t="s">
         <v>293</v>
-      </c>
-      <c r="O14" s="6" t="s">
-        <v>294</v>
-      </c>
-      <c r="P14" s="6" t="s">
-        <v>295</v>
-      </c>
-      <c r="Q14" s="6" t="s">
-        <v>296</v>
-      </c>
-      <c r="R14" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="S14" s="6" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="15" spans="1:19" ht="191.25" x14ac:dyDescent="0.25">
@@ -2704,58 +2710,58 @@
         <v>13</v>
       </c>
       <c r="B15" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="G15" s="5" t="s">
         <v>299</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="H15" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="I15" s="5" t="s">
         <v>301</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="J15" s="5" t="s">
         <v>302</v>
       </c>
-      <c r="F15" s="5" t="s">
+      <c r="K15" s="5" t="s">
         <v>303</v>
       </c>
-      <c r="G15" s="5" t="s">
+      <c r="L15" s="5" t="s">
         <v>304</v>
       </c>
-      <c r="H15" s="5" t="s">
+      <c r="M15" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="I15" s="5" t="s">
+      <c r="N15" s="5" t="s">
         <v>306</v>
       </c>
-      <c r="J15" s="5" t="s">
+      <c r="O15" s="5" t="s">
         <v>307</v>
       </c>
-      <c r="K15" s="5" t="s">
+      <c r="P15" s="5" t="s">
         <v>308</v>
       </c>
-      <c r="L15" s="5" t="s">
+      <c r="Q15" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="M15" s="5" t="s">
+      <c r="R15" s="5" t="s">
         <v>310</v>
       </c>
-      <c r="N15" s="5" t="s">
+      <c r="S15" s="5" t="s">
         <v>311</v>
-      </c>
-      <c r="O15" s="5" t="s">
-        <v>312</v>
-      </c>
-      <c r="P15" s="5" t="s">
-        <v>313</v>
-      </c>
-      <c r="Q15" s="5" t="s">
-        <v>314</v>
-      </c>
-      <c r="R15" s="5" t="s">
-        <v>315</v>
-      </c>
-      <c r="S15" s="5" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="16" spans="1:19" ht="229.5" x14ac:dyDescent="0.25">
@@ -2763,58 +2769,58 @@
         <v>14</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="G16" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="H16" s="6" t="s">
         <v>318</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="I16" s="6" t="s">
         <v>319</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="J16" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="L16" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="M16" s="6" t="s">
         <v>321</v>
       </c>
-      <c r="G16" s="6" t="s">
+      <c r="N16" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="O16" s="6" t="s">
         <v>322</v>
       </c>
-      <c r="H16" s="6" t="s">
+      <c r="P16" s="6" t="s">
         <v>323</v>
       </c>
-      <c r="I16" s="6" t="s">
+      <c r="Q16" s="6" t="s">
         <v>324</v>
       </c>
-      <c r="J16" s="6" t="s">
-        <v>324</v>
-      </c>
-      <c r="K16" s="6" t="s">
-        <v>324</v>
-      </c>
-      <c r="L16" s="6" t="s">
+      <c r="R16" s="6" t="s">
         <v>325</v>
       </c>
-      <c r="M16" s="6" t="s">
+      <c r="S16" s="6" t="s">
         <v>326</v>
-      </c>
-      <c r="N16" s="6" t="s">
-        <v>324</v>
-      </c>
-      <c r="O16" s="6" t="s">
-        <v>327</v>
-      </c>
-      <c r="P16" s="6" t="s">
-        <v>328</v>
-      </c>
-      <c r="Q16" s="6" t="s">
-        <v>329</v>
-      </c>
-      <c r="R16" s="6" t="s">
-        <v>330</v>
-      </c>
-      <c r="S16" s="6" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="17" spans="1:19" ht="165.75" x14ac:dyDescent="0.25">
@@ -2822,58 +2828,58 @@
         <v>15</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>327</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="G17" s="5" t="s">
         <v>332</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="H17" s="5" t="s">
         <v>333</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="I17" s="5" t="s">
         <v>334</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="J17" s="5" t="s">
         <v>335</v>
       </c>
-      <c r="F17" s="5" t="s">
+      <c r="K17" s="5" t="s">
         <v>336</v>
       </c>
-      <c r="G17" s="5" t="s">
+      <c r="L17" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="M17" s="5" t="s">
         <v>338</v>
       </c>
-      <c r="I17" s="5" t="s">
+      <c r="N17" s="5" t="s">
         <v>339</v>
       </c>
-      <c r="J17" s="5" t="s">
+      <c r="O17" s="5" t="s">
         <v>340</v>
       </c>
-      <c r="K17" s="5" t="s">
+      <c r="P17" s="5" t="s">
         <v>341</v>
       </c>
-      <c r="L17" s="5" t="s">
+      <c r="Q17" s="5" t="s">
         <v>342</v>
       </c>
-      <c r="M17" s="5" t="s">
+      <c r="R17" s="5" t="s">
         <v>343</v>
       </c>
-      <c r="N17" s="5" t="s">
+      <c r="S17" s="5" t="s">
         <v>344</v>
-      </c>
-      <c r="O17" s="5" t="s">
-        <v>345</v>
-      </c>
-      <c r="P17" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="Q17" s="5" t="s">
-        <v>347</v>
-      </c>
-      <c r="R17" s="5" t="s">
-        <v>348</v>
-      </c>
-      <c r="S17" s="5" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="127.5" x14ac:dyDescent="0.25">
@@ -2881,58 +2887,58 @@
         <v>16</v>
       </c>
       <c r="B18" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="J18" s="6" t="s">
         <v>350</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="K18" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="L18" s="6" t="s">
         <v>351</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="M18" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="N18" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="O18" s="6" t="s">
         <v>352</v>
       </c>
-      <c r="E18" s="6" t="s">
-        <v>352</v>
-      </c>
-      <c r="F18" s="6" t="s">
+      <c r="P18" s="6" t="s">
         <v>353</v>
       </c>
-      <c r="G18" s="6" t="s">
+      <c r="Q18" s="6" t="s">
         <v>354</v>
       </c>
-      <c r="H18" s="6" t="s">
-        <v>352</v>
-      </c>
-      <c r="I18" s="6" t="s">
-        <v>352</v>
-      </c>
-      <c r="J18" s="6" t="s">
+      <c r="R18" s="6" t="s">
         <v>355</v>
       </c>
-      <c r="K18" s="6" t="s">
-        <v>352</v>
-      </c>
-      <c r="L18" s="6" t="s">
+      <c r="S18" s="6" t="s">
         <v>356</v>
-      </c>
-      <c r="M18" s="6" t="s">
-        <v>352</v>
-      </c>
-      <c r="N18" s="6" t="s">
-        <v>352</v>
-      </c>
-      <c r="O18" s="6" t="s">
-        <v>357</v>
-      </c>
-      <c r="P18" s="6" t="s">
-        <v>358</v>
-      </c>
-      <c r="Q18" s="6" t="s">
-        <v>359</v>
-      </c>
-      <c r="R18" s="6" t="s">
-        <v>360</v>
-      </c>
-      <c r="S18" s="6" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
@@ -3058,122 +3064,122 @@
         <v>19</v>
       </c>
       <c r="B21" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="G21" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="H21" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="I21" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="J21" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="F21" s="5" t="s">
+      <c r="K21" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="G21" s="5" t="s">
+      <c r="L21" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="H21" s="5" t="s">
+      <c r="M21" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="I21" s="5" t="s">
+      <c r="N21" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="J21" s="5" t="s">
+      <c r="O21" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="K21" s="5" t="s">
+      <c r="P21" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="L21" s="5" t="s">
+      <c r="Q21" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="M21" s="5" t="s">
+      <c r="R21" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="N21" s="5" t="s">
+      <c r="S21" s="5" t="s">
         <v>197</v>
-      </c>
-      <c r="O21" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="P21" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="Q21" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="R21" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="S21" s="5" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="22" spans="1:19" ht="102" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B22" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="G22" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="H22" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="I22" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="J22" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="K22" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="G22" s="6" t="s">
+      <c r="L22" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="H22" s="6" t="s">
+      <c r="M22" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="I22" s="6" t="s">
+      <c r="N22" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="J22" s="6" t="s">
+      <c r="O22" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="K22" s="6" t="s">
+      <c r="P22" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="L22" s="6" t="s">
+      <c r="Q22" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="M22" s="6" t="s">
+      <c r="R22" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="N22" s="6" t="s">
+      <c r="S22" s="6" t="s">
         <v>215</v>
-      </c>
-      <c r="O22" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="P22" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="Q22" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="R22" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="S22" s="6" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="B23" s="2">
         <v>89</v>
@@ -3181,7 +3187,7 @@
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="B24" s="2">
         <v>65</v>
@@ -3189,7 +3195,7 @@
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="B25" s="2">
         <v>135</v>
@@ -3197,7 +3203,7 @@
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="B26" s="2">
         <v>110</v>
@@ -3205,7 +3211,7 @@
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="B27" s="2">
         <v>95</v>
@@ -3213,7 +3219,7 @@
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="B28" s="2">
         <v>128</v>
@@ -3221,7 +3227,7 @@
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="B29" s="2">
         <v>135</v>
@@ -52334,991 +52340,991 @@
     </row>
     <row r="2" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>90</v>
-      </c>
       <c r="F3" s="1" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>76</v>
-      </c>
       <c r="E8" s="1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>64</v>
-      </c>
       <c r="F11" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C16" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>49</v>
-      </c>
       <c r="E16" s="1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="B21" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="B22" t="s">
+        <v>370</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="E22" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="B22" t="s">
-        <v>375</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>380</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>381</v>
-      </c>
       <c r="F22" s="1" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="B23" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="B24" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="B25" t="s">
+        <v>379</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="B25" t="s">
-        <v>384</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>386</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>389</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>390</v>
-      </c>
       <c r="F25" s="1" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="B26" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="C26" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="E26" s="1" t="s">
         <v>386</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>448</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="B27" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="B28" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>450</v>
+        <v>445</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="B29" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>451</v>
+        <v>446</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>453</v>
+        <v>448</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>454</v>
+        <v>449</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>455</v>
+        <v>450</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>456</v>
+        <v>451</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>457</v>
+        <v>452</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="B37" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="63" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="B38" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="B39" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="D39" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="B40" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="D40" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="B41" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="D41" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B42" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="F42" s="10" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B43" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="F43" s="10" t="s">
-        <v>417</v>
+        <v>412</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B44" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="F44" s="10" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B45" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>421</v>
+        <v>416</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>422</v>
+        <v>417</v>
       </c>
       <c r="F45" s="10" t="s">
-        <v>423</v>
+        <v>418</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B46" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>425</v>
+        <v>420</v>
       </c>
       <c r="F46" s="10" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B47" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="F47" s="10" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B48" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>431</v>
+        <v>426</v>
       </c>
       <c r="F48" s="10" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B49" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="F49" s="10" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B50" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>436</v>
+        <v>431</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="F50" s="10" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B51" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>439</v>
+        <v>434</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="F51" s="10" t="s">
-        <v>441</v>
+        <v>436</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B52" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>442</v>
+        <v>437</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>443</v>
+        <v>438</v>
       </c>
       <c r="F52" s="10" t="s">
-        <v>444</v>
+        <v>439</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B53" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D53" s="9" t="s">
-        <v>439</v>
+        <v>434</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>445</v>
+        <v>440</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>446</v>
+        <v>441</v>
       </c>
     </row>
   </sheetData>
@@ -53346,46 +53352,46 @@
     <col min="2" max="2" width="14.875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.25" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="4.875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.5" style="1" customWidth="1"/>
     <col min="6" max="9" width="44.25" style="1" customWidth="1"/>
     <col min="10" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>460</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="G1" s="1" t="s">
-        <v>31</v>
+        <v>456</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>32</v>
+        <v>457</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="D2" s="1">
         <v>2023</v>
@@ -53394,24 +53400,24 @@
         <v>200</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="D3" s="1">
         <v>2025</v>
@@ -53420,24 +53426,24 @@
         <v>320</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="D4" s="1">
         <v>1546</v>
@@ -53446,19 +53452,19 @@
         <v>352</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:H1 A2:F2 H2" numberStoredAsText="1"/>
+    <ignoredError sqref="A2:F2 H2 F1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: persist adopted routine immediately and fallback to old localStorage keys to prevent data loss on updates
</commit_message>
<xml_diff>
--- a/Update_App_Data/upsc_toppers_data.xlsx
+++ b/Update_App_Data/upsc_toppers_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\Storage  Driver\upsc-cse-master-hub\Update_App_Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\New folder (3)\CSE PREP\Update_App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78255C39-90F8-4D3F-BCE1-AEA23B80D507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA3CB149-F915-49AD-83F4-F30BC79BAA6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Strategy" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="421">
   <si>
     <t>id</t>
   </si>
@@ -1250,191 +1250,6 @@
     <t>08:00 PM - 12:30 AM</t>
   </si>
   <si>
-    <t>अपना स्टडी पैटर्न</t>
-  </si>
-  <si>
-    <t>"हेलो एवरीवन।</t>
-  </si>
-  <si>
-    <t>आप हर रोज़ पढ़ाई करो और जो एवरेज है वो 7 टू 8 आवर्स रहे।</t>
-  </si>
-  <si>
-    <t>06:30 AM – 07:30 AM</t>
-  </si>
-  <si>
-    <t>मॉर्निंग रूटीन</t>
-  </si>
-  <si>
-    <t>फ्रेश होना, हल्का व्यायाम या ध्यान</t>
-  </si>
-  <si>
-    <t>07:30 AM – 09:30 AM</t>
-  </si>
-  <si>
-    <r>
-      <t>स्लॉट 1: करंट अफेयर्स</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (2 घंटे)</t>
-    </r>
-  </si>
-  <si>
-    <t>दैनिक समाचार पत्र (द हिंदू/इंडियन एक्सप्रेस) और समसामयिकी नोट्स</t>
-  </si>
-  <si>
-    <t>09:30 AM – 10:30 AM</t>
-  </si>
-  <si>
-    <t>ब्रेकफास्ट ब्रेक</t>
-  </si>
-  <si>
-    <t>नाश्ता और आराम</t>
-  </si>
-  <si>
-    <t>10:30 AM – 01:30 PM</t>
-  </si>
-  <si>
-    <r>
-      <t>स्लॉट 2: सामान्य अध्ययन (GS)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (3 घंटे)</t>
-    </r>
-  </si>
-  <si>
-    <t>कोर जीएस विषय (पॉलिटी, हिस्ट्री, इकॉनमी, या ज्योग्राफी)</t>
-  </si>
-  <si>
-    <t>01:30 PM – 03:00 PM</t>
-  </si>
-  <si>
-    <t>लंच &amp; पावर नैप</t>
-  </si>
-  <si>
-    <t>दोपहर का भोजन और विश्राम</t>
-  </si>
-  <si>
-    <t>03:00 PM – 06:00 PM</t>
-  </si>
-  <si>
-    <r>
-      <t>स्लॉट 3: ऑप्शनल सब्जेक्ट</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (3 घंटे)</t>
-    </r>
-  </si>
-  <si>
-    <t>वैकल्पिक विषय का गहन अध्ययन और नोट्स रिवीज़न</t>
-  </si>
-  <si>
-    <t>06:00 PM – 07:00 PM</t>
-  </si>
-  <si>
-    <t>इवनिंग ब्रेक</t>
-  </si>
-  <si>
-    <t>चाय, वॉक या हल्का समय</t>
-  </si>
-  <si>
-    <t>07:00 PM – 08:00 PM</t>
-  </si>
-  <si>
-    <t>जीएस / ऑप्शनल रिवीज़न (1 घंटा)</t>
-  </si>
-  <si>
-    <t>दिनभर पढ़े गए टॉपिक्स का क्विक रीकॉल</t>
-  </si>
-  <si>
-    <t>08:00 PM – 09:00 PM</t>
-  </si>
-  <si>
-    <t>डिनर ब्रेक</t>
-  </si>
-  <si>
-    <t>रात का खाना</t>
-  </si>
-  <si>
-    <t>09:00 PM – 11:00 PM</t>
-  </si>
-  <si>
-    <r>
-      <t>स्लॉट 4: टेस्ट प्रैक्टिस &amp; एक्टिव रीकॉल</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (2 घंटे)</t>
-    </r>
-  </si>
-  <si>
-    <t>10 CA MCQs, 25 स्टैटिक MCQs, 1-2 मेन्स प्रश्नों की ब्रेनस्टॉर्मिंग</t>
-  </si>
-  <si>
-    <t>11:00 PM – 06:30 AM</t>
-  </si>
-  <si>
-    <t>नींद</t>
-  </si>
-  <si>
-    <t>7.5 घंटे की पूरी नींद</t>
-  </si>
-  <si>
-    <r>
-      <t>एक्टिव रीकॉल पर ज़ोर:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> केवल किताबें खुली रखकर पढ़ने के बजाय पन्ने पलटकर आँखें बंद करके पॉइंट्स को खुद से दोहराएँ।</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>फ्लेक्सिबिलिटी:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> जिस विषय में स्कोर कम हो (जैसे ऑप्शनल), स्लॉट 2 और स्लॉट 3 के समय को अपनी आवश्यकतानुसार आपस में अदल-बदल सकते हैं।</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">3rd  </t>
-  </si>
-  <si>
     <t>01:30 PM - 03:00 PM</t>
   </si>
   <si>
@@ -1465,9 +1280,6 @@
     <t>08:00 AM - 09:0 AM</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>Your rank</t>
   </si>
   <si>
@@ -1493,7 +1305,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1512,19 +1324,6 @@
     <font>
       <sz val="10"/>
       <color rgb="FF1C2833"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -1549,7 +1348,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1572,26 +1371,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFC4C7C5"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFC4C7C5"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFC4C7C5"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFC4C7C5"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1615,12 +1399,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -52307,7 +52085,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.625" style="1" bestFit="1" customWidth="1"/>
@@ -52826,7 +52604,7 @@
         <v>381</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>443</v>
+        <v>404</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>386</v>
@@ -52843,7 +52621,7 @@
         <v>381</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>444</v>
+        <v>405</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>388</v>
@@ -52860,7 +52638,7 @@
         <v>381</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>445</v>
+        <v>406</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>387</v>
@@ -52877,7 +52655,7 @@
         <v>381</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>446</v>
+        <v>407</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>389</v>
@@ -52894,7 +52672,7 @@
         <v>381</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>447</v>
+        <v>408</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>391</v>
@@ -52911,7 +52689,7 @@
         <v>381</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>448</v>
+        <v>409</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>392</v>
@@ -52928,13 +52706,13 @@
         <v>381</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>449</v>
+        <v>410</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>390</v>
       </c>
@@ -52945,13 +52723,13 @@
         <v>381</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>450</v>
+        <v>411</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
         <v>395</v>
       </c>
@@ -52962,13 +52740,13 @@
         <v>381</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>451</v>
+        <v>412</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
         <v>395</v>
       </c>
@@ -52985,7 +52763,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
         <v>395</v>
       </c>
@@ -52996,13 +52774,13 @@
         <v>381</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>452</v>
+        <v>413</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>400</v>
       </c>
@@ -53019,7 +52797,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="63" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" ht="63" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>400</v>
       </c>
@@ -53034,297 +52812,6 @@
       </c>
       <c r="E38" s="1" t="s">
         <v>402</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>405</v>
-      </c>
-      <c r="B39" t="s">
-        <v>404</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="D39" t="s">
-        <v>453</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>405</v>
-      </c>
-      <c r="B40" t="s">
-        <v>404</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="D40" t="s">
-        <v>453</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>405</v>
-      </c>
-      <c r="B41" t="s">
-        <v>404</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="D41" t="s">
-        <v>453</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B42" t="s">
-        <v>97</v>
-      </c>
-      <c r="C42" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="D42" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="E42" s="10" t="s">
-        <v>408</v>
-      </c>
-      <c r="F42" s="10" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B43" t="s">
-        <v>97</v>
-      </c>
-      <c r="C43" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="D43" s="9" t="s">
-        <v>410</v>
-      </c>
-      <c r="E43" s="9" t="s">
-        <v>411</v>
-      </c>
-      <c r="F43" s="10" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B44" t="s">
-        <v>97</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="D44" s="9" t="s">
-        <v>413</v>
-      </c>
-      <c r="E44" s="10" t="s">
-        <v>414</v>
-      </c>
-      <c r="F44" s="10" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B45" t="s">
-        <v>97</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="D45" s="9" t="s">
-        <v>416</v>
-      </c>
-      <c r="E45" s="9" t="s">
-        <v>417</v>
-      </c>
-      <c r="F45" s="10" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B46" t="s">
-        <v>97</v>
-      </c>
-      <c r="C46" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="D46" s="9" t="s">
-        <v>419</v>
-      </c>
-      <c r="E46" s="10" t="s">
-        <v>420</v>
-      </c>
-      <c r="F46" s="10" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B47" t="s">
-        <v>97</v>
-      </c>
-      <c r="C47" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="D47" s="9" t="s">
-        <v>422</v>
-      </c>
-      <c r="E47" s="9" t="s">
-        <v>423</v>
-      </c>
-      <c r="F47" s="10" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B48" t="s">
-        <v>97</v>
-      </c>
-      <c r="C48" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="D48" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="E48" s="10" t="s">
-        <v>426</v>
-      </c>
-      <c r="F48" s="10" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B49" t="s">
-        <v>97</v>
-      </c>
-      <c r="C49" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="D49" s="9" t="s">
-        <v>428</v>
-      </c>
-      <c r="E49" s="10" t="s">
-        <v>429</v>
-      </c>
-      <c r="F49" s="10" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B50" t="s">
-        <v>97</v>
-      </c>
-      <c r="C50" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="D50" s="9" t="s">
-        <v>431</v>
-      </c>
-      <c r="E50" s="10" t="s">
-        <v>432</v>
-      </c>
-      <c r="F50" s="10" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B51" t="s">
-        <v>97</v>
-      </c>
-      <c r="C51" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="D51" s="9" t="s">
-        <v>434</v>
-      </c>
-      <c r="E51" s="9" t="s">
-        <v>435</v>
-      </c>
-      <c r="F51" s="10" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B52" t="s">
-        <v>97</v>
-      </c>
-      <c r="C52" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="D52" s="9" t="s">
-        <v>437</v>
-      </c>
-      <c r="E52" s="10" t="s">
-        <v>438</v>
-      </c>
-      <c r="F52" s="10" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B53" t="s">
-        <v>97</v>
-      </c>
-      <c r="C53" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="D53" s="9" t="s">
-        <v>434</v>
-      </c>
-      <c r="E53" s="4" t="s">
-        <v>440</v>
-      </c>
-      <c r="F53" s="4" t="s">
-        <v>441</v>
       </c>
     </row>
   </sheetData>
@@ -53359,28 +52846,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>460</v>
+        <v>420</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>458</v>
+        <v>418</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>459</v>
+        <v>419</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>454</v>
+        <v>414</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>455</v>
+        <v>415</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>456</v>
+        <v>416</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>457</v>
+        <v>417</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">

</xml_diff>